<commit_message>
Actualizar Data-ETFPESOV.xlsx (15/10/2026 00:39)
</commit_message>
<xml_diff>
--- a/ETFPESOV/General/Data-ETFPESOV.xlsx
+++ b/ETFPESOV/General/Data-ETFPESOV.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eldorado275.sharepoint.com/sites/Compartidos/Documentos compartidos/INVERSIONES/Claude - Fernando/Dashboards ETFs/Dashboards/ETFPESOV/General/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="13_ncr:1_{92F23378-0498-4D77-8B70-1F22B2DCC606}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BE39A42B-A1C0-4488-9EA7-05A8A58D69F3}"/>
+  <xr:revisionPtr revIDLastSave="7" documentId="13_ncr:1_{92F23378-0498-4D77-8B70-1F22B2DCC606}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A7C32A59-1137-4938-AC21-925F17D9BB51}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{F6F75CCC-009E-413C-B55D-A670828334F1}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="36">
   <si>
     <t>Fecha</t>
   </si>
@@ -530,7 +530,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E89EACC1-FF2B-4ECD-9B28-49A6BC374F12}">
-  <dimension ref="A1:AI381"/>
+  <dimension ref="A1:AI382"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="27" max="31" width="11.5546875" style="3"/>
@@ -33818,21 +33818,119 @@
         <v>10166.85</v>
       </c>
     </row>
+    <row r="382" spans="1:35" x14ac:dyDescent="0.3">
+      <c r="A382" s="1">
+        <v>46309</v>
+      </c>
+      <c r="B382">
+        <v>110.93324331103148</v>
+      </c>
+      <c r="C382">
+        <v>149482545.36161491</v>
+      </c>
+      <c r="D382" t="s">
+        <v>23</v>
+      </c>
+      <c r="E382">
+        <v>7081</v>
+      </c>
+      <c r="F382">
+        <v>3</v>
+      </c>
+      <c r="G382">
+        <v>6.288239921945328</v>
+      </c>
+      <c r="H382">
+        <v>6.0903486862256191</v>
+      </c>
+      <c r="I382">
+        <v>182.35</v>
+      </c>
+      <c r="J382">
+        <v>6.37</v>
+      </c>
+      <c r="K382">
+        <v>6.1400000000000006</v>
+      </c>
+      <c r="L382">
+        <v>10.933243311031472</v>
+      </c>
+      <c r="M382">
+        <v>11.46428840218241</v>
+      </c>
+      <c r="N382">
+        <v>6.5801933195998439</v>
+      </c>
+      <c r="O382">
+        <v>6.59</v>
+      </c>
+      <c r="P382">
+        <v>4.5363769667598388E-3</v>
+      </c>
+      <c r="Q382">
+        <v>4.3801355153983736E-3</v>
+      </c>
+      <c r="R382">
+        <v>0.10887413000386073</v>
+      </c>
+      <c r="S382">
+        <v>0.16180189630928665</v>
+      </c>
+      <c r="T382">
+        <v>6.9598406231108356E-2</v>
+      </c>
+      <c r="U382">
+        <v>0.10206207688402413</v>
+      </c>
+      <c r="V382">
+        <v>0.27708819090093151</v>
+      </c>
+      <c r="W382">
+        <v>0.80353982728544882</v>
+      </c>
+      <c r="X382">
+        <v>110.64</v>
+      </c>
+      <c r="Y382">
+        <v>-2.2065340798904209</v>
+      </c>
+      <c r="Z382">
+        <v>-3.9109511967821864</v>
+      </c>
+      <c r="AA382" s="3">
+        <v>2.6434214152496471E-3</v>
+      </c>
+      <c r="AB382" s="3">
+        <v>6.1196594259988503E-3</v>
+      </c>
+      <c r="AC382" s="3">
+        <v>5.0996755716583072E-3</v>
+      </c>
+      <c r="AD382" s="3">
+        <v>4.4939128242007E-3</v>
+      </c>
+      <c r="AE382" s="3">
+        <v>5.0225149276161727E-3</v>
+      </c>
+      <c r="AF382">
+        <v>8012.5249999999996</v>
+      </c>
+      <c r="AG382">
+        <v>9703.1049999999996</v>
+      </c>
+      <c r="AH382">
+        <v>11769.724999999999</v>
+      </c>
+      <c r="AI382">
+        <v>10133.625</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101006CC87EF38A8DD0408B89B7B34D0336DC" ma:contentTypeVersion="20" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="a30c2ca5bc864785a186dec6b0346788">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="0902cc7b-e4ce-48dd-a92e-a98e18ec7ffe" xmlns:ns3="dd854d95-092e-48c7-992a-80d5cc5badc3" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2932ec1554b414302dd4a6579c5666bc" ns2:_="" ns3:_="">
     <xsd:import namespace="0902cc7b-e4ce-48dd-a92e-a98e18ec7ffe"/>
@@ -34087,6 +34185,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -34099,14 +34206,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3FDE56E9-7C64-4C15-9C33-5B738E73FACD}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BABE8802-F313-4DEC-9147-95F411D9A097}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -34125,6 +34224,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3FDE56E9-7C64-4C15-9C33-5B738E73FACD}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9C21325A-2FA6-4D29-AED0-CA44A2859AE9}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Actualizar Data-ETFPESOV.xlsx (16/10/2026 00:54)
</commit_message>
<xml_diff>
--- a/ETFPESOV/General/Data-ETFPESOV.xlsx
+++ b/ETFPESOV/General/Data-ETFPESOV.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eldorado275.sharepoint.com/sites/Compartidos/Documentos compartidos/INVERSIONES/Claude - Fernando/Dashboards ETFs/Dashboards/ETFPESOV/General/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="7" documentId="13_ncr:1_{92F23378-0498-4D77-8B70-1F22B2DCC606}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A7C32A59-1137-4938-AC21-925F17D9BB51}"/>
+  <xr:revisionPtr revIDLastSave="10" documentId="13_ncr:1_{92F23378-0498-4D77-8B70-1F22B2DCC606}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{46E1BE6E-3CD5-4B25-B6B5-847DBB7D6BCD}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{F6F75CCC-009E-413C-B55D-A670828334F1}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="36">
   <si>
     <t>Fecha</t>
   </si>
@@ -530,7 +530,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E89EACC1-FF2B-4ECD-9B28-49A6BC374F12}">
-  <dimension ref="A1:AI382"/>
+  <dimension ref="A1:AI383"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="27" max="31" width="11.5546875" style="3"/>
@@ -33925,12 +33925,130 @@
         <v>10133.625</v>
       </c>
     </row>
+    <row r="383" spans="1:35" x14ac:dyDescent="0.3">
+      <c r="A383" s="1">
+        <v>46310</v>
+      </c>
+      <c r="B383">
+        <v>111.00291718372182</v>
+      </c>
+      <c r="C383">
+        <v>149576430.90506515</v>
+      </c>
+      <c r="D383" t="s">
+        <v>23</v>
+      </c>
+      <c r="E383">
+        <v>5626</v>
+      </c>
+      <c r="F383">
+        <v>0</v>
+      </c>
+      <c r="G383">
+        <v>6.2844734273861818</v>
+      </c>
+      <c r="H383">
+        <v>6.0775785996445233</v>
+      </c>
+      <c r="I383">
+        <v>182.46</v>
+      </c>
+      <c r="J383">
+        <v>6.37</v>
+      </c>
+      <c r="K383">
+        <v>6.13</v>
+      </c>
+      <c r="L383">
+        <v>11.002917183721816</v>
+      </c>
+      <c r="M383">
+        <v>11.531527621947912</v>
+      </c>
+      <c r="N383">
+        <v>6.5802389363795344</v>
+      </c>
+      <c r="O383">
+        <v>6.59</v>
+      </c>
+      <c r="P383">
+        <v>3.7651254182885976E-3</v>
+      </c>
+      <c r="Q383">
+        <v>4.4009893427019746E-3</v>
+      </c>
+      <c r="R383">
+        <v>0.10887456566897875</v>
+      </c>
+      <c r="S383">
+        <v>0.16176920419437477</v>
+      </c>
+      <c r="T383">
+        <v>6.6216530631635351E-2</v>
+      </c>
+      <c r="U383">
+        <v>9.6219291162780163E-2</v>
+      </c>
+      <c r="V383">
+        <v>0.2686153053359952</v>
+      </c>
+      <c r="W383">
+        <v>0.73013291473398301</v>
+      </c>
+      <c r="X383">
+        <v>110.31</v>
+      </c>
+      <c r="Y383">
+        <v>-2.1451129108062239</v>
+      </c>
+      <c r="Z383">
+        <v>-3.9109511967821864</v>
+      </c>
+      <c r="AA383" s="3">
+        <v>6.2423330963001789E-3</v>
+      </c>
+      <c r="AB383" s="3">
+        <v>6.2623817475528252E-3</v>
+      </c>
+      <c r="AC383" s="3">
+        <v>5.1958176410386121E-3</v>
+      </c>
+      <c r="AD383" s="3">
+        <v>4.5274259400711796E-3</v>
+      </c>
+      <c r="AE383" s="3">
+        <v>5.0356170096278923E-3</v>
+      </c>
+      <c r="AF383">
+        <v>8012.5249999999996</v>
+      </c>
+      <c r="AG383">
+        <v>9411.880000000001</v>
+      </c>
+      <c r="AH383">
+        <v>11551.599999999999</v>
+      </c>
+      <c r="AI383">
+        <v>10133.625</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="dd854d95-092e-48c7-992a-80d5cc5badc3" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="0902cc7b-e4ce-48dd-a92e-a98e18ec7ffe">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101006CC87EF38A8DD0408B89B7B34D0336DC" ma:contentTypeVersion="20" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="a30c2ca5bc864785a186dec6b0346788">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="0902cc7b-e4ce-48dd-a92e-a98e18ec7ffe" xmlns:ns3="dd854d95-092e-48c7-992a-80d5cc5badc3" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2932ec1554b414302dd4a6579c5666bc" ns2:_="" ns3:_="">
     <xsd:import namespace="0902cc7b-e4ce-48dd-a92e-a98e18ec7ffe"/>
@@ -34185,7 +34303,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -34194,18 +34312,18 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="dd854d95-092e-48c7-992a-80d5cc5badc3" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="0902cc7b-e4ce-48dd-a92e-a98e18ec7ffe">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9C21325A-2FA6-4D29-AED0-CA44A2859AE9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="dd854d95-092e-48c7-992a-80d5cc5badc3"/>
+    <ds:schemaRef ds:uri="0902cc7b-e4ce-48dd-a92e-a98e18ec7ffe"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BABE8802-F313-4DEC-9147-95F411D9A097}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -34224,21 +34342,10 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3FDE56E9-7C64-4C15-9C33-5B738E73FACD}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9C21325A-2FA6-4D29-AED0-CA44A2859AE9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="dd854d95-092e-48c7-992a-80d5cc5badc3"/>
-    <ds:schemaRef ds:uri="0902cc7b-e4ce-48dd-a92e-a98e18ec7ffe"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Actualizar Data-ETFPESOV.xlsx (16/10/2026 00:57)
</commit_message>
<xml_diff>
--- a/ETFPESOV/General/Data-ETFPESOV.xlsx
+++ b/ETFPESOV/General/Data-ETFPESOV.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eldorado275.sharepoint.com/sites/Compartidos/Documentos compartidos/INVERSIONES/Claude - Fernando/Dashboards ETFs/Dashboards/ETFPESOV/General/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10" documentId="13_ncr:1_{92F23378-0498-4D77-8B70-1F22B2DCC606}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{46E1BE6E-3CD5-4B25-B6B5-847DBB7D6BCD}"/>
+  <xr:revisionPtr revIDLastSave="13" documentId="13_ncr:1_{92F23378-0498-4D77-8B70-1F22B2DCC606}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2551843B-4ABC-48D4-A6AB-35263E529AF9}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{F6F75CCC-009E-413C-B55D-A670828334F1}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
   <si>
     <t>Fecha</t>
   </si>
@@ -33721,8 +33721,8 @@
       <c r="C381">
         <v>149522405.18141958</v>
       </c>
-      <c r="D381" t="s">
-        <v>23</v>
+      <c r="D381">
+        <v>547</v>
       </c>
       <c r="E381">
         <v>6330</v>
@@ -33828,8 +33828,8 @@
       <c r="C382">
         <v>149482545.36161491</v>
       </c>
-      <c r="D382" t="s">
-        <v>23</v>
+      <c r="D382">
+        <v>547</v>
       </c>
       <c r="E382">
         <v>7081</v>
@@ -34038,17 +34038,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="dd854d95-092e-48c7-992a-80d5cc5badc3" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="0902cc7b-e4ce-48dd-a92e-a98e18ec7ffe">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101006CC87EF38A8DD0408B89B7B34D0336DC" ma:contentTypeVersion="20" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="a30c2ca5bc864785a186dec6b0346788">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="0902cc7b-e4ce-48dd-a92e-a98e18ec7ffe" xmlns:ns3="dd854d95-092e-48c7-992a-80d5cc5badc3" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2932ec1554b414302dd4a6579c5666bc" ns2:_="" ns3:_="">
     <xsd:import namespace="0902cc7b-e4ce-48dd-a92e-a98e18ec7ffe"/>
@@ -34303,6 +34292,17 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="dd854d95-092e-48c7-992a-80d5cc5badc3" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="0902cc7b-e4ce-48dd-a92e-a98e18ec7ffe">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -34313,17 +34313,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9C21325A-2FA6-4D29-AED0-CA44A2859AE9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="dd854d95-092e-48c7-992a-80d5cc5badc3"/>
-    <ds:schemaRef ds:uri="0902cc7b-e4ce-48dd-a92e-a98e18ec7ffe"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BABE8802-F313-4DEC-9147-95F411D9A097}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -34342,6 +34331,17 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9C21325A-2FA6-4D29-AED0-CA44A2859AE9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="dd854d95-092e-48c7-992a-80d5cc5badc3"/>
+    <ds:schemaRef ds:uri="0902cc7b-e4ce-48dd-a92e-a98e18ec7ffe"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3FDE56E9-7C64-4C15-9C33-5B738E73FACD}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Actualizar Data-ETFPESOV.xlsx (18/10/2026 13:47)
</commit_message>
<xml_diff>
--- a/ETFPESOV/General/Data-ETFPESOV.xlsx
+++ b/ETFPESOV/General/Data-ETFPESOV.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eldorado275.sharepoint.com/sites/Compartidos/Documentos compartidos/INVERSIONES/Claude - Fernando/Dashboards ETFs/Dashboards/ETFPESOV/General/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="13" documentId="13_ncr:1_{92F23378-0498-4D77-8B70-1F22B2DCC606}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2551843B-4ABC-48D4-A6AB-35263E529AF9}"/>
+  <xr:revisionPtr revIDLastSave="15" documentId="13_ncr:1_{92F23378-0498-4D77-8B70-1F22B2DCC606}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4FD8F9CE-4411-4A5E-B27C-F1276393B866}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{F6F75CCC-009E-413C-B55D-A670828334F1}"/>
   </bookViews>
@@ -530,7 +530,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E89EACC1-FF2B-4ECD-9B28-49A6BC374F12}">
-  <dimension ref="A1:AI383"/>
+  <dimension ref="A1:AI384"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="27" max="31" width="11.5546875" style="3"/>
@@ -33935,8 +33935,8 @@
       <c r="C383">
         <v>149576430.90506515</v>
       </c>
-      <c r="D383" t="s">
-        <v>23</v>
+      <c r="D383">
+        <v>547</v>
       </c>
       <c r="E383">
         <v>5626</v>
@@ -34029,6 +34029,113 @@
         <v>11551.599999999999</v>
       </c>
       <c r="AI383">
+        <v>10133.625</v>
+      </c>
+    </row>
+    <row r="384" spans="1:35" x14ac:dyDescent="0.3">
+      <c r="A384" s="1">
+        <v>46311</v>
+      </c>
+      <c r="B384">
+        <v>110.97623471985419</v>
+      </c>
+      <c r="C384">
+        <v>149540476.28500351</v>
+      </c>
+      <c r="D384" t="s">
+        <v>23</v>
+      </c>
+      <c r="E384">
+        <v>3640</v>
+      </c>
+      <c r="F384">
+        <v>4</v>
+      </c>
+      <c r="G384">
+        <v>6.2805929937581944</v>
+      </c>
+      <c r="H384">
+        <v>6.0816649836833481</v>
+      </c>
+      <c r="I384">
+        <v>182.41</v>
+      </c>
+      <c r="J384">
+        <v>6.36</v>
+      </c>
+      <c r="K384">
+        <v>6.1400000000000006</v>
+      </c>
+      <c r="L384">
+        <v>10.976234719854183</v>
+      </c>
+      <c r="M384">
+        <v>11.500964340236308</v>
+      </c>
+      <c r="N384">
+        <v>6.5804516284538277</v>
+      </c>
+      <c r="O384">
+        <v>6.59</v>
+      </c>
+      <c r="P384">
+        <v>3.850815397768304E-3</v>
+      </c>
+      <c r="Q384">
+        <v>4.4417928758354033E-3</v>
+      </c>
+      <c r="R384">
+        <v>0.10887471534382859</v>
+      </c>
+      <c r="S384">
+        <v>0.16164506699333742</v>
+      </c>
+      <c r="T384">
+        <v>6.3394660549775939E-2</v>
+      </c>
+      <c r="U384">
+        <v>9.4837944022285736E-2</v>
+      </c>
+      <c r="V384">
+        <v>0.26352267466290824</v>
+      </c>
+      <c r="W384">
+        <v>0.85319385399147407</v>
+      </c>
+      <c r="X384">
+        <v>110.3</v>
+      </c>
+      <c r="Y384">
+        <v>-2.1686349006356131</v>
+      </c>
+      <c r="Z384">
+        <v>-3.9109511967821864</v>
+      </c>
+      <c r="AA384" s="3">
+        <v>6.0935093136045282E-3</v>
+      </c>
+      <c r="AB384" s="3">
+        <v>6.4334827566881504E-3</v>
+      </c>
+      <c r="AC384" s="3">
+        <v>5.2157077984132921E-3</v>
+      </c>
+      <c r="AD384" s="3">
+        <v>4.556874568558713E-3</v>
+      </c>
+      <c r="AE384" s="3">
+        <v>5.0504394127232934E-3</v>
+      </c>
+      <c r="AF384">
+        <v>7699.6</v>
+      </c>
+      <c r="AG384">
+        <v>9313.7799999999988</v>
+      </c>
+      <c r="AH384">
+        <v>11262.025</v>
+      </c>
+      <c r="AI384">
         <v>10133.625</v>
       </c>
     </row>
@@ -34293,6 +34400,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="dd854d95-092e-48c7-992a-80d5cc5badc3" xsi:nil="true"/>
@@ -34301,15 +34417,6 @@
     </lcf76f155ced4ddcb4097134ff3c332f>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -34332,6 +34439,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3FDE56E9-7C64-4C15-9C33-5B738E73FACD}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9C21325A-2FA6-4D29-AED0-CA44A2859AE9}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -34340,12 +34455,4 @@
     <ds:schemaRef ds:uri="0902cc7b-e4ce-48dd-a92e-a98e18ec7ffe"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3FDE56E9-7C64-4C15-9C33-5B738E73FACD}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Actualizar Data-ETFPESOV.xlsx (20/10/2026 00:30)
</commit_message>
<xml_diff>
--- a/ETFPESOV/General/Data-ETFPESOV.xlsx
+++ b/ETFPESOV/General/Data-ETFPESOV.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eldorado275.sharepoint.com/sites/Compartidos/Documentos compartidos/INVERSIONES/Claude - Fernando/Dashboards ETFs/Dashboards/ETFPESOV/General/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="15" documentId="13_ncr:1_{92F23378-0498-4D77-8B70-1F22B2DCC606}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4FD8F9CE-4411-4A5E-B27C-F1276393B866}"/>
+  <xr:revisionPtr revIDLastSave="17" documentId="13_ncr:1_{92F23378-0498-4D77-8B70-1F22B2DCC606}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F7374E15-A041-4DBF-BB08-8F4F00249DD6}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{F6F75CCC-009E-413C-B55D-A670828334F1}"/>
   </bookViews>
@@ -530,7 +530,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E89EACC1-FF2B-4ECD-9B28-49A6BC374F12}">
-  <dimension ref="A1:AI384"/>
+  <dimension ref="A1:AI385"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="27" max="31" width="11.5546875" style="3"/>
@@ -34042,8 +34042,8 @@
       <c r="C384">
         <v>149540476.28500351</v>
       </c>
-      <c r="D384" t="s">
-        <v>23</v>
+      <c r="D384">
+        <v>547</v>
       </c>
       <c r="E384">
         <v>3640</v>
@@ -34137,6 +34137,113 @@
       </c>
       <c r="AI384">
         <v>10133.625</v>
+      </c>
+    </row>
+    <row r="385" spans="1:35" x14ac:dyDescent="0.3">
+      <c r="A385" s="1">
+        <v>46314</v>
+      </c>
+      <c r="B385">
+        <v>110.66204782017122</v>
+      </c>
+      <c r="C385">
+        <v>149117109.43768072</v>
+      </c>
+      <c r="D385" t="s">
+        <v>23</v>
+      </c>
+      <c r="E385">
+        <v>3875</v>
+      </c>
+      <c r="F385">
+        <v>1</v>
+      </c>
+      <c r="G385">
+        <v>6.257994912695966</v>
+      </c>
+      <c r="H385">
+        <v>6.1178635602105329</v>
+      </c>
+      <c r="I385">
+        <v>181.86</v>
+      </c>
+      <c r="J385">
+        <v>6.34</v>
+      </c>
+      <c r="K385">
+        <v>6.18</v>
+      </c>
+      <c r="L385">
+        <v>10.662047820171217</v>
+      </c>
+      <c r="M385">
+        <v>11.164768241408796</v>
+      </c>
+      <c r="N385">
+        <v>6.5802089420869345</v>
+      </c>
+      <c r="O385">
+        <v>6.59</v>
+      </c>
+      <c r="P385">
+        <v>5.3274140873484253E-3</v>
+      </c>
+      <c r="Q385">
+        <v>5.1201673453697997E-3</v>
+      </c>
+      <c r="R385">
+        <v>0.10888490052658138</v>
+      </c>
+      <c r="S385">
+        <v>0.16162454220478117</v>
+      </c>
+      <c r="T385">
+        <v>3.97819975342939E-2</v>
+      </c>
+      <c r="U385">
+        <v>7.7602417112676569E-2</v>
+      </c>
+      <c r="V385">
+        <v>0.24290535903727095</v>
+      </c>
+      <c r="W385">
+        <v>0.88550105268481172</v>
+      </c>
+      <c r="X385">
+        <v>110.71</v>
+      </c>
+      <c r="Y385">
+        <v>-2.4456071133793111</v>
+      </c>
+      <c r="Z385">
+        <v>-3.9109511967821864</v>
+      </c>
+      <c r="AA385" s="3">
+        <v>4.3332091510439597E-4</v>
+      </c>
+      <c r="AB385" s="3">
+        <v>6.3636340066774546E-3</v>
+      </c>
+      <c r="AC385" s="3">
+        <v>5.2063039663814703E-3</v>
+      </c>
+      <c r="AD385" s="3">
+        <v>4.5295848565040956E-3</v>
+      </c>
+      <c r="AE385" s="3">
+        <v>5.0422406809099854E-3</v>
+      </c>
+      <c r="AF385">
+        <v>7699.6</v>
+      </c>
+      <c r="AG385">
+        <v>9185.5600000000013</v>
+      </c>
+      <c r="AH385">
+        <v>11262.025</v>
+      </c>
+      <c r="AI385">
+        <v>10047.755000000001</v>
       </c>
     </row>
   </sheetData>
@@ -34145,6 +34252,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101006CC87EF38A8DD0408B89B7B34D0336DC" ma:contentTypeVersion="20" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="a30c2ca5bc864785a186dec6b0346788">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="0902cc7b-e4ce-48dd-a92e-a98e18ec7ffe" xmlns:ns3="dd854d95-092e-48c7-992a-80d5cc5badc3" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2932ec1554b414302dd4a6579c5666bc" ns2:_="" ns3:_="">
     <xsd:import namespace="0902cc7b-e4ce-48dd-a92e-a98e18ec7ffe"/>
@@ -34399,15 +34515,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -34420,6 +34527,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3FDE56E9-7C64-4C15-9C33-5B738E73FACD}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BABE8802-F313-4DEC-9147-95F411D9A097}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -34438,14 +34553,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3FDE56E9-7C64-4C15-9C33-5B738E73FACD}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9C21325A-2FA6-4D29-AED0-CA44A2859AE9}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Actualizar Data-ETFPESOV.xlsx (21/10/2026 01:21)
</commit_message>
<xml_diff>
--- a/ETFPESOV/General/Data-ETFPESOV.xlsx
+++ b/ETFPESOV/General/Data-ETFPESOV.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eldorado275.sharepoint.com/sites/Compartidos/Documentos compartidos/INVERSIONES/Claude - Fernando/Dashboards ETFs/Dashboards/ETFPESOV/General/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="17" documentId="13_ncr:1_{92F23378-0498-4D77-8B70-1F22B2DCC606}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F7374E15-A041-4DBF-BB08-8F4F00249DD6}"/>
+  <xr:revisionPtr revIDLastSave="19" documentId="13_ncr:1_{92F23378-0498-4D77-8B70-1F22B2DCC606}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4DFE71AC-73D6-4C04-B582-D4C61979B77F}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{F6F75CCC-009E-413C-B55D-A670828334F1}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="36">
   <si>
     <t>Fecha</t>
   </si>
@@ -530,7 +530,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E89EACC1-FF2B-4ECD-9B28-49A6BC374F12}">
-  <dimension ref="A1:AI385"/>
+  <dimension ref="A1:AI386"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="27" max="31" width="11.5546875" style="3"/>
@@ -34246,21 +34246,119 @@
         <v>10047.755000000001</v>
       </c>
     </row>
+    <row r="386" spans="1:35" x14ac:dyDescent="0.3">
+      <c r="A386" s="1">
+        <v>46315</v>
+      </c>
+      <c r="B386">
+        <v>110.70075809273899</v>
+      </c>
+      <c r="C386">
+        <v>149169271.52996579</v>
+      </c>
+      <c r="D386" t="s">
+        <v>23</v>
+      </c>
+      <c r="E386">
+        <v>4207</v>
+      </c>
+      <c r="F386">
+        <v>1</v>
+      </c>
+      <c r="G386">
+        <v>6.2535662709234412</v>
+      </c>
+      <c r="H386">
+        <v>6.1074799672460438</v>
+      </c>
+      <c r="I386">
+        <v>181.91</v>
+      </c>
+      <c r="J386">
+        <v>6.33</v>
+      </c>
+      <c r="K386">
+        <v>6.17</v>
+      </c>
+      <c r="L386">
+        <v>10.700758092739004</v>
+      </c>
+      <c r="M386">
+        <v>11.195331523120377</v>
+      </c>
+      <c r="N386">
+        <v>6.5801247994769483</v>
+      </c>
+      <c r="O386">
+        <v>6.59</v>
+      </c>
+      <c r="P386">
+        <v>5.5558377229501833E-3</v>
+      </c>
+      <c r="Q386">
+        <v>5.2370325567100019E-3</v>
+      </c>
+      <c r="R386">
+        <v>0.10888694254458398</v>
+      </c>
+      <c r="S386">
+        <v>0.16020987650211513</v>
+      </c>
+      <c r="T386">
+        <v>3.3845142585198218E-2</v>
+      </c>
+      <c r="U386">
+        <v>6.7183424765249189E-2</v>
+      </c>
+      <c r="V386">
+        <v>0.23164322254511927</v>
+      </c>
+      <c r="W386">
+        <v>1.3062801901675192</v>
+      </c>
+      <c r="X386">
+        <v>110.71</v>
+      </c>
+      <c r="Y386">
+        <v>-2.4114819800277076</v>
+      </c>
+      <c r="Z386">
+        <v>-3.9109511967821864</v>
+      </c>
+      <c r="AA386" s="3">
+        <v>8.3485492061941002E-5</v>
+      </c>
+      <c r="AB386" s="3">
+        <v>6.3608324852667984E-3</v>
+      </c>
+      <c r="AC386" s="3">
+        <v>5.1734594067870858E-3</v>
+      </c>
+      <c r="AD386" s="3">
+        <v>4.489232869199597E-3</v>
+      </c>
+      <c r="AE386" s="3">
+        <v>5.0351787096865469E-3</v>
+      </c>
+      <c r="AF386">
+        <v>7309.25</v>
+      </c>
+      <c r="AG386">
+        <v>9185.5600000000013</v>
+      </c>
+      <c r="AH386">
+        <v>11097.075000000001</v>
+      </c>
+      <c r="AI386">
+        <v>10047.755000000001</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101006CC87EF38A8DD0408B89B7B34D0336DC" ma:contentTypeVersion="20" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="a30c2ca5bc864785a186dec6b0346788">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="0902cc7b-e4ce-48dd-a92e-a98e18ec7ffe" xmlns:ns3="dd854d95-092e-48c7-992a-80d5cc5badc3" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2932ec1554b414302dd4a6579c5666bc" ns2:_="" ns3:_="">
     <xsd:import namespace="0902cc7b-e4ce-48dd-a92e-a98e18ec7ffe"/>
@@ -34515,6 +34613,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -34527,14 +34634,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3FDE56E9-7C64-4C15-9C33-5B738E73FACD}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BABE8802-F313-4DEC-9147-95F411D9A097}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -34553,6 +34652,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3FDE56E9-7C64-4C15-9C33-5B738E73FACD}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9C21325A-2FA6-4D29-AED0-CA44A2859AE9}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Actualizar Data-ETFPESOV.xlsx (21/10/2026 21:36)
</commit_message>
<xml_diff>
--- a/ETFPESOV/General/Data-ETFPESOV.xlsx
+++ b/ETFPESOV/General/Data-ETFPESOV.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eldorado275.sharepoint.com/sites/Compartidos/Documentos compartidos/INVERSIONES/Claude - Fernando/Dashboards ETFs/Dashboards/ETFPESOV/General/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="19" documentId="13_ncr:1_{92F23378-0498-4D77-8B70-1F22B2DCC606}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4DFE71AC-73D6-4C04-B582-D4C61979B77F}"/>
+  <xr:revisionPtr revIDLastSave="22" documentId="13_ncr:1_{92F23378-0498-4D77-8B70-1F22B2DCC606}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A6BA0012-12F2-4CBA-A0AF-4BBA180F91D9}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{F6F75CCC-009E-413C-B55D-A670828334F1}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
   <si>
     <t>Fecha</t>
   </si>
@@ -530,7 +530,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E89EACC1-FF2B-4ECD-9B28-49A6BC374F12}">
-  <dimension ref="A1:AI386"/>
+  <dimension ref="A1:AI387"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="27" max="31" width="11.5546875" style="3"/>
@@ -34149,8 +34149,8 @@
       <c r="C385">
         <v>149117109.43768072</v>
       </c>
-      <c r="D385" t="s">
-        <v>23</v>
+      <c r="D385">
+        <v>547</v>
       </c>
       <c r="E385">
         <v>3875</v>
@@ -34256,8 +34256,8 @@
       <c r="C386">
         <v>149169271.52996579</v>
       </c>
-      <c r="D386" t="s">
-        <v>23</v>
+      <c r="D386">
+        <v>547</v>
       </c>
       <c r="E386">
         <v>4207</v>
@@ -34350,6 +34350,113 @@
         <v>11097.075000000001</v>
       </c>
       <c r="AI386">
+        <v>10047.755000000001</v>
+      </c>
+    </row>
+    <row r="387" spans="1:35" x14ac:dyDescent="0.3">
+      <c r="A387" s="1">
+        <v>46316</v>
+      </c>
+      <c r="B387">
+        <v>110.56514855473955</v>
+      </c>
+      <c r="C387">
+        <v>148986537.67751154</v>
+      </c>
+      <c r="D387" t="s">
+        <v>23</v>
+      </c>
+      <c r="E387">
+        <v>1661</v>
+      </c>
+      <c r="F387">
+        <v>0</v>
+      </c>
+      <c r="G387">
+        <v>6.2447554962820693</v>
+      </c>
+      <c r="H387">
+        <v>6.1236818868259881</v>
+      </c>
+      <c r="I387">
+        <v>181.69</v>
+      </c>
+      <c r="J387">
+        <v>6.33</v>
+      </c>
+      <c r="K387">
+        <v>6.18</v>
+      </c>
+      <c r="L387">
+        <v>10.565148554739556</v>
+      </c>
+      <c r="M387">
+        <v>11.060853083589372</v>
+      </c>
+      <c r="N387">
+        <v>6.5801848419009143</v>
+      </c>
+      <c r="O387">
+        <v>6.59</v>
+      </c>
+      <c r="P387">
+        <v>5.5056735938059089E-3</v>
+      </c>
+      <c r="Q387">
+        <v>5.2308816689338811E-3</v>
+      </c>
+      <c r="R387">
+        <v>0.10888683573370395</v>
+      </c>
+      <c r="S387">
+        <v>0.15742296462881389</v>
+      </c>
+      <c r="T387">
+        <v>3.5802485459057731E-2</v>
+      </c>
+      <c r="U387">
+        <v>7.0734026280738771E-2</v>
+      </c>
+      <c r="V387">
+        <v>0.23536755742641358</v>
+      </c>
+      <c r="W387">
+        <v>0.69268353362095247</v>
+      </c>
+      <c r="X387">
+        <v>110.73</v>
+      </c>
+      <c r="Y387">
+        <v>-2.5310288925398328</v>
+      </c>
+      <c r="Z387">
+        <v>-3.9109511967821864</v>
+      </c>
+      <c r="AA387" s="3">
+        <v>1.4909892259480362E-3</v>
+      </c>
+      <c r="AB387" s="3">
+        <v>6.326647911982097E-3</v>
+      </c>
+      <c r="AC387" s="3">
+        <v>5.1695087203325555E-3</v>
+      </c>
+      <c r="AD387" s="3">
+        <v>4.4552992191686947E-3</v>
+      </c>
+      <c r="AE387" s="3">
+        <v>5.0246184530679588E-3</v>
+      </c>
+      <c r="AF387">
+        <v>7309.25</v>
+      </c>
+      <c r="AG387">
+        <v>9107.5250000000015</v>
+      </c>
+      <c r="AH387">
+        <v>11002.15</v>
+      </c>
+      <c r="AI387">
         <v>10047.755000000001</v>
       </c>
     </row>
@@ -34359,6 +34466,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="dd854d95-092e-48c7-992a-80d5cc5badc3" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="0902cc7b-e4ce-48dd-a92e-a98e18ec7ffe">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101006CC87EF38A8DD0408B89B7B34D0336DC" ma:contentTypeVersion="20" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="a30c2ca5bc864785a186dec6b0346788">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="0902cc7b-e4ce-48dd-a92e-a98e18ec7ffe" xmlns:ns3="dd854d95-092e-48c7-992a-80d5cc5badc3" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2932ec1554b414302dd4a6579c5666bc" ns2:_="" ns3:_="">
     <xsd:import namespace="0902cc7b-e4ce-48dd-a92e-a98e18ec7ffe"/>
@@ -34613,27 +34740,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9C21325A-2FA6-4D29-AED0-CA44A2859AE9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="dd854d95-092e-48c7-992a-80d5cc5badc3"/>
+    <ds:schemaRef ds:uri="0902cc7b-e4ce-48dd-a92e-a98e18ec7ffe"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="dd854d95-092e-48c7-992a-80d5cc5badc3" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="0902cc7b-e4ce-48dd-a92e-a98e18ec7ffe">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3FDE56E9-7C64-4C15-9C33-5B738E73FACD}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BABE8802-F313-4DEC-9147-95F411D9A097}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -34650,23 +34776,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3FDE56E9-7C64-4C15-9C33-5B738E73FACD}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9C21325A-2FA6-4D29-AED0-CA44A2859AE9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="dd854d95-092e-48c7-992a-80d5cc5badc3"/>
-    <ds:schemaRef ds:uri="0902cc7b-e4ce-48dd-a92e-a98e18ec7ffe"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Actualizar Data-ETFPESOV.xlsx (23/10/2026 01:02)
</commit_message>
<xml_diff>
--- a/ETFPESOV/General/Data-ETFPESOV.xlsx
+++ b/ETFPESOV/General/Data-ETFPESOV.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eldorado275.sharepoint.com/sites/Compartidos/Documentos compartidos/INVERSIONES/Claude - Fernando/Dashboards ETFs/Dashboards/ETFPESOV/General/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="22" documentId="13_ncr:1_{92F23378-0498-4D77-8B70-1F22B2DCC606}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A6BA0012-12F2-4CBA-A0AF-4BBA180F91D9}"/>
+  <xr:revisionPtr revIDLastSave="24" documentId="13_ncr:1_{92F23378-0498-4D77-8B70-1F22B2DCC606}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EAADA12D-C4D9-4D5B-92A4-5C09ADB4CEF1}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{F6F75CCC-009E-413C-B55D-A670828334F1}"/>
   </bookViews>
@@ -530,7 +530,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E89EACC1-FF2B-4ECD-9B28-49A6BC374F12}">
-  <dimension ref="A1:AI387"/>
+  <dimension ref="A1:AI388"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="27" max="31" width="11.5546875" style="3"/>
@@ -34363,8 +34363,8 @@
       <c r="C387">
         <v>148986537.67751154</v>
       </c>
-      <c r="D387" t="s">
-        <v>23</v>
+      <c r="D387">
+        <v>547</v>
       </c>
       <c r="E387">
         <v>1661</v>
@@ -34457,6 +34457,113 @@
         <v>11002.15</v>
       </c>
       <c r="AI387">
+        <v>10047.755000000001</v>
+      </c>
+    </row>
+    <row r="388" spans="1:35" x14ac:dyDescent="0.3">
+      <c r="A388" s="1">
+        <v>46317</v>
+      </c>
+      <c r="B388">
+        <v>110.58423558292399</v>
+      </c>
+      <c r="C388">
+        <v>149012257.44799009</v>
+      </c>
+      <c r="D388" t="s">
+        <v>23</v>
+      </c>
+      <c r="E388">
+        <v>4901</v>
+      </c>
+      <c r="F388">
+        <v>0</v>
+      </c>
+      <c r="G388">
+        <v>6.2429520537401331</v>
+      </c>
+      <c r="H388">
+        <v>6.122656671910419</v>
+      </c>
+      <c r="I388">
+        <v>181.72</v>
+      </c>
+      <c r="J388">
+        <v>6.32</v>
+      </c>
+      <c r="K388">
+        <v>6.18</v>
+      </c>
+      <c r="L388">
+        <v>10.584235582923984</v>
+      </c>
+      <c r="M388">
+        <v>11.079191052616322</v>
+      </c>
+      <c r="N388">
+        <v>6.5802634505977471</v>
+      </c>
+      <c r="O388">
+        <v>6.59</v>
+      </c>
+      <c r="P388">
+        <v>5.4971790400755944E-3</v>
+      </c>
+      <c r="Q388">
+        <v>5.2190993416640907E-3</v>
+      </c>
+      <c r="R388">
+        <v>0.10888648013886966</v>
+      </c>
+      <c r="S388">
+        <v>0.15742295613487764</v>
+      </c>
+      <c r="T388">
+        <v>3.7165276177741902E-2</v>
+      </c>
+      <c r="U388">
+        <v>6.7268705945622287E-2</v>
+      </c>
+      <c r="V388">
+        <v>0.38391924093205132</v>
+      </c>
+      <c r="W388">
+        <v>0.69240833664638846</v>
+      </c>
+      <c r="X388">
+        <v>111.39</v>
+      </c>
+      <c r="Y388">
+        <v>-2.514202677200239</v>
+      </c>
+      <c r="Z388">
+        <v>-3.9109511967821864</v>
+      </c>
+      <c r="AA388" s="3">
+        <v>7.2864311339546628E-3</v>
+      </c>
+      <c r="AB388" s="3">
+        <v>6.5077773272583569E-3</v>
+      </c>
+      <c r="AC388" s="3">
+        <v>5.2311016256708903E-3</v>
+      </c>
+      <c r="AD388" s="3">
+        <v>4.4636686001837244E-3</v>
+      </c>
+      <c r="AE388" s="3">
+        <v>5.0362676944243302E-3</v>
+      </c>
+      <c r="AF388">
+        <v>7309.25</v>
+      </c>
+      <c r="AG388">
+        <v>9107.5250000000015</v>
+      </c>
+      <c r="AH388">
+        <v>11002.15</v>
+      </c>
+      <c r="AI388">
         <v>10047.755000000001</v>
       </c>
     </row>
@@ -34466,26 +34573,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="dd854d95-092e-48c7-992a-80d5cc5badc3" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="0902cc7b-e4ce-48dd-a92e-a98e18ec7ffe">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101006CC87EF38A8DD0408B89B7B34D0336DC" ma:contentTypeVersion="20" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="a30c2ca5bc864785a186dec6b0346788">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="0902cc7b-e4ce-48dd-a92e-a98e18ec7ffe" xmlns:ns3="dd854d95-092e-48c7-992a-80d5cc5badc3" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2932ec1554b414302dd4a6579c5666bc" ns2:_="" ns3:_="">
     <xsd:import namespace="0902cc7b-e4ce-48dd-a92e-a98e18ec7ffe"/>
@@ -34740,26 +34827,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9C21325A-2FA6-4D29-AED0-CA44A2859AE9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="dd854d95-092e-48c7-992a-80d5cc5badc3"/>
-    <ds:schemaRef ds:uri="0902cc7b-e4ce-48dd-a92e-a98e18ec7ffe"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3FDE56E9-7C64-4C15-9C33-5B738E73FACD}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="dd854d95-092e-48c7-992a-80d5cc5badc3" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="0902cc7b-e4ce-48dd-a92e-a98e18ec7ffe">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BABE8802-F313-4DEC-9147-95F411D9A097}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -34776,4 +34864,23 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3FDE56E9-7C64-4C15-9C33-5B738E73FACD}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9C21325A-2FA6-4D29-AED0-CA44A2859AE9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="dd854d95-092e-48c7-992a-80d5cc5badc3"/>
+    <ds:schemaRef ds:uri="0902cc7b-e4ce-48dd-a92e-a98e18ec7ffe"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Actualizar Data-ETFPESOV.xlsx (26/10/2026 10:46)
</commit_message>
<xml_diff>
--- a/ETFPESOV/General/Data-ETFPESOV.xlsx
+++ b/ETFPESOV/General/Data-ETFPESOV.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eldorado275.sharepoint.com/sites/Compartidos/Documentos compartidos/INVERSIONES/Claude - Fernando/Dashboards ETFs/Dashboards/ETFPESOV/General/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="24" documentId="13_ncr:1_{92F23378-0498-4D77-8B70-1F22B2DCC606}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EAADA12D-C4D9-4D5B-92A4-5C09ADB4CEF1}"/>
+  <xr:revisionPtr revIDLastSave="26" documentId="13_ncr:1_{92F23378-0498-4D77-8B70-1F22B2DCC606}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{04F98192-866C-41F4-83E7-79F6E06BA807}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{F6F75CCC-009E-413C-B55D-A670828334F1}"/>
   </bookViews>
@@ -530,7 +530,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E89EACC1-FF2B-4ECD-9B28-49A6BC374F12}">
-  <dimension ref="A1:AI388"/>
+  <dimension ref="A1:AI389"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="27" max="31" width="11.5546875" style="3"/>
@@ -34470,8 +34470,8 @@
       <c r="C388">
         <v>149012257.44799009</v>
       </c>
-      <c r="D388" t="s">
-        <v>23</v>
+      <c r="D388">
+        <v>547</v>
       </c>
       <c r="E388">
         <v>4901</v>
@@ -34564,6 +34564,113 @@
         <v>11002.15</v>
       </c>
       <c r="AI388">
+        <v>10047.755000000001</v>
+      </c>
+    </row>
+    <row r="389" spans="1:35" x14ac:dyDescent="0.3">
+      <c r="A389" s="1">
+        <v>46318</v>
+      </c>
+      <c r="B389">
+        <v>110.63281666031268</v>
+      </c>
+      <c r="C389">
+        <v>149077720.44977134</v>
+      </c>
+      <c r="D389" t="s">
+        <v>23</v>
+      </c>
+      <c r="E389">
+        <v>5982.21</v>
+      </c>
+      <c r="F389">
+        <v>1</v>
+      </c>
+      <c r="G389">
+        <v>6.2415686970464197</v>
+      </c>
+      <c r="H389">
+        <v>6.1189093714566933</v>
+      </c>
+      <c r="I389">
+        <v>181.8</v>
+      </c>
+      <c r="J389">
+        <v>6.32</v>
+      </c>
+      <c r="K389">
+        <v>6.18</v>
+      </c>
+      <c r="L389">
+        <v>10.632816660312683</v>
+      </c>
+      <c r="M389">
+        <v>11.128092303354876</v>
+      </c>
+      <c r="N389">
+        <v>6.5804636810530992</v>
+      </c>
+      <c r="O389">
+        <v>6.59</v>
+      </c>
+      <c r="P389">
+        <v>5.492734709737223E-3</v>
+      </c>
+      <c r="Q389">
+        <v>5.2167169673811376E-3</v>
+      </c>
+      <c r="R389">
+        <v>0.10828629997367131</v>
+      </c>
+      <c r="S389">
+        <v>0.15703411239196041</v>
+      </c>
+      <c r="T389">
+        <v>3.4154539787378813E-2</v>
+      </c>
+      <c r="U389">
+        <v>6.3370987070965334E-2</v>
+      </c>
+      <c r="V389">
+        <v>0.25273781275788609</v>
+      </c>
+      <c r="W389">
+        <v>0.46557458543317054</v>
+      </c>
+      <c r="X389">
+        <v>110.78</v>
+      </c>
+      <c r="Y389">
+        <v>-2.4713759122542922</v>
+      </c>
+      <c r="Z389">
+        <v>-3.9109511967821864</v>
+      </c>
+      <c r="AA389" s="3">
+        <v>1.3303768640295921E-3</v>
+      </c>
+      <c r="AB389" s="3">
+        <v>6.2342213568824445E-3</v>
+      </c>
+      <c r="AC389" s="3">
+        <v>5.2280246597041944E-3</v>
+      </c>
+      <c r="AD389" s="3">
+        <v>4.459940166150804E-3</v>
+      </c>
+      <c r="AE389" s="3">
+        <v>5.0227889299083008E-3</v>
+      </c>
+      <c r="AF389">
+        <v>7309.25</v>
+      </c>
+      <c r="AG389">
+        <v>8662.9650000000001</v>
+      </c>
+      <c r="AH389">
+        <v>10857.38</v>
+      </c>
+      <c r="AI389">
         <v>10047.755000000001</v>
       </c>
     </row>
@@ -34573,6 +34680,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="dd854d95-092e-48c7-992a-80d5cc5badc3" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="0902cc7b-e4ce-48dd-a92e-a98e18ec7ffe">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101006CC87EF38A8DD0408B89B7B34D0336DC" ma:contentTypeVersion="20" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="a30c2ca5bc864785a186dec6b0346788">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="0902cc7b-e4ce-48dd-a92e-a98e18ec7ffe" xmlns:ns3="dd854d95-092e-48c7-992a-80d5cc5badc3" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2932ec1554b414302dd4a6579c5666bc" ns2:_="" ns3:_="">
     <xsd:import namespace="0902cc7b-e4ce-48dd-a92e-a98e18ec7ffe"/>
@@ -34827,27 +34954,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9C21325A-2FA6-4D29-AED0-CA44A2859AE9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="dd854d95-092e-48c7-992a-80d5cc5badc3"/>
+    <ds:schemaRef ds:uri="0902cc7b-e4ce-48dd-a92e-a98e18ec7ffe"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="dd854d95-092e-48c7-992a-80d5cc5badc3" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="0902cc7b-e4ce-48dd-a92e-a98e18ec7ffe">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3FDE56E9-7C64-4C15-9C33-5B738E73FACD}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BABE8802-F313-4DEC-9147-95F411D9A097}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -34864,23 +34990,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3FDE56E9-7C64-4C15-9C33-5B738E73FACD}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9C21325A-2FA6-4D29-AED0-CA44A2859AE9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="dd854d95-092e-48c7-992a-80d5cc5badc3"/>
-    <ds:schemaRef ds:uri="0902cc7b-e4ce-48dd-a92e-a98e18ec7ffe"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Actualizar Data-ETFPESOV.xlsx (26/10/2026 15:59)
</commit_message>
<xml_diff>
--- a/ETFPESOV/General/Data-ETFPESOV.xlsx
+++ b/ETFPESOV/General/Data-ETFPESOV.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eldorado275.sharepoint.com/sites/Compartidos/Documentos compartidos/INVERSIONES/Claude - Fernando/Dashboards ETFs/Dashboards/ETFPESOV/General/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="29" documentId="13_ncr:1_{92F23378-0498-4D77-8B70-1F22B2DCC606}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A8BF8D58-7A32-47FC-AE16-FBBAC81ABD6C}"/>
+  <xr:revisionPtr revIDLastSave="32" documentId="13_ncr:1_{92F23378-0498-4D77-8B70-1F22B2DCC606}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{832548A3-27EB-4C0C-AC3C-4D25B168E83D}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{F6F75CCC-009E-413C-B55D-A670828334F1}"/>
   </bookViews>
@@ -2407,7 +2407,7 @@
         <v>0.30294945219025993</v>
       </c>
       <c r="T31">
-        <v>-0.16586847056285769</v>
+        <v>0.16586847056285769</v>
       </c>
       <c r="X31">
         <v>102.5</v>
@@ -2478,7 +2478,7 @@
         <v>0.30431344337139582</v>
       </c>
       <c r="T32">
-        <v>0.13277207632080845</v>
+        <v>-0.13277207632080845</v>
       </c>
       <c r="X32">
         <v>101.94</v>
@@ -2549,7 +2549,7 @@
         <v>0.305100491964586</v>
       </c>
       <c r="T33">
-        <v>0.23717380542305211</v>
+        <v>-0.23717380542305211</v>
       </c>
       <c r="X33">
         <v>102.51</v>
@@ -2620,7 +2620,7 @@
         <v>0.2961945061194588</v>
       </c>
       <c r="T34">
-        <v>0.4771538732093461</v>
+        <v>-0.4771538732093461</v>
       </c>
       <c r="X34">
         <v>102.5</v>
@@ -2691,7 +2691,7 @@
         <v>0.28824596820532106</v>
       </c>
       <c r="T35">
-        <v>0.23823230697217479</v>
+        <v>-0.23823230697217479</v>
       </c>
       <c r="X35">
         <v>101.56</v>
@@ -2762,7 +2762,7 @@
         <v>0.2894240740853784</v>
       </c>
       <c r="T36">
-        <v>-0.1525297900064837</v>
+        <v>0.1525297900064837</v>
       </c>
       <c r="X36">
         <v>102.5</v>
@@ -2833,7 +2833,7 @@
         <v>0.28869207388967699</v>
       </c>
       <c r="T37">
-        <v>0.25504715969324465</v>
+        <v>-0.25504715969324465</v>
       </c>
       <c r="X37">
         <v>101.18</v>
@@ -2904,7 +2904,7 @@
         <v>0.28636629100858579</v>
       </c>
       <c r="T38">
-        <v>0.32584039102421247</v>
+        <v>-0.32584039102421247</v>
       </c>
       <c r="X38">
         <v>101.6</v>
@@ -2975,7 +2975,7 @@
         <v>0.26476418610496177</v>
       </c>
       <c r="T39">
-        <v>-0.55458279029683144</v>
+        <v>0.55458279029683144</v>
       </c>
       <c r="X39">
         <v>101.53</v>
@@ -3046,7 +3046,7 @@
         <v>0.25189060153654891</v>
       </c>
       <c r="T40">
-        <v>-0.11427332877713692</v>
+        <v>0.11427332877713692</v>
       </c>
       <c r="X40">
         <v>102.12</v>
@@ -3117,7 +3117,7 @@
         <v>0.25050790859340955</v>
       </c>
       <c r="T41">
-        <v>-0.4109019663137925</v>
+        <v>0.4109019663137925</v>
       </c>
       <c r="X41">
         <v>101</v>
@@ -3188,7 +3188,7 @@
         <v>0.28713443969229363</v>
       </c>
       <c r="T42">
-        <v>0.26476650728568529</v>
+        <v>-0.26476650728568529</v>
       </c>
       <c r="X42">
         <v>102.5</v>
@@ -3259,7 +3259,7 @@
         <v>0.2864162976244643</v>
       </c>
       <c r="T43">
-        <v>0.35668669435469091</v>
+        <v>-0.35668669435469091</v>
       </c>
       <c r="X43">
         <v>102.5</v>
@@ -3330,7 +3330,7 @@
         <v>0.28311279057165339</v>
       </c>
       <c r="T44">
-        <v>-6.1872812771901486E-2</v>
+        <v>6.1872812771901486E-2</v>
       </c>
       <c r="X44">
         <v>101.82</v>
@@ -3401,7 +3401,7 @@
         <v>0.28960896676111031</v>
       </c>
       <c r="T45">
-        <v>-0.4915256361817999</v>
+        <v>0.4915256361817999</v>
       </c>
       <c r="X45">
         <v>101.01</v>
@@ -3472,7 +3472,7 @@
         <v>0.30363810212026271</v>
       </c>
       <c r="T46">
-        <v>0.40367253175106477</v>
+        <v>-0.40367253175106477</v>
       </c>
       <c r="X46">
         <v>100.79</v>
@@ -3543,7 +3543,7 @@
         <v>0.30273888424643219</v>
       </c>
       <c r="T47">
-        <v>1.9013064346040665E-2</v>
+        <v>-1.9013064346040665E-2</v>
       </c>
       <c r="X47">
         <v>102</v>
@@ -3614,7 +3614,7 @@
         <v>0.29834924169731902</v>
       </c>
       <c r="T48">
-        <v>0.17240067653474522</v>
+        <v>-0.17240067653474522</v>
       </c>
       <c r="X48">
         <v>100.45</v>
@@ -3685,7 +3685,7 @@
         <v>0.29650548129182319</v>
       </c>
       <c r="T49">
-        <v>0.56405159102548286</v>
+        <v>-0.56405159102548286</v>
       </c>
       <c r="X49">
         <v>101.57</v>
@@ -3756,7 +3756,7 @@
         <v>0.28110282218802563</v>
       </c>
       <c r="T50">
-        <v>0.90496544303184656</v>
+        <v>-0.90496544303184656</v>
       </c>
       <c r="X50">
         <v>102.2</v>
@@ -3827,7 +3827,7 @@
         <v>0.3048210151140594</v>
       </c>
       <c r="T51">
-        <v>-1.0538747993882325E-2</v>
+        <v>1.0538747993882325E-2</v>
       </c>
       <c r="X51">
         <v>101.01</v>
@@ -3898,7 +3898,7 @@
         <v>0.33600856497188569</v>
       </c>
       <c r="T52">
-        <v>0.44572035979875135</v>
+        <v>-0.44572035979875135</v>
       </c>
       <c r="X52">
         <v>102.2</v>
@@ -3969,7 +3969,7 @@
         <v>0.33601684622617856</v>
       </c>
       <c r="T53">
-        <v>0.4405180546191767</v>
+        <v>-0.4405180546191767</v>
       </c>
       <c r="X53">
         <v>102.54</v>
@@ -4040,7 +4040,7 @@
         <v>0.33656083566355521</v>
       </c>
       <c r="T54">
-        <v>0.26937410533030004</v>
+        <v>-0.26937410533030004</v>
       </c>
       <c r="X54">
         <v>101.3</v>
@@ -4111,7 +4111,7 @@
         <v>0.33644475684751057</v>
       </c>
       <c r="T55">
-        <v>0.5250273739976663</v>
+        <v>-0.5250273739976663</v>
       </c>
       <c r="X55">
         <v>103.45</v>
@@ -4182,7 +4182,7 @@
         <v>0.33699756791654228</v>
       </c>
       <c r="T56">
-        <v>0.46724512128679674</v>
+        <v>-0.46724512128679674</v>
       </c>
       <c r="X56">
         <v>101.32</v>
@@ -4253,7 +4253,7 @@
         <v>0.32792654243765784</v>
       </c>
       <c r="T57">
-        <v>0.82931903581133781</v>
+        <v>-0.82931903581133781</v>
       </c>
       <c r="X57">
         <v>103.25</v>
@@ -4324,7 +4324,7 @@
         <v>0.31178800395628492</v>
       </c>
       <c r="T58">
-        <v>0.25641910996507811</v>
+        <v>-0.25641910996507811</v>
       </c>
       <c r="X58">
         <v>101.52</v>
@@ -4395,7 +4395,7 @@
         <v>0.31239213488297052</v>
       </c>
       <c r="T59">
-        <v>0.15879269596359435</v>
+        <v>-0.15879269596359435</v>
       </c>
       <c r="X59">
         <v>103.25</v>
@@ -4466,7 +4466,7 @@
         <v>0.31136397195063997</v>
       </c>
       <c r="T60">
-        <v>-0.2191773322663737</v>
+        <v>0.2191773322663737</v>
       </c>
       <c r="X60">
         <v>101.5</v>
@@ -4543,10 +4543,10 @@
         <v>0.30434202531812099</v>
       </c>
       <c r="T61">
-        <v>0.11130541826362972</v>
+        <v>-0.11130541826362972</v>
       </c>
       <c r="U61">
-        <v>-5.4242095293743908E-2</v>
+        <v>5.4242095293743908E-2</v>
       </c>
       <c r="X61">
         <v>103</v>
@@ -4626,10 +4626,10 @@
         <v>0.3048710315682831</v>
       </c>
       <c r="T62">
-        <v>0.100360578944092</v>
+        <v>-0.100360578944092</v>
       </c>
       <c r="U62">
-        <v>0.23744651087276303</v>
+        <v>-0.23744651087276303</v>
       </c>
       <c r="X62">
         <v>104</v>
@@ -4709,10 +4709,10 @@
         <v>0.3055912478610609</v>
       </c>
       <c r="T63">
-        <v>-0.18937741376567896</v>
+        <v>0.18937741376567896</v>
       </c>
       <c r="U63">
-        <v>4.8263845890250678E-2</v>
+        <v>-4.8263845890250678E-2</v>
       </c>
       <c r="X63">
         <v>104</v>
@@ -4792,10 +4792,10 @@
         <v>0.30044276710532941</v>
       </c>
       <c r="T64">
-        <v>-5.0600309464465809E-2</v>
+        <v>5.0600309464465809E-2</v>
       </c>
       <c r="U64">
-        <v>0.43652774262814553</v>
+        <v>-0.43652774262814553</v>
       </c>
       <c r="X64">
         <v>104.25</v>
@@ -4875,10 +4875,10 @@
         <v>0.29566615100092081</v>
       </c>
       <c r="T65">
-        <v>-0.20749215875262017</v>
+        <v>0.20749215875262017</v>
       </c>
       <c r="U65">
-        <v>3.6366438592705386E-2</v>
+        <v>-3.6366438592705386E-2</v>
       </c>
       <c r="X65">
         <v>104.25</v>
@@ -4958,10 +4958,10 @@
         <v>0.29549329311978223</v>
       </c>
       <c r="T66">
-        <v>0.17216062618543582</v>
+        <v>-0.17216062618543582</v>
       </c>
       <c r="U66">
-        <v>1.633400259504203E-2</v>
+        <v>-1.633400259504203E-2</v>
       </c>
       <c r="X66">
         <v>103.16</v>
@@ -5041,10 +5041,10 @@
         <v>0.29428971285306094</v>
       </c>
       <c r="T67">
-        <v>-9.371941386722149E-2</v>
+        <v>9.371941386722149E-2</v>
       </c>
       <c r="U67">
-        <v>0.1678107990768174</v>
+        <v>-0.1678107990768174</v>
       </c>
       <c r="X67">
         <v>104.5</v>
@@ -5124,10 +5124,10 @@
         <v>0.2923119128282623</v>
       </c>
       <c r="T68">
-        <v>0.34921060349255573</v>
+        <v>-0.34921060349255573</v>
       </c>
       <c r="U68">
-        <v>0.68812067061949644</v>
+        <v>-0.68812067061949644</v>
       </c>
       <c r="X68">
         <v>102.75</v>
@@ -5207,10 +5207,10 @@
         <v>0.28077074598859109</v>
       </c>
       <c r="T69">
-        <v>0.57608831852047349</v>
+        <v>-0.57608831852047349</v>
       </c>
       <c r="U69">
-        <v>1.2462117354195001E-2</v>
+        <v>-1.2462117354195001E-2</v>
       </c>
       <c r="X69">
         <v>104.5</v>
@@ -5290,10 +5290,10 @@
         <v>0.2758692418831542</v>
       </c>
       <c r="T70">
-        <v>0.37979608404357101</v>
+        <v>-0.37979608404357101</v>
       </c>
       <c r="U70">
-        <v>0.26737718841292057</v>
+        <v>-0.26737718841292057</v>
       </c>
       <c r="X70">
         <v>102.77</v>
@@ -5373,10 +5373,10 @@
         <v>0.27513509219369092</v>
       </c>
       <c r="T71">
-        <v>0.57964449709142496</v>
+        <v>-0.57964449709142496</v>
       </c>
       <c r="U71">
-        <v>0.16361967430429392</v>
+        <v>-0.16361967430429392</v>
       </c>
       <c r="X71">
         <v>104.5</v>
@@ -5456,10 +5456,10 @@
         <v>0.27549964208727562</v>
       </c>
       <c r="T72">
-        <v>-5.2159896193981758E-2</v>
+        <v>5.2159896193981758E-2</v>
       </c>
       <c r="U72">
-        <v>0.21845648353326919</v>
+        <v>-0.21845648353326919</v>
       </c>
       <c r="X72">
         <v>103.12</v>
@@ -5539,10 +5539,10 @@
         <v>0.27520300471504167</v>
       </c>
       <c r="T73">
-        <v>-7.572169786351779E-2</v>
+        <v>7.572169786351779E-2</v>
       </c>
       <c r="U73">
-        <v>0.28913420023759517</v>
+        <v>-0.28913420023759517</v>
       </c>
       <c r="X73">
         <v>103.25</v>
@@ -5622,10 +5622,10 @@
         <v>0.27402045842780243</v>
       </c>
       <c r="T74">
-        <v>0.26348073682957995</v>
+        <v>-0.26348073682957995</v>
       </c>
       <c r="U74">
-        <v>0.20345450907375273</v>
+        <v>-0.20345450907375273</v>
       </c>
       <c r="X74">
         <v>104.53</v>
@@ -5705,10 +5705,10 @@
         <v>0.27391958659078125</v>
       </c>
       <c r="T75">
-        <v>0.6666986310522427</v>
+        <v>-0.6666986310522427</v>
       </c>
       <c r="U75">
-        <v>0.17453300347749501</v>
+        <v>-0.17453300347749501</v>
       </c>
       <c r="X75">
         <v>104.75</v>
@@ -5788,10 +5788,10 @@
         <v>0.27091916960983436</v>
       </c>
       <c r="T76">
-        <v>6.6392380503632609E-2</v>
+        <v>-6.6392380503632609E-2</v>
       </c>
       <c r="U76">
-        <v>0.47892168775085509</v>
+        <v>-0.47892168775085509</v>
       </c>
       <c r="X76">
         <v>103.49</v>
@@ -5871,10 +5871,10 @@
         <v>0.26958271296067776</v>
       </c>
       <c r="T77">
-        <v>0.28104290803347975</v>
+        <v>-0.28104290803347975</v>
       </c>
       <c r="U77">
-        <v>0.30434451800576134</v>
+        <v>-0.30434451800576134</v>
       </c>
       <c r="X77">
         <v>104.75</v>
@@ -5954,10 +5954,10 @@
         <v>0.26864838176409989</v>
       </c>
       <c r="T78">
-        <v>0.17649388956055834</v>
+        <v>-0.17649388956055834</v>
       </c>
       <c r="U78">
-        <v>0.35494757473324423</v>
+        <v>-0.35494757473324423</v>
       </c>
       <c r="X78">
         <v>104.75</v>
@@ -6037,10 +6037,10 @@
         <v>0.26807217245172865</v>
       </c>
       <c r="T79">
-        <v>-0.17264079153496148</v>
+        <v>0.17264079153496148</v>
       </c>
       <c r="U79">
-        <v>0.40006263469034575</v>
+        <v>-0.40006263469034575</v>
       </c>
       <c r="X79">
         <v>103.3</v>
@@ -6120,10 +6120,10 @@
         <v>0.25942231680543143</v>
       </c>
       <c r="T80">
-        <v>0.1726325058544198</v>
+        <v>-0.1726325058544198</v>
       </c>
       <c r="U80">
-        <v>1.0979708851545311</v>
+        <v>-1.0979708851545311</v>
       </c>
       <c r="X80">
         <v>103.44</v>
@@ -6203,10 +6203,10 @@
         <v>0.25931016820421837</v>
       </c>
       <c r="T81">
-        <v>0.62741805730919253</v>
+        <v>-0.62741805730919253</v>
       </c>
       <c r="U81">
-        <v>0.6268124387514451</v>
+        <v>-0.6268124387514451</v>
       </c>
       <c r="X81">
         <v>103.1</v>
@@ -6286,10 +6286,10 @@
         <v>0.25453031504029922</v>
       </c>
       <c r="T82">
-        <v>-7.9425563956525558E-2</v>
+        <v>7.9425563956525558E-2</v>
       </c>
       <c r="U82">
-        <v>0.37241665443319416</v>
+        <v>-0.37241665443319416</v>
       </c>
       <c r="X82">
         <v>103.1</v>
@@ -6369,10 +6369,10 @@
         <v>0.25460218481223845</v>
       </c>
       <c r="T83">
-        <v>-2.0487719904060953E-2</v>
+        <v>2.0487719904060953E-2</v>
       </c>
       <c r="U83">
-        <v>0.42704144118119736</v>
+        <v>-0.42704144118119736</v>
       </c>
       <c r="X83">
         <v>103.07</v>
@@ -6452,10 +6452,10 @@
         <v>0.2597211988327276</v>
       </c>
       <c r="T84">
-        <v>-0.31708950793074564</v>
+        <v>0.31708950793074564</v>
       </c>
       <c r="U84">
-        <v>-4.8221518696722754E-2</v>
+        <v>4.8221518696722754E-2</v>
       </c>
       <c r="X84">
         <v>104.75</v>
@@ -6535,10 +6535,10 @@
         <v>0.25981546970534919</v>
       </c>
       <c r="T85">
-        <v>-0.32103377549155265</v>
+        <v>0.32103377549155265</v>
       </c>
       <c r="U85">
-        <v>0.21045808944302191</v>
+        <v>-0.21045808944302191</v>
       </c>
       <c r="X85">
         <v>103.25</v>
@@ -6618,10 +6618,10 @@
         <v>0.25994572451340098</v>
       </c>
       <c r="T86">
-        <v>-0.29325599026068794</v>
+        <v>0.29325599026068794</v>
       </c>
       <c r="U86">
-        <v>0.18038162998019747</v>
+        <v>-0.18038162998019747</v>
       </c>
       <c r="X86">
         <v>104.74</v>
@@ -6701,10 +6701,10 @@
         <v>0.254482297358672</v>
       </c>
       <c r="T87">
-        <v>-0.23710927772604418</v>
+        <v>0.23710927772604418</v>
       </c>
       <c r="U87">
-        <v>0.61120888189845068</v>
+        <v>-0.61120888189845068</v>
       </c>
       <c r="X87">
         <v>104.22</v>
@@ -6784,10 +6784,10 @@
         <v>0.24400101328765966</v>
       </c>
       <c r="T88">
-        <v>-0.15486061074869717</v>
+        <v>0.15486061074869717</v>
       </c>
       <c r="U88">
-        <v>0.1070559420852879</v>
+        <v>-0.1070559420852879</v>
       </c>
       <c r="X88">
         <v>105.79</v>
@@ -6867,10 +6867,10 @@
         <v>0.24416673299195407</v>
       </c>
       <c r="T89">
-        <v>1.8808636546729929E-2</v>
+        <v>-1.8808636546729929E-2</v>
       </c>
       <c r="U89">
-        <v>0.18184327526700184</v>
+        <v>-0.18184327526700184</v>
       </c>
       <c r="X89">
         <v>105.43</v>
@@ -6950,10 +6950,10 @@
         <v>0.24266356764227068</v>
       </c>
       <c r="T90">
-        <v>0.21312240273978489</v>
+        <v>-0.21312240273978489</v>
       </c>
       <c r="U90">
-        <v>-8.7144885698720032E-3</v>
+        <v>8.7144885698720032E-3</v>
       </c>
       <c r="X90">
         <v>105.65</v>
@@ -7033,10 +7033,10 @@
         <v>0.24277497438618431</v>
       </c>
       <c r="T91">
-        <v>-0.12978836687695949</v>
+        <v>0.12978836687695949</v>
       </c>
       <c r="U91">
-        <v>-1.7519673932953062E-2</v>
+        <v>1.7519673932953062E-2</v>
       </c>
       <c r="X91">
         <v>106.2</v>
@@ -7116,10 +7116,10 @@
         <v>0.24696107729170552</v>
       </c>
       <c r="T92">
-        <v>9.5196805924180339E-2</v>
+        <v>-9.5196805924180339E-2</v>
       </c>
       <c r="U92">
-        <v>0.1994358251707018</v>
+        <v>-0.1994358251707018</v>
       </c>
       <c r="X92">
         <v>106.14</v>
@@ -7199,10 +7199,10 @@
         <v>0.24676334915942968</v>
       </c>
       <c r="T93">
-        <v>0.3593938631895055</v>
+        <v>-0.3593938631895055</v>
       </c>
       <c r="U93">
-        <v>0.17199032617507548</v>
+        <v>-0.17199032617507548</v>
       </c>
       <c r="X93">
         <v>106.4</v>
@@ -7282,10 +7282,10 @@
         <v>0.24588432580840533</v>
       </c>
       <c r="T94">
-        <v>0.51564013364808758</v>
+        <v>-0.51564013364808758</v>
       </c>
       <c r="U94">
-        <v>0.47532837274280038</v>
+        <v>-0.47532837274280038</v>
       </c>
       <c r="X94">
         <v>105.51</v>
@@ -7365,10 +7365,10 @@
         <v>0.24502290499909471</v>
       </c>
       <c r="T95">
-        <v>0.5604552923748285</v>
+        <v>-0.5604552923748285</v>
       </c>
       <c r="U95">
-        <v>0.36366482543028766</v>
+        <v>-0.36366482543028766</v>
       </c>
       <c r="X95">
         <v>106.2</v>
@@ -7448,10 +7448,10 @@
         <v>0.24409085322714461</v>
       </c>
       <c r="T96">
-        <v>0.57467243637374654</v>
+        <v>-0.57467243637374654</v>
       </c>
       <c r="U96">
-        <v>0.76497993599617953</v>
+        <v>-0.76497993599617953</v>
       </c>
       <c r="X96">
         <v>106.2</v>
@@ -7531,10 +7531,10 @@
         <v>0.24299058947557031</v>
       </c>
       <c r="T97">
-        <v>0.65358020448542664</v>
+        <v>-0.65358020448542664</v>
       </c>
       <c r="U97">
-        <v>0.57717286181795391</v>
+        <v>-0.57717286181795391</v>
       </c>
       <c r="X97">
         <v>105.7</v>
@@ -7614,10 +7614,10 @@
         <v>0.24939709482174185</v>
       </c>
       <c r="T98">
-        <v>-3.3719781034635687E-2</v>
+        <v>3.3719781034635687E-2</v>
       </c>
       <c r="U98">
-        <v>0.32011494468136004</v>
+        <v>-0.32011494468136004</v>
       </c>
       <c r="X98">
         <v>104.15</v>
@@ -7697,10 +7697,10 @@
         <v>0.24727965122663029</v>
       </c>
       <c r="T99">
-        <v>-3.3090260285795203E-2</v>
+        <v>3.3090260285795203E-2</v>
       </c>
       <c r="U99">
-        <v>0.55006086213813532</v>
+        <v>-0.55006086213813532</v>
       </c>
       <c r="X99">
         <v>106.5</v>
@@ -7780,10 +7780,10 @@
         <v>0.24770644886637477</v>
       </c>
       <c r="T100">
-        <v>0.30239270077903058</v>
+        <v>-0.30239270077903058</v>
       </c>
       <c r="U100">
-        <v>0.69517769454652267</v>
+        <v>-0.69517769454652267</v>
       </c>
       <c r="X100">
         <v>105.65</v>
@@ -7863,10 +7863,10 @@
         <v>0.24713807229731125</v>
       </c>
       <c r="T101">
-        <v>0.20296212724753016</v>
+        <v>-0.20296212724753016</v>
       </c>
       <c r="U101">
-        <v>0.79531416800475707</v>
+        <v>-0.79531416800475707</v>
       </c>
       <c r="X101">
         <v>106</v>
@@ -7946,10 +7946,10 @@
         <v>0.2269077514804535</v>
       </c>
       <c r="T102">
-        <v>5.8110151570667234E-2</v>
+        <v>-5.8110151570667234E-2</v>
       </c>
       <c r="U102">
-        <v>6.6956234438420026E-3</v>
+        <v>-6.6956234438420026E-3</v>
       </c>
       <c r="X102">
         <v>106</v>
@@ -8029,10 +8029,10 @@
         <v>0.2270670152903306</v>
       </c>
       <c r="T103">
-        <v>2.4759762355830439E-2</v>
+        <v>-2.4759762355830439E-2</v>
       </c>
       <c r="U103">
-        <v>-5.1333977562628696E-2</v>
+        <v>5.1333977562628696E-2</v>
       </c>
       <c r="X103">
         <v>105.21</v>
@@ -8112,10 +8112,10 @@
         <v>0.23427842684394432</v>
       </c>
       <c r="T104">
-        <v>-0.64672724533747505</v>
+        <v>0.64672724533747505</v>
       </c>
       <c r="U104">
-        <v>-0.39418540160935933</v>
+        <v>0.39418540160935933</v>
       </c>
       <c r="X104">
         <v>104.7</v>
@@ -8195,10 +8195,10 @@
         <v>0.23238257438899379</v>
       </c>
       <c r="T105">
-        <v>-0.43132956116540555</v>
+        <v>0.43132956116540555</v>
       </c>
       <c r="U105">
-        <v>0.23864827686550516</v>
+        <v>-0.23864827686550516</v>
       </c>
       <c r="X105">
         <v>106</v>
@@ -8278,10 +8278,10 @@
         <v>0.2200227685886656</v>
       </c>
       <c r="T106">
-        <v>-0.48802320103100705</v>
+        <v>0.48802320103100705</v>
       </c>
       <c r="U106">
-        <v>-0.42957003612986711</v>
+        <v>0.42957003612986711</v>
       </c>
       <c r="X106">
         <v>105.84</v>
@@ -8361,10 +8361,10 @@
         <v>0.21916697381554928</v>
       </c>
       <c r="T107">
-        <v>-0.49631677293611176</v>
+        <v>0.49631677293611176</v>
       </c>
       <c r="U107">
-        <v>-0.21784168580061269</v>
+        <v>0.21784168580061269</v>
       </c>
       <c r="X107">
         <v>105.5</v>
@@ -8444,10 +8444,10 @@
         <v>0.22326205299828963</v>
       </c>
       <c r="T108">
-        <v>-0.59549361087249952</v>
+        <v>0.59549361087249952</v>
       </c>
       <c r="U108">
-        <v>-0.42544284597416659</v>
+        <v>0.42544284597416659</v>
       </c>
       <c r="X108">
         <v>106.9</v>
@@ -8527,10 +8527,10 @@
         <v>0.22348566183104573</v>
       </c>
       <c r="T109">
-        <v>-0.22672699630754689</v>
+        <v>0.22672699630754689</v>
       </c>
       <c r="U109">
-        <v>-0.40923019372558489</v>
+        <v>0.40923019372558489</v>
       </c>
       <c r="X109">
         <v>107.4</v>
@@ -8610,10 +8610,10 @@
         <v>0.22995520347818257</v>
       </c>
       <c r="T110">
-        <v>8.3755622093684146E-2</v>
+        <v>-8.3755622093684146E-2</v>
       </c>
       <c r="U110">
-        <v>0.26337714382669297</v>
+        <v>-0.26337714382669297</v>
       </c>
       <c r="X110">
         <v>107.7</v>
@@ -8693,10 +8693,10 @@
         <v>0.21540457911946564</v>
       </c>
       <c r="T111">
-        <v>4.7004986292820128E-2</v>
+        <v>-4.7004986292820128E-2</v>
       </c>
       <c r="U111">
-        <v>0.6948279098613952</v>
+        <v>-0.6948279098613952</v>
       </c>
       <c r="X111">
         <v>107.57</v>
@@ -8776,10 +8776,10 @@
         <v>0.1859227484499687</v>
       </c>
       <c r="T112">
-        <v>-0.39887047597444436</v>
+        <v>0.39887047597444436</v>
       </c>
       <c r="U112">
-        <v>-0.48752433974186271</v>
+        <v>0.48752433974186271</v>
       </c>
       <c r="X112">
         <v>107</v>
@@ -8859,10 +8859,10 @@
         <v>0.19159021570548326</v>
       </c>
       <c r="T113">
-        <v>-9.377635323202238E-2</v>
+        <v>9.377635323202238E-2</v>
       </c>
       <c r="U113">
-        <v>-0.11647618452903519</v>
+        <v>0.11647618452903519</v>
       </c>
       <c r="X113">
         <v>108.2</v>
@@ -8942,10 +8942,10 @@
         <v>0.2012171886494655</v>
       </c>
       <c r="T114">
-        <v>0.81202610866766278</v>
+        <v>-0.81202610866766278</v>
       </c>
       <c r="U114">
-        <v>0.50316184625716076</v>
+        <v>-0.50316184625716076</v>
       </c>
       <c r="X114">
         <v>108.4</v>
@@ -9025,10 +9025,10 @@
         <v>0.20538678769212571</v>
       </c>
       <c r="T115">
-        <v>1.0324625573207458</v>
+        <v>-1.0324625573207458</v>
       </c>
       <c r="U115">
-        <v>0.726997119700723</v>
+        <v>-0.726997119700723</v>
       </c>
       <c r="X115">
         <v>108</v>
@@ -9108,10 +9108,10 @@
         <v>0.2307657573804282</v>
       </c>
       <c r="T116">
-        <v>0.28602310631313799</v>
+        <v>-0.28602310631313799</v>
       </c>
       <c r="U116">
-        <v>-6.1476236171698062E-3</v>
+        <v>6.1476236171698062E-3</v>
       </c>
       <c r="X116">
         <v>107.5</v>
@@ -9191,10 +9191,10 @@
         <v>0.23077179250732655</v>
       </c>
       <c r="T117">
-        <v>0.22650774335788437</v>
+        <v>-0.22650774335788437</v>
       </c>
       <c r="U117">
-        <v>-8.3729439149360374E-3</v>
+        <v>8.3729439149360374E-3</v>
       </c>
       <c r="X117">
         <v>107.17</v>
@@ -9274,10 +9274,10 @@
         <v>0.23080633160768274</v>
       </c>
       <c r="T118">
-        <v>0.17965099888463953</v>
+        <v>-0.17965099888463953</v>
       </c>
       <c r="U118">
-        <v>2.7146709000347435E-2</v>
+        <v>-2.7146709000347435E-2</v>
       </c>
       <c r="X118">
         <v>107.8</v>
@@ -9357,10 +9357,10 @@
         <v>0.23048210443713202</v>
       </c>
       <c r="T119">
-        <v>0.1415297221213585</v>
+        <v>-0.1415297221213585</v>
       </c>
       <c r="U119">
-        <v>0.16426081005671556</v>
+        <v>-0.16426081005671556</v>
       </c>
       <c r="X119">
         <v>107.01</v>
@@ -9440,10 +9440,10 @@
         <v>0.22945630946908371</v>
       </c>
       <c r="T120">
-        <v>0.11817131974407591</v>
+        <v>-0.11817131974407591</v>
       </c>
       <c r="U120">
-        <v>0.3372835600634394</v>
+        <v>-0.3372835600634394</v>
       </c>
       <c r="X120">
         <v>107.7</v>
@@ -9523,10 +9523,10 @@
         <v>0.22907592714945377</v>
       </c>
       <c r="T121">
-        <v>0.41348911058090021</v>
+        <v>-0.41348911058090021</v>
       </c>
       <c r="U121">
-        <v>0.29256446096310729</v>
+        <v>-0.29256446096310729</v>
       </c>
       <c r="X121">
         <v>107.7</v>
@@ -9606,10 +9606,10 @@
         <v>0.22809461959824093</v>
       </c>
       <c r="T122">
-        <v>7.4746882628629052E-2</v>
+        <v>-7.4746882628629052E-2</v>
       </c>
       <c r="U122">
-        <v>0.17271167037851143</v>
+        <v>-0.17271167037851143</v>
       </c>
       <c r="X122">
         <v>107.01</v>
@@ -9689,10 +9689,10 @@
         <v>0.2279975399464414</v>
       </c>
       <c r="T123">
-        <v>-0.17827217482873081</v>
+        <v>0.17827217482873081</v>
       </c>
       <c r="U123">
-        <v>0.18092238360123414</v>
+        <v>-0.18092238360123414</v>
       </c>
       <c r="X123">
         <v>107.95</v>
@@ -9772,10 +9772,10 @@
         <v>0.22841601667406114</v>
       </c>
       <c r="T124">
-        <v>-0.40371994531223088</v>
+        <v>0.40371994531223088</v>
       </c>
       <c r="U124">
-        <v>0.11158020921380185</v>
+        <v>-0.11158020921380185</v>
       </c>
       <c r="X124">
         <v>107.05</v>
@@ -9855,10 +9855,10 @@
         <v>0.22841869991788089</v>
       </c>
       <c r="T125">
-        <v>-0.44930908288656202</v>
+        <v>0.44930908288656202</v>
       </c>
       <c r="U125">
-        <v>0.11317914294735054</v>
+        <v>-0.11317914294735054</v>
       </c>
       <c r="X125">
         <v>107.65</v>
@@ -9938,10 +9938,10 @@
         <v>0.22767052140411681</v>
       </c>
       <c r="T126">
-        <v>-0.67435222876106593</v>
+        <v>0.67435222876106593</v>
       </c>
       <c r="U126">
-        <v>-9.8822432512424285E-2</v>
+        <v>9.8822432512424285E-2</v>
       </c>
       <c r="X126">
         <v>107.79</v>
@@ -10021,10 +10021,10 @@
         <v>0.23007500322865471</v>
       </c>
       <c r="T127">
-        <v>-0.41363097531010862</v>
+        <v>0.41363097531010862</v>
       </c>
       <c r="U127">
-        <v>0.24857345942839171</v>
+        <v>-0.24857345942839171</v>
       </c>
       <c r="X127">
         <v>108</v>
@@ -10104,10 +10104,10 @@
         <v>0.22947181475881628</v>
       </c>
       <c r="T128">
-        <v>0.22597372916444147</v>
+        <v>-0.22597372916444147</v>
       </c>
       <c r="U128">
-        <v>0.19524105954462634</v>
+        <v>-0.19524105954462634</v>
       </c>
       <c r="X128">
         <v>107.32</v>
@@ -10187,10 +10187,10 @@
         <v>0.2294915209250169</v>
       </c>
       <c r="T129">
-        <v>0.2864674121396904</v>
+        <v>-0.2864674121396904</v>
       </c>
       <c r="U129">
-        <v>0.2567177827104361</v>
+        <v>-0.2567177827104361</v>
       </c>
       <c r="X129">
         <v>107.77</v>
@@ -10270,10 +10270,10 @@
         <v>0.22801918370904664</v>
       </c>
       <c r="T130">
-        <v>9.0824269267431035E-2</v>
+        <v>-9.0824269267431035E-2</v>
       </c>
       <c r="U130">
-        <v>0.39953048989407325</v>
+        <v>-0.39953048989407325</v>
       </c>
       <c r="X130">
         <v>107.8</v>
@@ -10353,10 +10353,10 @@
         <v>0.22857298889539718</v>
       </c>
       <c r="T131">
-        <v>0.26446998213229822</v>
+        <v>-0.26446998213229822</v>
       </c>
       <c r="U131">
-        <v>0.4739233687379496</v>
+        <v>-0.4739233687379496</v>
       </c>
       <c r="X131">
         <v>107.14</v>
@@ -10436,10 +10436,10 @@
         <v>0.227932641472535</v>
       </c>
       <c r="T132">
-        <v>0.30301510122978659</v>
+        <v>-0.30301510122978659</v>
       </c>
       <c r="U132">
-        <v>0.36579822857243371</v>
+        <v>-0.36579822857243371</v>
       </c>
       <c r="X132">
         <v>107.6</v>
@@ -10519,10 +10519,10 @@
         <v>0.22788420678328958</v>
       </c>
       <c r="T133">
-        <v>0.36008544667300857</v>
+        <v>-0.36008544667300857</v>
       </c>
       <c r="U133">
-        <v>0.38994838798873666</v>
+        <v>-0.38994838798873666</v>
       </c>
       <c r="X133">
         <v>107.28</v>
@@ -10602,10 +10602,10 @@
         <v>0.23094184841984219</v>
       </c>
       <c r="T134">
-        <v>0.47970014651050885</v>
+        <v>-0.47970014651050885</v>
       </c>
       <c r="U134">
-        <v>-0.16498637432473817</v>
+        <v>0.16498637432473817</v>
       </c>
       <c r="X134">
         <v>107.3</v>
@@ -10685,10 +10685,10 @@
         <v>0.23183548219453329</v>
       </c>
       <c r="T135">
-        <v>4.6551211628620415E-2</v>
+        <v>-4.6551211628620415E-2</v>
       </c>
       <c r="U135">
-        <v>-0.38868785055476973</v>
+        <v>0.38868785055476973</v>
       </c>
       <c r="X135">
         <v>106.81</v>
@@ -10768,10 +10768,10 @@
         <v>0.23201946302388454</v>
       </c>
       <c r="T136">
-        <v>0.17850427697416738</v>
+        <v>-0.17850427697416738</v>
       </c>
       <c r="U136">
-        <v>-0.31000332551156529</v>
+        <v>0.31000332551156529</v>
       </c>
       <c r="X136">
         <v>107.13</v>
@@ -10851,10 +10851,10 @@
         <v>0.2319246038235451</v>
       </c>
       <c r="T137">
-        <v>0.11090301635401367</v>
+        <v>-0.11090301635401367</v>
       </c>
       <c r="U137">
-        <v>-0.38652766153353113</v>
+        <v>0.38652766153353113</v>
       </c>
       <c r="X137">
         <v>106.9</v>
@@ -10934,10 +10934,10 @@
         <v>0.22917474737888954</v>
       </c>
       <c r="T138">
-        <v>0.4941409216229431</v>
+        <v>-0.4941409216229431</v>
       </c>
       <c r="U138">
-        <v>-9.0354586409380211E-2</v>
+        <v>9.0354586409380211E-2</v>
       </c>
       <c r="X138">
         <v>107.8</v>
@@ -11017,10 +11017,10 @@
         <v>0.22802410206859675</v>
       </c>
       <c r="T139">
-        <v>0.28652744856234591</v>
+        <v>-0.28652744856234591</v>
       </c>
       <c r="U139">
-        <v>6.7636724900088652E-2</v>
+        <v>-6.7636724900088652E-2</v>
       </c>
       <c r="X139">
         <v>107.99</v>
@@ -11100,10 +11100,10 @@
         <v>0.22830531855111266</v>
       </c>
       <c r="T140">
-        <v>7.5325130670655938E-3</v>
+        <v>-7.5325130670655938E-3</v>
       </c>
       <c r="U140">
-        <v>9.1824806232043699E-2</v>
+        <v>-9.1824806232043699E-2</v>
       </c>
       <c r="X140">
         <v>108</v>
@@ -11183,10 +11183,10 @@
         <v>0.22661620696769977</v>
       </c>
       <c r="T141">
-        <v>0.23330900941431754</v>
+        <v>-0.23330900941431754</v>
       </c>
       <c r="U141">
-        <v>0.28766014673582418</v>
+        <v>-0.28766014673582418</v>
       </c>
       <c r="X141">
         <v>107.46</v>
@@ -11266,10 +11266,10 @@
         <v>0.22643523727510481</v>
       </c>
       <c r="T142">
-        <v>0.32722096304126369</v>
+        <v>-0.32722096304126369</v>
       </c>
       <c r="U142">
-        <v>-6.255365043086325E-2</v>
+        <v>6.255365043086325E-2</v>
       </c>
       <c r="X142">
         <v>108</v>
@@ -11349,10 +11349,10 @@
         <v>0.2270084227649799</v>
       </c>
       <c r="T143">
-        <v>0.11138139898569932</v>
+        <v>-0.11138139898569932</v>
       </c>
       <c r="U143">
-        <v>2.0869160093739403E-2</v>
+        <v>-2.0869160093739403E-2</v>
       </c>
       <c r="X143">
         <v>107.2</v>
@@ -11432,10 +11432,10 @@
         <v>0.22150323347788839</v>
       </c>
       <c r="T144">
-        <v>-0.49325561235988857</v>
+        <v>0.49325561235988857</v>
       </c>
       <c r="U144">
-        <v>0.31302940705530968</v>
+        <v>-0.31302940705530968</v>
       </c>
       <c r="X144">
         <v>107.41</v>
@@ -11515,10 +11515,10 @@
         <v>0.22153791904756709</v>
       </c>
       <c r="T145">
-        <v>-0.71160457022736434</v>
+        <v>0.71160457022736434</v>
       </c>
       <c r="U145">
-        <v>0.31651646248282983</v>
+        <v>-0.31651646248282983</v>
       </c>
       <c r="X145">
         <v>108</v>
@@ -11598,10 +11598,10 @@
         <v>0.2214576864088541</v>
       </c>
       <c r="T146">
-        <v>0.18746223368319992</v>
+        <v>-0.18746223368319992</v>
       </c>
       <c r="U146">
-        <v>0.47978581308112389</v>
+        <v>-0.47978581308112389</v>
       </c>
       <c r="X146">
         <v>107.2</v>
@@ -11681,10 +11681,10 @@
         <v>0.22146489066150166</v>
       </c>
       <c r="T147">
-        <v>0.25279277609948636</v>
+        <v>-0.25279277609948636</v>
       </c>
       <c r="U147">
-        <v>0.48531090121424203</v>
+        <v>-0.48531090121424203</v>
       </c>
       <c r="X147">
         <v>108.8</v>
@@ -11764,10 +11764,10 @@
         <v>0.22169032115875903</v>
       </c>
       <c r="T148">
-        <v>0.12269426037452291</v>
+        <v>-0.12269426037452291</v>
       </c>
       <c r="U148">
-        <v>0.30588403471243364</v>
+        <v>-0.30588403471243364</v>
       </c>
       <c r="X148">
         <v>108.94</v>
@@ -11847,10 +11847,10 @@
         <v>0.22216005968669297</v>
       </c>
       <c r="T149">
-        <v>-3.9661716418071258E-2</v>
+        <v>3.9661716418071258E-2</v>
       </c>
       <c r="U149">
-        <v>0.10264442924319273</v>
+        <v>-0.10264442924319273</v>
       </c>
       <c r="X149">
         <v>109.18</v>
@@ -11930,10 +11930,10 @@
         <v>0.22427760862462112</v>
       </c>
       <c r="T150">
-        <v>0.1990650171509234</v>
+        <v>-0.1990650171509234</v>
       </c>
       <c r="U150">
-        <v>0.32099404731047443</v>
+        <v>-0.32099404731047443</v>
       </c>
       <c r="X150">
         <v>108.34</v>
@@ -12013,10 +12013,10 @@
         <v>0.22405500052299493</v>
       </c>
       <c r="T151">
-        <v>-7.9978265063895826E-2</v>
+        <v>7.9978265063895826E-2</v>
       </c>
       <c r="U151">
-        <v>0.33680177888699703</v>
+        <v>-0.33680177888699703</v>
       </c>
       <c r="X151">
         <v>108.34</v>
@@ -12096,10 +12096,10 @@
         <v>0.21812385494207495</v>
       </c>
       <c r="T152">
-        <v>-0.1444697243025761</v>
+        <v>0.1444697243025761</v>
       </c>
       <c r="U152">
-        <v>-7.036388283832018E-2</v>
+        <v>7.036388283832018E-2</v>
       </c>
       <c r="X152">
         <v>107.7</v>
@@ -12179,10 +12179,10 @@
         <v>0.21817887784961579</v>
       </c>
       <c r="T153">
-        <v>0.1154668606887066</v>
+        <v>-0.1154668606887066</v>
       </c>
       <c r="U153">
-        <v>-6.3421144473085889E-2</v>
+        <v>6.3421144473085889E-2</v>
       </c>
       <c r="X153">
         <v>108.2</v>
@@ -12262,10 +12262,10 @@
         <v>0.2177795581671215</v>
       </c>
       <c r="T154">
-        <v>0.18909056136540148</v>
+        <v>-0.18909056136540148</v>
       </c>
       <c r="U154">
-        <v>-0.21564195242680384</v>
+        <v>0.21564195242680384</v>
       </c>
       <c r="X154">
         <v>108</v>
@@ -12345,10 +12345,10 @@
         <v>0.21778907197612038</v>
       </c>
       <c r="T155">
-        <v>8.1659754039309362E-2</v>
+        <v>-8.1659754039309362E-2</v>
       </c>
       <c r="U155">
-        <v>-0.37018829151662658</v>
+        <v>0.37018829151662658</v>
       </c>
       <c r="X155">
         <v>108.6</v>
@@ -12428,10 +12428,10 @@
         <v>0.21797078302504472</v>
       </c>
       <c r="T156">
-        <v>0.31565828258361961</v>
+        <v>-0.31565828258361961</v>
       </c>
       <c r="U156">
-        <v>-0.35709277807798312</v>
+        <v>0.35709277807798312</v>
       </c>
       <c r="X156">
         <v>109.2</v>
@@ -12511,10 +12511,10 @@
         <v>0.21833392936460574</v>
       </c>
       <c r="T157">
-        <v>0.141341981405807</v>
+        <v>-0.141341981405807</v>
       </c>
       <c r="U157">
-        <v>-0.27182035438633179</v>
+        <v>0.27182035438633179</v>
       </c>
       <c r="X157">
         <v>108.94</v>
@@ -12594,10 +12594,10 @@
         <v>0.20891913434482795</v>
       </c>
       <c r="T158">
-        <v>-5.8425110761728405E-2</v>
+        <v>5.8425110761728405E-2</v>
       </c>
       <c r="U158">
-        <v>0.16820339032341813</v>
+        <v>-0.16820339032341813</v>
       </c>
       <c r="X158">
         <v>109.01</v>
@@ -12677,10 +12677,10 @@
         <v>0.20954465463950667</v>
       </c>
       <c r="T159">
-        <v>-0.22246237508241062</v>
+        <v>0.22246237508241062</v>
       </c>
       <c r="U159">
-        <v>6.2539346481993441E-2</v>
+        <v>-6.2539346481993441E-2</v>
       </c>
       <c r="X159">
         <v>108.27</v>
@@ -12760,10 +12760,10 @@
         <v>0.20917014083065866</v>
       </c>
       <c r="T160">
-        <v>-0.2360271777374523</v>
+        <v>0.2360271777374523</v>
       </c>
       <c r="U160">
-        <v>-0.14824427060866618</v>
+        <v>0.14824427060866618</v>
       </c>
       <c r="X160">
         <v>109</v>
@@ -12843,10 +12843,10 @@
         <v>0.2096712666752919</v>
       </c>
       <c r="T161">
-        <v>-0.50335690922462817</v>
+        <v>0.50335690922462817</v>
       </c>
       <c r="U161">
-        <v>-0.24265528535967196</v>
+        <v>0.24265528535967196</v>
       </c>
       <c r="X161">
         <v>108.61</v>
@@ -12926,10 +12926,10 @@
         <v>0.20971076747614931</v>
       </c>
       <c r="T162">
-        <v>-0.57858333323812516</v>
+        <v>0.57858333323812516</v>
       </c>
       <c r="U162">
-        <v>-0.27790877106221856</v>
+        <v>0.27790877106221856</v>
       </c>
       <c r="X162">
         <v>109</v>
@@ -13009,10 +13009,10 @@
         <v>0.20976349372491251</v>
       </c>
       <c r="T163">
-        <v>-0.49847967855896069</v>
+        <v>0.49847967855896069</v>
       </c>
       <c r="U163">
-        <v>-0.13829825330182732</v>
+        <v>0.13829825330182732</v>
       </c>
       <c r="X163">
         <v>108.89</v>
@@ -13092,10 +13092,10 @@
         <v>0.20096262302658896</v>
       </c>
       <c r="T164">
-        <v>-0.21672467914106708</v>
+        <v>0.21672467914106708</v>
       </c>
       <c r="U164">
-        <v>0.27067420207991244</v>
+        <v>-0.27067420207991244</v>
       </c>
       <c r="X164">
         <v>109.2</v>
@@ -13175,10 +13175,10 @@
         <v>0.19824901131054753</v>
       </c>
       <c r="T165">
-        <v>7.8378729542194492E-3</v>
+        <v>-7.8378729542194492E-3</v>
       </c>
       <c r="U165">
-        <v>5.5365621200409443E-2</v>
+        <v>-5.5365621200409443E-2</v>
       </c>
       <c r="X165">
         <v>108.94</v>
@@ -13258,10 +13258,10 @@
         <v>0.19863391301325339</v>
       </c>
       <c r="T166">
-        <v>-0.17610912769512321</v>
+        <v>0.17610912769512321</v>
       </c>
       <c r="U166">
-        <v>4.1440716202156835E-3</v>
+        <v>-4.1440716202156835E-3</v>
       </c>
       <c r="X166">
         <v>109.49</v>
@@ -13341,10 +13341,10 @@
         <v>0.20215282908732948</v>
       </c>
       <c r="T167">
-        <v>0.14769801730061261</v>
+        <v>-0.14769801730061261</v>
       </c>
       <c r="U167">
-        <v>0.26194391239253711</v>
+        <v>-0.26194391239253711</v>
       </c>
       <c r="X167">
         <v>109.53</v>
@@ -13424,10 +13424,10 @@
         <v>0.19627062393468253</v>
       </c>
       <c r="T168">
-        <v>6.3513747110843788E-2</v>
+        <v>-6.3513747110843788E-2</v>
       </c>
       <c r="U168">
-        <v>0.5668618960751548</v>
+        <v>-0.5668618960751548</v>
       </c>
       <c r="X168">
         <v>109.8</v>
@@ -13507,10 +13507,10 @@
         <v>0.19497349120694479</v>
       </c>
       <c r="T169">
-        <v>9.7139688537861701E-2</v>
+        <v>-9.7139688537861701E-2</v>
       </c>
       <c r="U169">
-        <v>0.38908332998388584</v>
+        <v>-0.38908332998388584</v>
       </c>
       <c r="X169">
         <v>109.8</v>
@@ -13590,10 +13590,10 @@
         <v>0.18590417131818632</v>
       </c>
       <c r="T170">
-        <v>-8.3800777845555174E-2</v>
+        <v>8.3800777845555174E-2</v>
       </c>
       <c r="U170">
-        <v>-7.6428795186855858E-2</v>
+        <v>7.6428795186855858E-2</v>
       </c>
       <c r="X170">
         <v>109.91</v>
@@ -13673,10 +13673,10 @@
         <v>0.18307911990349665</v>
       </c>
       <c r="T171">
-        <v>-5.9733161016661818E-2</v>
+        <v>5.9733161016661818E-2</v>
       </c>
       <c r="U171">
-        <v>0.17809566743585137</v>
+        <v>-0.17809566743585137</v>
       </c>
       <c r="X171">
         <v>109.8</v>
@@ -13756,10 +13756,10 @@
         <v>0.17992308809325749</v>
       </c>
       <c r="T172">
-        <v>0.10075237201643272</v>
+        <v>-0.10075237201643272</v>
       </c>
       <c r="U172">
-        <v>0.43483174554164172</v>
+        <v>-0.43483174554164172</v>
       </c>
       <c r="X172">
         <v>110.56</v>
@@ -13839,10 +13839,10 @@
         <v>0.17418750829181004</v>
       </c>
       <c r="T173">
-        <v>-2.7396878311747308E-2</v>
+        <v>2.7396878311747308E-2</v>
       </c>
       <c r="U173">
-        <v>8.6207685847106141E-2</v>
+        <v>-8.6207685847106141E-2</v>
       </c>
       <c r="X173">
         <v>111.04</v>
@@ -13922,10 +13922,10 @@
         <v>0.16208535544083</v>
       </c>
       <c r="T174">
-        <v>8.0303028040096258E-2</v>
+        <v>-8.0303028040096258E-2</v>
       </c>
       <c r="U174">
-        <v>-0.42288157855447928</v>
+        <v>0.42288157855447928</v>
       </c>
       <c r="X174">
         <v>112.5</v>
@@ -14005,10 +14005,10 @@
         <v>0.15571358238887623</v>
       </c>
       <c r="T175">
-        <v>3.1581570430994077E-2</v>
+        <v>-3.1581570430994077E-2</v>
       </c>
       <c r="U175">
-        <v>-0.69402685449262425</v>
+        <v>0.69402685449262425</v>
       </c>
       <c r="X175">
         <v>111.2</v>
@@ -14088,10 +14088,10 @@
         <v>0.1155415262000794</v>
       </c>
       <c r="T176">
-        <v>-0.13020486454491387</v>
+        <v>0.13020486454491387</v>
       </c>
       <c r="U176">
-        <v>6.0311127787837648E-2</v>
+        <v>-6.0311127787837648E-2</v>
       </c>
       <c r="X176">
         <v>111.2</v>
@@ -14171,10 +14171,10 @@
         <v>0.11541691058669495</v>
       </c>
       <c r="T177">
-        <v>-0.15113899663712349</v>
+        <v>0.15113899663712349</v>
       </c>
       <c r="U177">
-        <v>0.10631735945827447</v>
+        <v>-0.10631735945827447</v>
       </c>
       <c r="X177">
         <v>110.81</v>
@@ -14254,10 +14254,10 @@
         <v>0.11535353474835022</v>
       </c>
       <c r="T178">
-        <v>-4.7814121655553876E-2</v>
+        <v>4.7814121655553876E-2</v>
       </c>
       <c r="U178">
-        <v>7.7458640093208686E-2</v>
+        <v>-7.7458640093208686E-2</v>
       </c>
       <c r="X178">
         <v>111.2</v>
@@ -14337,10 +14337,10 @@
         <v>0.1152743756831454</v>
       </c>
       <c r="T179">
-        <v>7.9724812572457004E-2</v>
+        <v>-7.9724812572457004E-2</v>
       </c>
       <c r="U179">
-        <v>3.9888893607908926E-2</v>
+        <v>-3.9888893607908926E-2</v>
       </c>
       <c r="X179">
         <v>111.2</v>
@@ -14420,10 +14420,10 @@
         <v>0.11527349003511125</v>
       </c>
       <c r="T180">
-        <v>-0.16607151250811469</v>
+        <v>0.16607151250811469</v>
       </c>
       <c r="U180">
-        <v>3.6246326358146952E-2</v>
+        <v>-3.6246326358146952E-2</v>
       </c>
       <c r="X180">
         <v>110.79</v>
@@ -14509,10 +14509,10 @@
         <v>0.22836758145830718</v>
       </c>
       <c r="T181">
-        <v>1.5867701095340081E-2</v>
+        <v>-1.5867701095340081E-2</v>
       </c>
       <c r="U181">
-        <v>-6.5544497272251867E-2</v>
+        <v>6.5544497272251867E-2</v>
       </c>
       <c r="V181">
         <v>-0.18443909503138567</v>
@@ -14604,10 +14604,10 @@
         <v>0.22822902128229952</v>
       </c>
       <c r="T182">
-        <v>2.2371713088276124E-2</v>
+        <v>-2.2371713088276124E-2</v>
       </c>
       <c r="U182">
-        <v>-0.12423688190867921</v>
+        <v>0.12423688190867921</v>
       </c>
       <c r="V182">
         <v>-0.30318462588976303</v>
@@ -14699,10 +14699,10 @@
         <v>0.22822369869438269</v>
       </c>
       <c r="T183">
-        <v>-8.0911040124154177E-2</v>
+        <v>8.0911040124154177E-2</v>
       </c>
       <c r="U183">
-        <v>3.5721320448089955E-2</v>
+        <v>-3.5721320448089955E-2</v>
       </c>
       <c r="V183">
         <v>-0.2824625158833749</v>
@@ -14794,10 +14794,10 @@
         <v>0.22594600926735001</v>
       </c>
       <c r="T184">
-        <v>-5.5209740151385134E-2</v>
+        <v>5.5209740151385134E-2</v>
       </c>
       <c r="U184">
-        <v>0.13661056236884406</v>
+        <v>-0.13661056236884406</v>
       </c>
       <c r="V184">
         <v>-0.72680466200087945</v>
@@ -14889,10 +14889,10 @@
         <v>0.22384220417968759</v>
       </c>
       <c r="T185">
-        <v>4.0909623469875811E-2</v>
+        <v>-4.0909623469875811E-2</v>
       </c>
       <c r="U185">
-        <v>0.12429355059297986</v>
+        <v>-0.12429355059297986</v>
       </c>
       <c r="V185">
         <v>-0.28971663159698124</v>
@@ -14984,10 +14984,10 @@
         <v>0.22348380024425435</v>
       </c>
       <c r="T186">
-        <v>-0.13943069697774924</v>
+        <v>0.13943069697774924</v>
       </c>
       <c r="U186">
-        <v>0.18094582620744593</v>
+        <v>-0.18094582620744593</v>
       </c>
       <c r="V186">
         <v>-0.10608957263136265</v>
@@ -15079,10 +15079,10 @@
         <v>0.22289825031949953</v>
       </c>
       <c r="T187">
-        <v>-0.22520432165014093</v>
+        <v>0.22520432165014093</v>
       </c>
       <c r="U187">
-        <v>-8.2661544851858615E-2</v>
+        <v>8.2661544851858615E-2</v>
       </c>
       <c r="V187">
         <v>-0.35326785934335359</v>
@@ -15174,10 +15174,10 @@
         <v>0.22166273801026679</v>
       </c>
       <c r="T188">
-        <v>-0.17328805093892452</v>
+        <v>0.17328805093892452</v>
       </c>
       <c r="U188">
-        <v>-0.23406124189397914</v>
+        <v>0.23406124189397914</v>
       </c>
       <c r="V188">
         <v>-0.68623515299630622</v>
@@ -15269,10 +15269,10 @@
         <v>0.21661639430741686</v>
       </c>
       <c r="T189">
-        <v>-3.8248998782108856E-2</v>
+        <v>3.8248998782108856E-2</v>
       </c>
       <c r="U189">
-        <v>-0.26510084359225861</v>
+        <v>0.26510084359225861</v>
       </c>
       <c r="V189">
         <v>-2.9919578151016424E-3</v>
@@ -15364,10 +15364,10 @@
         <v>0.21397117752824016</v>
       </c>
       <c r="T190">
-        <v>4.6230264281854616E-2</v>
+        <v>-4.6230264281854616E-2</v>
       </c>
       <c r="U190">
-        <v>-0.19332504799973727</v>
+        <v>0.19332504799973727</v>
       </c>
       <c r="V190">
         <v>-0.50311807221234961</v>
@@ -15459,10 +15459,10 @@
         <v>0.21358982625314088</v>
       </c>
       <c r="T191">
-        <v>0.16272571026936244</v>
+        <v>-0.16272571026936244</v>
       </c>
       <c r="U191">
-        <v>-0.34578592164584698</v>
+        <v>0.34578592164584698</v>
       </c>
       <c r="V191">
         <v>-0.31065754673784696</v>
@@ -15554,10 +15554,10 @@
         <v>0.21349027155207903</v>
       </c>
       <c r="T192">
-        <v>0.19701321594358667</v>
+        <v>-0.19701321594358667</v>
       </c>
       <c r="U192">
-        <v>-0.38563676958665027</v>
+        <v>0.38563676958665027</v>
       </c>
       <c r="V192">
         <v>-0.21169215571339439</v>
@@ -15649,10 +15649,10 @@
         <v>0.21335307956147692</v>
       </c>
       <c r="T193">
-        <v>0.1275264413773014</v>
+        <v>-0.1275264413773014</v>
       </c>
       <c r="U193">
-        <v>-0.37415547454717757</v>
+        <v>0.37415547454717757</v>
       </c>
       <c r="V193">
         <v>-0.32397252500886431</v>
@@ -15744,10 +15744,10 @@
         <v>0.21234988595716292</v>
       </c>
       <c r="T194">
-        <v>0.20488826704756491</v>
+        <v>-0.20488826704756491</v>
       </c>
       <c r="U194">
-        <v>-9.6925957193683132E-3</v>
+        <v>9.6925957193683132E-3</v>
       </c>
       <c r="V194">
         <v>-2.8809835127119321E-2</v>
@@ -15839,10 +15839,10 @@
         <v>0.21227462566659008</v>
       </c>
       <c r="T195">
-        <v>0.15398976350833316</v>
+        <v>-0.15398976350833316</v>
       </c>
       <c r="U195">
-        <v>0.16484180777911472</v>
+        <v>-0.16484180777911472</v>
       </c>
       <c r="V195">
         <v>5.3438482164747114E-2</v>
@@ -15934,10 +15934,10 @@
         <v>0.21103620650496893</v>
       </c>
       <c r="T196">
-        <v>0.27240843741718201</v>
+        <v>-0.27240843741718201</v>
       </c>
       <c r="U196">
-        <v>0.10005194037085996</v>
+        <v>-0.10005194037085996</v>
       </c>
       <c r="V196">
         <v>-0.28506541189332602</v>
@@ -16029,10 +16029,10 @@
         <v>0.21041643826091444</v>
       </c>
       <c r="T197">
-        <v>-2.3032464182959345E-2</v>
+        <v>2.3032464182959345E-2</v>
       </c>
       <c r="U197">
-        <v>0.1251295467911584</v>
+        <v>-0.1251295467911584</v>
       </c>
       <c r="V197">
         <v>-4.665949898952082E-2</v>
@@ -16124,10 +16124,10 @@
         <v>0.20899091059683822</v>
       </c>
       <c r="T198">
-        <v>4.9117781797636262E-2</v>
+        <v>-4.9117781797636262E-2</v>
       </c>
       <c r="U198">
-        <v>0.11387396964874785</v>
+        <v>-0.11387396964874785</v>
       </c>
       <c r="V198">
         <v>-0.40274762744831882</v>
@@ -16219,10 +16219,10 @@
         <v>0.20831253511963752</v>
       </c>
       <c r="T199">
-        <v>4.494850690361929E-2</v>
+        <v>-4.494850690361929E-2</v>
       </c>
       <c r="U199">
-        <v>0.14340646424191306</v>
+        <v>-0.14340646424191306</v>
       </c>
       <c r="V199">
         <v>-0.64938937694116738</v>
@@ -16314,10 +16314,10 @@
         <v>0.20450761302709444</v>
       </c>
       <c r="T200">
-        <v>5.0029119615313533E-2</v>
+        <v>-5.0029119615313533E-2</v>
       </c>
       <c r="U200">
-        <v>-3.3124519061611402E-2</v>
+        <v>3.3124519061611402E-2</v>
       </c>
       <c r="V200">
         <v>-1.223699819031987</v>
@@ -16409,10 +16409,10 @@
         <v>0.20371235305348054</v>
       </c>
       <c r="T201">
-        <v>4.7384734362676539E-2</v>
+        <v>-4.7384734362676539E-2</v>
       </c>
       <c r="U201">
-        <v>-1.1620718256710738E-2</v>
+        <v>1.1620718256710738E-2</v>
       </c>
       <c r="V201">
         <v>-0.95436009205129846</v>
@@ -16504,10 +16504,10 @@
         <v>0.2012605914380162</v>
       </c>
       <c r="T202">
-        <v>5.6529720882525503E-2</v>
+        <v>-5.6529720882525503E-2</v>
       </c>
       <c r="U202">
-        <v>0.1588278025432599</v>
+        <v>-0.1588278025432599</v>
       </c>
       <c r="V202">
         <v>-0.4963260149436044</v>
@@ -16599,10 +16599,10 @@
         <v>0.20126053302524019</v>
       </c>
       <c r="T203">
-        <v>4.938744486351343E-2</v>
+        <v>-4.938744486351343E-2</v>
       </c>
       <c r="U203">
-        <v>2.2902084465159511E-2</v>
+        <v>-2.2902084465159511E-2</v>
       </c>
       <c r="V203">
         <v>-0.49840590660670259</v>
@@ -16694,10 +16694,10 @@
         <v>0.20120844929209458</v>
       </c>
       <c r="T204">
-        <v>6.1189226285618403E-2</v>
+        <v>-6.1189226285618403E-2</v>
       </c>
       <c r="U204">
-        <v>0.14302839450754945</v>
+        <v>-0.14302839450754945</v>
       </c>
       <c r="V204">
         <v>-0.43478971541073275</v>
@@ -16789,10 +16789,10 @@
         <v>0.20100696754337799</v>
       </c>
       <c r="T205">
-        <v>-2.5702139856309536E-2</v>
+        <v>2.5702139856309536E-2</v>
       </c>
       <c r="U205">
-        <v>5.519955542232502E-3</v>
+        <v>-5.519955542232502E-3</v>
       </c>
       <c r="V205">
         <v>-0.56448734206455686</v>
@@ -16884,10 +16884,10 @@
         <v>0.20096703112390982</v>
       </c>
       <c r="T206">
-        <v>5.4510669968266257E-2</v>
+        <v>-5.4510669968266257E-2</v>
       </c>
       <c r="U206">
-        <v>-7.4930142691131962E-2</v>
+        <v>7.4930142691131962E-2</v>
       </c>
       <c r="V206">
         <v>-0.6217892997822716</v>
@@ -16979,10 +16979,10 @@
         <v>0.19867140266119024</v>
       </c>
       <c r="T207">
-        <v>5.361498786022878E-2</v>
+        <v>-5.361498786022878E-2</v>
       </c>
       <c r="U207">
-        <v>-9.6987480480259514E-2</v>
+        <v>9.6987480480259514E-2</v>
       </c>
       <c r="V207">
         <v>-1.0591600872294382</v>
@@ -17074,10 +17074,10 @@
         <v>0.19418409145472776</v>
       </c>
       <c r="T208">
-        <v>4.7804793381844846E-2</v>
+        <v>-4.7804793381844846E-2</v>
       </c>
       <c r="U208">
-        <v>9.2379988769764054E-4</v>
+        <v>-9.2379988769764054E-4</v>
       </c>
       <c r="V208">
         <v>-0.43965255677944626</v>
@@ -17169,10 +17169,10 @@
         <v>0.19451901680769801</v>
       </c>
       <c r="T209">
-        <v>-0.10147232322377242</v>
+        <v>0.10147232322377242</v>
       </c>
       <c r="U209">
-        <v>-2.3644778555387269E-2</v>
+        <v>2.3644778555387269E-2</v>
       </c>
       <c r="V209">
         <v>-0.27612920293194065</v>
@@ -17264,10 +17264,10 @@
         <v>0.19413502201932009</v>
       </c>
       <c r="T210">
-        <v>3.0972015506436357E-2</v>
+        <v>-3.0972015506436357E-2</v>
       </c>
       <c r="U210">
-        <v>-0.13605432181853505</v>
+        <v>0.13605432181853505</v>
       </c>
       <c r="V210">
         <v>-0.19060886135984223</v>
@@ -17359,10 +17359,10 @@
         <v>0.19367461021635698</v>
       </c>
       <c r="T211">
-        <v>5.561073885795853E-2</v>
+        <v>-5.561073885795853E-2</v>
       </c>
       <c r="U211">
-        <v>7.275836396258839E-2</v>
+        <v>-7.275836396258839E-2</v>
       </c>
       <c r="V211">
         <v>-0.41962043419230266</v>
@@ -17454,10 +17454,10 @@
         <v>0.19318056303065473</v>
       </c>
       <c r="T212">
-        <v>5.9045509171973265E-2</v>
+        <v>-5.9045509171973265E-2</v>
       </c>
       <c r="U212">
-        <v>8.2724768500619383E-2</v>
+        <v>-8.2724768500619383E-2</v>
       </c>
       <c r="V212">
         <v>-0.22238570691441861</v>
@@ -17549,10 +17549,10 @@
         <v>0.19295654755227906</v>
       </c>
       <c r="T213">
-        <v>5.5358996639154334E-2</v>
+        <v>-5.5358996639154334E-2</v>
       </c>
       <c r="U213">
-        <v>-2.5707785814232942E-2</v>
+        <v>2.5707785814232942E-2</v>
       </c>
       <c r="V213">
         <v>-8.5772316405652305E-2</v>
@@ -17644,10 +17644,10 @@
         <v>0.19246241905804506</v>
       </c>
       <c r="T214">
-        <v>8.4560091760410572E-2</v>
+        <v>-8.4560091760410572E-2</v>
       </c>
       <c r="U214">
-        <v>3.004725433106703E-2</v>
+        <v>-3.004725433106703E-2</v>
       </c>
       <c r="V214">
         <v>-0.30215065522909423</v>
@@ -17739,10 +17739,10 @@
         <v>0.19201434442268508</v>
       </c>
       <c r="T215">
-        <v>6.6802209893723763E-2</v>
+        <v>-6.6802209893723763E-2</v>
       </c>
       <c r="U215">
-        <v>0.10937035400873096</v>
+        <v>-0.10937035400873096</v>
       </c>
       <c r="V215">
         <v>-0.10375853527395673</v>
@@ -17834,10 +17834,10 @@
         <v>0.19131434623776111</v>
       </c>
       <c r="T216">
-        <v>6.5349158806426999E-2</v>
+        <v>-6.5349158806426999E-2</v>
       </c>
       <c r="U216">
-        <v>-7.461062039895161E-2</v>
+        <v>7.461062039895161E-2</v>
       </c>
       <c r="V216">
         <v>-0.34545190743404675</v>
@@ -17929,10 +17929,10 @@
         <v>0.1908025080953038</v>
       </c>
       <c r="T217">
-        <v>6.7344628493004599E-2</v>
+        <v>-6.7344628493004599E-2</v>
       </c>
       <c r="U217">
-        <v>-0.15925602501936087</v>
+        <v>0.15925602501936087</v>
       </c>
       <c r="V217">
         <v>-0.14890263851596863</v>
@@ -18024,10 +18024,10 @@
         <v>0.18992109730143822</v>
       </c>
       <c r="T218">
-        <v>7.721419169302024E-2</v>
+        <v>-7.721419169302024E-2</v>
       </c>
       <c r="U218">
-        <v>-9.6684854492212757E-2</v>
+        <v>9.6684854492212757E-2</v>
       </c>
       <c r="V218">
         <v>-0.41532468846161574</v>
@@ -18119,10 +18119,10 @@
         <v>0.18902533238095859</v>
       </c>
       <c r="T219">
-        <v>7.050800212204944E-2</v>
+        <v>-7.050800212204944E-2</v>
       </c>
       <c r="U219">
-        <v>3.3092348483343415E-2</v>
+        <v>-3.3092348483343415E-2</v>
       </c>
       <c r="V219">
         <v>-0.68432088652048417</v>
@@ -18214,10 +18214,10 @@
         <v>0.18902034159433223</v>
       </c>
       <c r="T220">
-        <v>6.8862372256961457E-2</v>
+        <v>-6.8862372256961457E-2</v>
       </c>
       <c r="U220">
-        <v>0.11684921753865041</v>
+        <v>-0.11684921753865041</v>
       </c>
       <c r="V220">
         <v>-0.70202782064887614</v>
@@ -18309,10 +18309,10 @@
         <v>0.18878632846363513</v>
       </c>
       <c r="T221">
-        <v>6.8033159873270854E-2</v>
+        <v>-6.8033159873270854E-2</v>
       </c>
       <c r="U221">
-        <v>0.23377974807099466</v>
+        <v>-0.23377974807099466</v>
       </c>
       <c r="V221">
         <v>-0.83315450583862916</v>
@@ -18404,10 +18404,10 @@
         <v>0.18011794798157094</v>
       </c>
       <c r="T222">
-        <v>7.0770582837620388E-2</v>
+        <v>-7.0770582837620388E-2</v>
       </c>
       <c r="U222">
-        <v>0.27134051902577561</v>
+        <v>-0.27134051902577561</v>
       </c>
       <c r="V222">
         <v>-1.3394022828183694E-3</v>
@@ -18499,10 +18499,10 @@
         <v>0.1801162667539975</v>
       </c>
       <c r="T223">
-        <v>7.2097527602177358E-2</v>
+        <v>-7.2097527602177358E-2</v>
       </c>
       <c r="U223">
-        <v>0.20208110149837477</v>
+        <v>-0.20208110149837477</v>
       </c>
       <c r="V223">
         <v>-1.5275545569681803E-2</v>
@@ -18594,10 +18594,10 @@
         <v>0.1798281192724869</v>
       </c>
       <c r="T224">
-        <v>6.4178052555652343E-2</v>
+        <v>-6.4178052555652343E-2</v>
       </c>
       <c r="U224">
-        <v>0.2724386951301172</v>
+        <v>-0.2724386951301172</v>
       </c>
       <c r="V224">
         <v>-0.16556472426152435</v>
@@ -18689,10 +18689,10 @@
         <v>0.1779135211733596</v>
       </c>
       <c r="T225">
-        <v>6.4581256509033125E-2</v>
+        <v>-6.4581256509033125E-2</v>
       </c>
       <c r="U225">
-        <v>0.22127695373403977</v>
+        <v>-0.22127695373403977</v>
       </c>
       <c r="V225">
         <v>-0.54774254176763737</v>
@@ -18784,10 +18784,10 @@
         <v>0.17264069340213634</v>
       </c>
       <c r="T226">
-        <v>6.3569475362812433E-2</v>
+        <v>-6.3569475362812433E-2</v>
       </c>
       <c r="U226">
-        <v>0.34027005733077154</v>
+        <v>-0.34027005733077154</v>
       </c>
       <c r="V226">
         <v>8.2276486460464149E-2</v>
@@ -18879,10 +18879,10 @@
         <v>0.17221825139009439</v>
       </c>
       <c r="T227">
-        <v>6.6799068782730231E-2</v>
+        <v>-6.6799068782730231E-2</v>
       </c>
       <c r="U227">
-        <v>4.385713448100681E-2</v>
+        <v>-4.385713448100681E-2</v>
       </c>
       <c r="V227">
         <v>-9.8354099910546999E-2</v>
@@ -18974,10 +18974,10 @@
         <v>0.17171388431926501</v>
       </c>
       <c r="T228">
-        <v>7.3552089471284887E-2</v>
+        <v>-7.3552089471284887E-2</v>
       </c>
       <c r="U228">
-        <v>0.12368594959619728</v>
+        <v>-0.12368594959619728</v>
       </c>
       <c r="V228">
         <v>-0.29521336331821413</v>
@@ -19069,10 +19069,10 @@
         <v>0.17128988099084894</v>
       </c>
       <c r="T229">
-        <v>9.6349041542831415E-2</v>
+        <v>-9.6349041542831415E-2</v>
       </c>
       <c r="U229">
-        <v>0.1422531140128136</v>
+        <v>-0.1422531140128136</v>
       </c>
       <c r="V229">
         <v>-0.14358858325838053</v>
@@ -19164,10 +19164,10 @@
         <v>0.17072720539142999</v>
       </c>
       <c r="T230">
-        <v>9.2781058537472205E-2</v>
+        <v>-9.2781058537472205E-2</v>
       </c>
       <c r="U230">
-        <v>0.14357637397179879</v>
+        <v>-0.14357637397179879</v>
       </c>
       <c r="V230">
         <v>-0.34581185917241797</v>
@@ -19259,10 +19259,10 @@
         <v>0.1633335162948826</v>
       </c>
       <c r="T231">
-        <v>9.3773070847436024E-2</v>
+        <v>-9.3773070847436024E-2</v>
       </c>
       <c r="U231">
-        <v>0.14170511402107344</v>
+        <v>-0.14170511402107344</v>
       </c>
       <c r="V231">
         <v>-1.0556481047270472</v>
@@ -19354,10 +19354,10 @@
         <v>0.14974919334195222</v>
       </c>
       <c r="T232">
-        <v>8.9034347292460403E-2</v>
+        <v>-8.9034347292460403E-2</v>
       </c>
       <c r="U232">
-        <v>0.14598585162042266</v>
+        <v>-0.14598585162042266</v>
       </c>
       <c r="V232">
         <v>-0.11304890558900826</v>
@@ -19449,10 +19449,10 @@
         <v>0.14975190221267753</v>
       </c>
       <c r="T233">
-        <v>7.4522410677602124E-2</v>
+        <v>-7.4522410677602124E-2</v>
       </c>
       <c r="U233">
-        <v>0.12399679394246022</v>
+        <v>-0.12399679394246022</v>
       </c>
       <c r="V233">
         <v>-0.10418214232710277</v>
@@ -19544,10 +19544,10 @@
         <v>0.14954901044867067</v>
       </c>
       <c r="T234">
-        <v>8.0040457257890552E-2</v>
+        <v>-8.0040457257890552E-2</v>
       </c>
       <c r="U234">
-        <v>0.1411676190746558</v>
+        <v>-0.1411676190746558</v>
       </c>
       <c r="V234">
         <v>-0.22775918202648793</v>
@@ -19639,10 +19639,10 @@
         <v>0.14921260636822206</v>
       </c>
       <c r="T235">
-        <v>7.9747980423838793E-2</v>
+        <v>-7.9747980423838793E-2</v>
       </c>
       <c r="U235">
-        <v>5.4603232961103476E-2</v>
+        <v>-5.4603232961103476E-2</v>
       </c>
       <c r="V235">
         <v>-8.4223807282701735E-2</v>
@@ -19734,10 +19734,10 @@
         <v>0.14899351585146897</v>
       </c>
       <c r="T236">
-        <v>8.189081257700126E-2</v>
+        <v>-8.189081257700126E-2</v>
       </c>
       <c r="U236">
-        <v>0.13629149096273663</v>
+        <v>-0.13629149096273663</v>
       </c>
       <c r="V236">
         <v>-0.20291198803457089</v>
@@ -19829,10 +19829,10 @@
         <v>0.14896481119152793</v>
       </c>
       <c r="T237">
-        <v>7.859493072936985E-2</v>
+        <v>-7.859493072936985E-2</v>
       </c>
       <c r="U237">
-        <v>0.13200624693293639</v>
+        <v>-0.13200624693293639</v>
       </c>
       <c r="V237">
         <v>-0.24350262379151388</v>
@@ -19924,10 +19924,10 @@
         <v>0.14896472514335693</v>
       </c>
       <c r="T238">
-        <v>7.8460019940285175E-2</v>
+        <v>-7.8460019940285175E-2</v>
       </c>
       <c r="U238">
-        <v>0.125995812297508</v>
+        <v>-0.125995812297508</v>
       </c>
       <c r="V238">
         <v>-0.24347645006408403</v>
@@ -20019,10 +20019,10 @@
         <v>0.16684020170631186</v>
       </c>
       <c r="T239">
-        <v>1.2255601757383161</v>
+        <v>-1.2255601757383161</v>
       </c>
       <c r="U239">
-        <v>1.1337998682038442</v>
+        <v>-1.1337998682038442</v>
       </c>
       <c r="V239">
         <v>-1.4277789051623246</v>
@@ -20114,10 +20114,10 @@
         <v>0.18308400193708302</v>
       </c>
       <c r="T240">
-        <v>0.10170792730889167</v>
+        <v>-0.10170792730889167</v>
       </c>
       <c r="U240">
-        <v>0.13310649280395825</v>
+        <v>-0.13310649280395825</v>
       </c>
       <c r="V240">
         <v>-0.52424016127528006</v>
@@ -20209,10 +20209,10 @@
         <v>0.18276530482685716</v>
       </c>
       <c r="T241">
-        <v>6.5728280103105607E-2</v>
+        <v>-6.5728280103105607E-2</v>
       </c>
       <c r="U241">
-        <v>0.12082108544552161</v>
+        <v>-0.12082108544552161</v>
       </c>
       <c r="V241">
         <v>-0.35979269075534503</v>
@@ -20304,10 +20304,10 @@
         <v>0.18229964292875214</v>
       </c>
       <c r="T242">
-        <v>6.1064363117646625E-2</v>
+        <v>-6.1064363117646625E-2</v>
       </c>
       <c r="U242">
-        <v>0.11959391883242798</v>
+        <v>-0.11959391883242798</v>
       </c>
       <c r="V242">
         <v>-0.17556754484098214</v>
@@ -20399,10 +20399,10 @@
         <v>0.18190018242363623</v>
       </c>
       <c r="T243">
-        <v>5.937181930940616E-2</v>
+        <v>-5.937181930940616E-2</v>
       </c>
       <c r="U243">
-        <v>0.11411998256123379</v>
+        <v>-0.11411998256123379</v>
       </c>
       <c r="V243">
         <v>-0.34138868275597201</v>
@@ -20494,10 +20494,10 @@
         <v>0.18186190388909204</v>
       </c>
       <c r="T244">
-        <v>4.683853804314797E-2</v>
+        <v>-4.683853804314797E-2</v>
       </c>
       <c r="U244">
-        <v>0.12996649920476999</v>
+        <v>-0.12996649920476999</v>
       </c>
       <c r="V244">
         <v>-0.39079068147680474</v>
@@ -20589,10 +20589,10 @@
         <v>0.18185449399141951</v>
       </c>
       <c r="T245">
-        <v>5.0243518943182686E-2</v>
+        <v>-5.0243518943182686E-2</v>
       </c>
       <c r="U245">
-        <v>0.11605802314017533</v>
+        <v>-0.11605802314017533</v>
       </c>
       <c r="V245">
         <v>-0.36468228947823533</v>
@@ -20684,10 +20684,10 @@
         <v>0.1815084007218781</v>
       </c>
       <c r="T246">
-        <v>5.0257463937475322E-2</v>
+        <v>-5.0257463937475322E-2</v>
       </c>
       <c r="U246">
-        <v>0.11457961402907557</v>
+        <v>-0.11457961402907557</v>
       </c>
       <c r="V246">
         <v>-0.20642353307152028</v>
@@ -20779,10 +20779,10 @@
         <v>0.18142983702298929</v>
       </c>
       <c r="T247">
-        <v>3.9474322605581591E-2</v>
+        <v>-3.9474322605581591E-2</v>
       </c>
       <c r="U247">
-        <v>0.10549781070171571</v>
+        <v>-0.10549781070171571</v>
       </c>
       <c r="V247">
         <v>-0.27846720249922186</v>
@@ -20874,10 +20874,10 @@
         <v>0.18089157018849539</v>
       </c>
       <c r="T248">
-        <v>3.4159909212549966E-2</v>
+        <v>-3.4159909212549966E-2</v>
       </c>
       <c r="U248">
-        <v>0.10927567845937514</v>
+        <v>-0.10927567845937514</v>
       </c>
       <c r="V248">
         <v>-7.5080874694744004E-2</v>
@@ -20969,10 +20969,10 @@
         <v>0.1808838547616328</v>
       </c>
       <c r="T249">
-        <v>3.5419971386996263E-2</v>
+        <v>-3.5419971386996263E-2</v>
       </c>
       <c r="U249">
-        <v>0.10390143864643653</v>
+        <v>-0.10390143864643653</v>
       </c>
       <c r="V249">
         <v>-0.10050220262676213</v>
@@ -21064,10 +21064,10 @@
         <v>0.18021281537136738</v>
       </c>
       <c r="T250">
-        <v>3.7762090806725546E-2</v>
+        <v>-3.7762090806725546E-2</v>
       </c>
       <c r="U250">
-        <v>0.1045803974027204</v>
+        <v>-0.1045803974027204</v>
       </c>
       <c r="V250">
         <v>-0.31710012184491543</v>
@@ -21159,10 +21159,10 @@
         <v>0.18013802541873219</v>
       </c>
       <c r="T251">
-        <v>2.4966249205848889E-2</v>
+        <v>-2.4966249205848889E-2</v>
       </c>
       <c r="U251">
-        <v>9.0720441979874611E-2</v>
+        <v>-9.0720441979874611E-2</v>
       </c>
       <c r="V251">
         <v>-0.22522148369643613</v>
@@ -21254,10 +21254,10 @@
         <v>0.17983285075735317</v>
       </c>
       <c r="T252">
-        <v>3.3618885345199079E-2</v>
+        <v>-3.3618885345199079E-2</v>
       </c>
       <c r="U252">
-        <v>0.10226628325666898</v>
+        <v>-0.10226628325666898</v>
       </c>
       <c r="V252">
         <v>-8.9899651081659648E-2</v>
@@ -21349,10 +21349,10 @@
         <v>0.17981475370855848</v>
       </c>
       <c r="T253">
-        <v>3.417693342204764E-2</v>
+        <v>-3.417693342204764E-2</v>
       </c>
       <c r="U253">
-        <v>0.10394836108666983</v>
+        <v>-0.10394836108666983</v>
       </c>
       <c r="V253">
         <v>-0.1269987291214747</v>
@@ -21444,10 +21444,10 @@
         <v>0.17922476877894061</v>
       </c>
       <c r="T254">
-        <v>3.562361795004243E-2</v>
+        <v>-3.562361795004243E-2</v>
       </c>
       <c r="U254">
-        <v>9.7985175491310805E-2</v>
+        <v>-9.7985175491310805E-2</v>
       </c>
       <c r="V254">
         <v>7.2090210302833135E-2</v>
@@ -21539,10 +21539,10 @@
         <v>0.17918923681305937</v>
       </c>
       <c r="T255">
-        <v>4.0343590717484279E-2</v>
+        <v>-4.0343590717484279E-2</v>
       </c>
       <c r="U255">
-        <v>0.10350126101833501</v>
+        <v>-0.10350126101833501</v>
       </c>
       <c r="V255">
         <v>0.11630804128250904</v>
@@ -21634,10 +21634,10 @@
         <v>0.1791875352811047</v>
       </c>
       <c r="T256">
-        <v>4.2303134366061812E-2</v>
+        <v>-4.2303134366061812E-2</v>
       </c>
       <c r="U256">
-        <v>0.10477417342986683</v>
+        <v>-0.10477417342986683</v>
       </c>
       <c r="V256">
         <v>0.10125879385234349</v>
@@ -21729,10 +21729,10 @@
         <v>0.17915514035746388</v>
       </c>
       <c r="T257">
-        <v>5.7164805181464384E-2</v>
+        <v>-5.7164805181464384E-2</v>
       </c>
       <c r="U257">
-        <v>0.12341552396178956</v>
+        <v>-0.12341552396178956</v>
       </c>
       <c r="V257">
         <v>0.13444243987574822</v>
@@ -21824,10 +21824,10 @@
         <v>0.17794813860586808</v>
       </c>
       <c r="T258">
-        <v>4.4300692889576165E-2</v>
+        <v>-4.4300692889576165E-2</v>
       </c>
       <c r="U258">
-        <v>0.11676528047442902</v>
+        <v>-0.11676528047442902</v>
       </c>
       <c r="V258">
         <v>-0.14902030401959809</v>
@@ -21919,10 +21919,10 @@
         <v>0.17744225086632956</v>
       </c>
       <c r="T259">
-        <v>1.1024710307405705E-2</v>
+        <v>-1.1024710307405705E-2</v>
       </c>
       <c r="U259">
-        <v>0.10540450058867945</v>
+        <v>-0.10540450058867945</v>
       </c>
       <c r="V259">
         <v>-0.32685775048189036</v>
@@ -22014,10 +22014,10 @@
         <v>0.17708166808633885</v>
       </c>
       <c r="T260">
-        <v>1.8596434448903132E-2</v>
+        <v>-1.8596434448903132E-2</v>
       </c>
       <c r="U260">
-        <v>0.10986053949241237</v>
+        <v>-0.10986053949241237</v>
       </c>
       <c r="V260">
         <v>-0.1753733254257428</v>
@@ -22109,10 +22109,10 @@
         <v>0.17636538624158302</v>
       </c>
       <c r="T261">
-        <v>1.509921635439726E-2</v>
+        <v>-1.509921635439726E-2</v>
       </c>
       <c r="U261">
-        <v>0.10792050912618034</v>
+        <v>-0.10792050912618034</v>
       </c>
       <c r="V261">
         <v>-0.39462707363324689</v>
@@ -22204,10 +22204,10 @@
         <v>0.17587032064410221</v>
       </c>
       <c r="T262">
-        <v>2.7347435534752496E-2</v>
+        <v>-2.7347435534752496E-2</v>
       </c>
       <c r="U262">
-        <v>0.11604420212917299</v>
+        <v>-0.11604420212917299</v>
       </c>
       <c r="V262">
         <v>-0.22171680071436661</v>
@@ -22299,10 +22299,10 @@
         <v>0.17590649671194902</v>
       </c>
       <c r="T263">
-        <v>0.11178034473057208</v>
+        <v>-0.11178034473057208</v>
       </c>
       <c r="U263">
-        <v>0.18586050684452626</v>
+        <v>-0.18586050684452626</v>
       </c>
       <c r="V263">
         <v>-0.24144268347494613</v>
@@ -22394,10 +22394,10 @@
         <v>0.17346388053131859</v>
       </c>
       <c r="T264">
-        <v>2.7159730118664349E-2</v>
+        <v>-2.7159730118664349E-2</v>
       </c>
       <c r="U264">
-        <v>0.1068687653973277</v>
+        <v>-0.1068687653973277</v>
       </c>
       <c r="V264">
         <v>-0.57750380756684816</v>
@@ -22489,10 +22489,10 @@
         <v>0.17319476184318694</v>
       </c>
       <c r="T265">
-        <v>3.2722778021576637E-2</v>
+        <v>-3.2722778021576637E-2</v>
       </c>
       <c r="U265">
-        <v>0.11200748048132425</v>
+        <v>-0.11200748048132425</v>
       </c>
       <c r="V265">
         <v>-0.44534528440349774</v>
@@ -22584,10 +22584,10 @@
         <v>0.17308490934284051</v>
       </c>
       <c r="T266">
-        <v>3.0139061869582928E-2</v>
+        <v>-3.0139061869582928E-2</v>
       </c>
       <c r="U266">
-        <v>0.11145634016795913</v>
+        <v>-0.11145634016795913</v>
       </c>
       <c r="V266">
         <v>-0.52855770287671966</v>
@@ -22679,10 +22679,10 @@
         <v>0.17308134976541611</v>
       </c>
       <c r="T267">
-        <v>3.3908007457672529E-2</v>
+        <v>-3.3908007457672529E-2</v>
       </c>
       <c r="U267">
-        <v>0.11183051248093712</v>
+        <v>-0.11183051248093712</v>
       </c>
       <c r="V267">
         <v>-0.51225274933195397</v>
@@ -22774,10 +22774,10 @@
         <v>0.17299290580511478</v>
       </c>
       <c r="T268">
-        <v>3.0592957681763178E-2</v>
+        <v>-3.0592957681763178E-2</v>
       </c>
       <c r="U268">
-        <v>0.10823830450971128</v>
+        <v>-0.10823830450971128</v>
       </c>
       <c r="V268">
         <v>-0.42426212181430056</v>
@@ -22869,10 +22869,10 @@
         <v>0.17291548559415024</v>
       </c>
       <c r="T269">
-        <v>-0.99075017678539323</v>
+        <v>0.99075017678539323</v>
       </c>
       <c r="U269">
-        <v>0.25441473740013265</v>
+        <v>-0.25441473740013265</v>
       </c>
       <c r="V269">
         <v>-0.34830403883703287</v>
@@ -22964,10 +22964,10 @@
         <v>0.17290536455498953</v>
       </c>
       <c r="T270">
-        <v>2.2348146573225591E-2</v>
+        <v>-2.2348146573225591E-2</v>
       </c>
       <c r="U270">
-        <v>0.12321945604614193</v>
+        <v>-0.12321945604614193</v>
       </c>
       <c r="V270">
         <v>-0.31814156217400136</v>
@@ -23059,10 +23059,10 @@
         <v>0.17231787333479034</v>
       </c>
       <c r="T271">
-        <v>3.3939640648716907E-2</v>
+        <v>-3.3939640648716907E-2</v>
       </c>
       <c r="U271">
-        <v>9.8878132093072058E-2</v>
+        <v>-9.8878132093072058E-2</v>
       </c>
       <c r="V271">
         <v>-0.51608645443730339</v>
@@ -23154,10 +23154,10 @@
         <v>0.16978681234915324</v>
       </c>
       <c r="T272">
-        <v>3.3197643393800824E-2</v>
+        <v>-3.3197643393800824E-2</v>
       </c>
       <c r="U272">
-        <v>9.3478540227154294E-2</v>
+        <v>-9.3478540227154294E-2</v>
       </c>
       <c r="V272">
         <v>-0.11003173169872316</v>
@@ -23249,10 +23249,10 @@
         <v>0.16962762478637108</v>
       </c>
       <c r="T273">
-        <v>3.2667261127250491E-2</v>
+        <v>-3.2667261127250491E-2</v>
       </c>
       <c r="U273">
-        <v>9.1367659777008559E-2</v>
+        <v>-9.1367659777008559E-2</v>
       </c>
       <c r="V273">
         <v>-6.6781877730459627E-3</v>
@@ -23344,10 +23344,10 @@
         <v>0.16944077286904433</v>
       </c>
       <c r="T274">
-        <v>3.7657464375451255E-2</v>
+        <v>-3.7657464375451255E-2</v>
       </c>
       <c r="U274">
-        <v>8.369893902038239E-2</v>
+        <v>-8.369893902038239E-2</v>
       </c>
       <c r="V274">
         <v>9.9038839926945954E-2</v>
@@ -23439,10 +23439,10 @@
         <v>0.16936011929487055</v>
       </c>
       <c r="T275">
-        <v>4.1551977473375246E-2</v>
+        <v>-4.1551977473375246E-2</v>
       </c>
       <c r="U275">
-        <v>9.0904320785745174E-2</v>
+        <v>-9.0904320785745174E-2</v>
       </c>
       <c r="V275">
         <v>0.16717614756047716</v>
@@ -23534,10 +23534,10 @@
         <v>0.16889767394900748</v>
       </c>
       <c r="T276">
-        <v>4.1676514216049121E-2</v>
+        <v>-4.1676514216049121E-2</v>
       </c>
       <c r="U276">
-        <v>9.1037694334872299E-2</v>
+        <v>-9.1037694334872299E-2</v>
       </c>
       <c r="V276">
         <v>0.33836693503941362</v>
@@ -23629,10 +23629,10 @@
         <v>0.16889601129328527</v>
       </c>
       <c r="T277">
-        <v>4.4779065717448496E-2</v>
+        <v>-4.4779065717448496E-2</v>
       </c>
       <c r="U277">
-        <v>8.3251541017603792E-2</v>
+        <v>-8.3251541017603792E-2</v>
       </c>
       <c r="V277">
         <v>0.34583025544836499</v>
@@ -23724,10 +23724,10 @@
         <v>0.16485261398574036</v>
       </c>
       <c r="T278">
-        <v>5.2926437538447502E-2</v>
+        <v>-5.2926437538447502E-2</v>
       </c>
       <c r="U278">
-        <v>8.5749234213161607E-2</v>
+        <v>-8.5749234213161607E-2</v>
       </c>
       <c r="V278">
         <v>-0.16307894314460114</v>
@@ -23819,10 +23819,10 @@
         <v>0.16484415789871876</v>
       </c>
       <c r="T279">
-        <v>5.0317072350192227E-2</v>
+        <v>-5.0317072350192227E-2</v>
       </c>
       <c r="U279">
-        <v>8.4455844680508818E-2</v>
+        <v>-8.4455844680508818E-2</v>
       </c>
       <c r="V279">
         <v>-0.18560165924443872</v>
@@ -23914,10 +23914,10 @@
         <v>0.16458494882326127</v>
       </c>
       <c r="T280">
-        <v>4.5855311032383383E-2</v>
+        <v>-4.5855311032383383E-2</v>
       </c>
       <c r="U280">
-        <v>8.242317551112599E-2</v>
+        <v>-8.242317551112599E-2</v>
       </c>
       <c r="V280">
         <v>-5.5474699020896523E-2</v>
@@ -24009,10 +24009,10 @@
         <v>0.1645740910935376</v>
       </c>
       <c r="T281">
-        <v>5.8465326058421141E-2</v>
+        <v>-5.8465326058421141E-2</v>
       </c>
       <c r="U281">
-        <v>8.1531395526890371E-2</v>
+        <v>-8.1531395526890371E-2</v>
       </c>
       <c r="V281">
         <v>-7.8066717568603394E-2</v>
@@ -24104,10 +24104,10 @@
         <v>0.16457407414327896</v>
       </c>
       <c r="T282">
-        <v>4.6788308923195743E-2</v>
+        <v>-4.6788308923195743E-2</v>
       </c>
       <c r="U282">
-        <v>7.9077833293927924E-2</v>
+        <v>-7.9077833293927924E-2</v>
       </c>
       <c r="V282">
         <v>-7.8297381934389065E-2</v>
@@ -24199,10 +24199,10 @@
         <v>0.16449757638943205</v>
       </c>
       <c r="T283">
-        <v>4.8384845633675511E-2</v>
+        <v>-4.8384845633675511E-2</v>
       </c>
       <c r="U283">
-        <v>8.1227847346709847E-2</v>
+        <v>-8.1227847346709847E-2</v>
       </c>
       <c r="V283">
         <v>-0.15122527907274197</v>
@@ -24294,10 +24294,10 @@
         <v>0.16073251696284144</v>
       </c>
       <c r="T284">
-        <v>5.0943500521372087E-2</v>
+        <v>-5.0943500521372087E-2</v>
       </c>
       <c r="U284">
-        <v>8.5217685646599151E-2</v>
+        <v>-8.5217685646599151E-2</v>
       </c>
       <c r="V284">
         <v>-0.63477500298945166</v>
@@ -24389,10 +24389,10 @@
         <v>0.15957905598622973</v>
       </c>
       <c r="T285">
-        <v>4.5343426454547142E-2</v>
+        <v>-4.5343426454547142E-2</v>
       </c>
       <c r="U285">
-        <v>8.4651172052174761E-2</v>
+        <v>-8.4651172052174761E-2</v>
       </c>
       <c r="V285">
         <v>-0.36757018712370026</v>
@@ -24484,10 +24484,10 @@
         <v>0.15949845371859575</v>
       </c>
       <c r="T286">
-        <v>4.2470061056176789E-2</v>
+        <v>-4.2470061056176789E-2</v>
       </c>
       <c r="U286">
-        <v>8.3865322890053218E-2</v>
+        <v>-8.3865322890053218E-2</v>
       </c>
       <c r="V286">
         <v>-0.43473709511303582</v>
@@ -24579,10 +24579,10 @@
         <v>0.15947094032617376</v>
       </c>
       <c r="T287">
-        <v>2.2618884402003658E-2</v>
+        <v>-2.2618884402003658E-2</v>
       </c>
       <c r="U287">
-        <v>7.9406764557843346E-2</v>
+        <v>-7.9406764557843346E-2</v>
       </c>
       <c r="V287">
         <v>-0.38969253404592674</v>
@@ -24674,10 +24674,10 @@
         <v>0.15696183821982507</v>
       </c>
       <c r="T288">
-        <v>3.3743831674759583E-2</v>
+        <v>-3.3743831674759583E-2</v>
       </c>
       <c r="U288">
-        <v>7.7572236267742234E-2</v>
+        <v>-7.7572236267742234E-2</v>
       </c>
       <c r="V288">
         <v>-0.77322944807847183</v>
@@ -24769,10 +24769,10 @@
         <v>0.15640372182401308</v>
       </c>
       <c r="T289">
-        <v>4.1334948651172709E-2</v>
+        <v>-4.1334948651172709E-2</v>
       </c>
       <c r="U289">
-        <v>5.1577306302019732E-2</v>
+        <v>-5.1577306302019732E-2</v>
       </c>
       <c r="V289">
         <v>-0.58729423700605299</v>
@@ -24864,10 +24864,10 @@
         <v>0.15271245381138462</v>
       </c>
       <c r="T290">
-        <v>3.3215369976535847E-2</v>
+        <v>-3.3215369976535847E-2</v>
       </c>
       <c r="U290">
-        <v>5.1380735464656713E-2</v>
+        <v>-5.1380735464656713E-2</v>
       </c>
       <c r="V290">
         <v>-0.12208908480926262</v>
@@ -24959,10 +24959,10 @@
         <v>0.15157787763906991</v>
       </c>
       <c r="T291">
-        <v>3.1507270821884426E-2</v>
+        <v>-3.1507270821884426E-2</v>
       </c>
       <c r="U291">
-        <v>4.6377232865546514E-2</v>
+        <v>-4.6377232865546514E-2</v>
       </c>
       <c r="V291">
         <v>-0.3708986819063842</v>
@@ -25054,10 +25054,10 @@
         <v>0.15034628151220789</v>
       </c>
       <c r="T292">
-        <v>2.4060242757983907E-2</v>
+        <v>-2.4060242757983907E-2</v>
       </c>
       <c r="U292">
-        <v>5.1481637590589102E-2</v>
+        <v>-5.1481637590589102E-2</v>
       </c>
       <c r="V292">
         <v>-0.64043803428375234</v>
@@ -25149,10 +25149,10 @@
         <v>0.14808197946039273</v>
       </c>
       <c r="T293">
-        <v>-4.293773708394788E-2</v>
+        <v>4.293773708394788E-2</v>
       </c>
       <c r="U293">
-        <v>6.9919176936839023E-2</v>
+        <v>-6.9919176936839023E-2</v>
       </c>
       <c r="V293">
         <v>-0.28635926110653909</v>
@@ -25244,10 +25244,10 @@
         <v>0.14353927005616507</v>
       </c>
       <c r="T294">
-        <v>3.3965302640615036E-2</v>
+        <v>-3.3965302640615036E-2</v>
       </c>
       <c r="U294">
-        <v>6.1393110580865162E-2</v>
+        <v>-6.1393110580865162E-2</v>
       </c>
       <c r="V294">
         <v>0.21671797149214189</v>
@@ -25339,10 +25339,10 @@
         <v>0.14110880548407775</v>
       </c>
       <c r="T295">
-        <v>1.9488113993926248E-2</v>
+        <v>-1.9488113993926248E-2</v>
       </c>
       <c r="U295">
-        <v>5.2481485001076855E-2</v>
+        <v>-5.2481485001076855E-2</v>
       </c>
       <c r="V295">
         <v>0.58732157795973183</v>
@@ -25434,10 +25434,10 @@
         <v>0.12747646841595753</v>
       </c>
       <c r="T296">
-        <v>2.1358086665523857E-2</v>
+        <v>-2.1358086665523857E-2</v>
       </c>
       <c r="U296">
-        <v>5.1684929495632304E-2</v>
+        <v>-5.1684929495632304E-2</v>
       </c>
       <c r="V296">
         <v>-0.25512529160711672</v>
@@ -25529,10 +25529,10 @@
         <v>0.12744130784843197</v>
       </c>
       <c r="T297">
-        <v>3.0398446138235613E-2</v>
+        <v>-3.0398446138235613E-2</v>
       </c>
       <c r="U297">
-        <v>6.4870086204105171E-2</v>
+        <v>-6.4870086204105171E-2</v>
       </c>
       <c r="V297">
         <v>-0.3127864950185355</v>
@@ -25624,10 +25624,10 @@
         <v>0.12742294637427556</v>
       </c>
       <c r="T298">
-        <v>3.4503772577587632E-2</v>
+        <v>-3.4503772577587632E-2</v>
       </c>
       <c r="U298">
-        <v>6.5620155906520594E-2</v>
+        <v>-6.5620155906520594E-2</v>
       </c>
       <c r="V298">
         <v>-0.27801387242445408</v>
@@ -25719,10 +25719,10 @@
         <v>0.12740104690249771</v>
       </c>
       <c r="T299">
-        <v>3.0160901985643029E-2</v>
+        <v>-3.0160901985643029E-2</v>
       </c>
       <c r="U299">
-        <v>-0.98449412391024005</v>
+        <v>0.98449412391024005</v>
       </c>
       <c r="V299">
         <v>-0.23672909968519562</v>
@@ -25814,10 +25814,10 @@
         <v>0.12740090097056819</v>
       </c>
       <c r="T300">
-        <v>3.2228606516016001E-2</v>
+        <v>-3.2228606516016001E-2</v>
       </c>
       <c r="U300">
-        <v>5.5082859633337478E-2</v>
+        <v>-5.5082859633337478E-2</v>
       </c>
       <c r="V300">
         <v>-0.23351072213875224</v>
@@ -25909,10 +25909,10 @@
         <v>0.12716608901256907</v>
       </c>
       <c r="T301">
-        <v>3.0553004058209154E-2</v>
+        <v>-3.0553004058209154E-2</v>
       </c>
       <c r="U301">
-        <v>6.5537664908243976E-2</v>
+        <v>-6.5537664908243976E-2</v>
       </c>
       <c r="V301">
         <v>-0.12826028421493163</v>
@@ -26004,10 +26004,10 @@
         <v>0.12708778348638528</v>
       </c>
       <c r="T302">
-        <v>3.0163378619829651E-2</v>
+        <v>-3.0163378619829651E-2</v>
       </c>
       <c r="U302">
-        <v>6.4447563062075552E-2</v>
+        <v>-6.4447563062075552E-2</v>
       </c>
       <c r="V302">
         <v>-6.540395035408153E-2</v>
@@ -26099,10 +26099,10 @@
         <v>0.12657592726487477</v>
       </c>
       <c r="T303">
-        <v>2.60246885446902E-2</v>
+        <v>-2.60246885446902E-2</v>
       </c>
       <c r="U303">
-        <v>5.9755640267633581E-2</v>
+        <v>-5.9755640267633581E-2</v>
       </c>
       <c r="V303">
         <v>-0.21832228859701708</v>
@@ -26194,10 +26194,10 @@
         <v>0.12627487007093235</v>
       </c>
       <c r="T304">
-        <v>1.9448166588675875E-2</v>
+        <v>-1.9448166588675875E-2</v>
       </c>
       <c r="U304">
-        <v>5.8220618973470195E-2</v>
+        <v>-5.8220618973470195E-2</v>
       </c>
       <c r="V304">
         <v>-0.33589899855432925</v>
@@ -26289,10 +26289,10 @@
         <v>0.12626278269246408</v>
       </c>
       <c r="T305">
-        <v>1.2481851917511833E-2</v>
+        <v>-1.2481851917511833E-2</v>
       </c>
       <c r="U305">
-        <v>5.5193721466872958E-2</v>
+        <v>-5.5193721466872958E-2</v>
       </c>
       <c r="V305">
         <v>-0.3050133991441939</v>
@@ -26384,10 +26384,10 @@
         <v>0.12619500552191396</v>
       </c>
       <c r="T306">
-        <v>1.4009033437289986E-2</v>
+        <v>-1.4009033437289986E-2</v>
       </c>
       <c r="U306">
-        <v>5.6880197140696254E-2</v>
+        <v>-5.6880197140696254E-2</v>
       </c>
       <c r="V306">
         <v>-0.36258896502829874</v>
@@ -26479,10 +26479,10 @@
         <v>0.12463858095765616</v>
       </c>
       <c r="T307">
-        <v>1.41139174577809E-2</v>
+        <v>-1.41139174577809E-2</v>
       </c>
       <c r="U307">
-        <v>6.0222539651966223E-2</v>
+        <v>-6.0222539651966223E-2</v>
       </c>
       <c r="V307">
         <v>-8.8340787964868994E-2</v>
@@ -26574,10 +26574,10 @@
         <v>0.12422240907296114</v>
       </c>
       <c r="T308">
-        <v>1.8625316362186339E-2</v>
+        <v>-1.8625316362186339E-2</v>
       </c>
       <c r="U308">
-        <v>7.3286112952364313E-2</v>
+        <v>-7.3286112952364313E-2</v>
       </c>
       <c r="V308">
         <v>4.8153668337858058E-2</v>
@@ -26669,10 +26669,10 @@
         <v>0.12418976306395837</v>
       </c>
       <c r="T309">
-        <v>1.6300038778660486E-2</v>
+        <v>-1.6300038778660486E-2</v>
       </c>
       <c r="U309">
-        <v>6.8251881277991977E-2</v>
+        <v>-6.8251881277991977E-2</v>
       </c>
       <c r="V309">
         <v>9.0063565873577112E-2</v>
@@ -26764,10 +26764,10 @@
         <v>0.12408721024594847</v>
       </c>
       <c r="T310">
-        <v>1.5547043479613443E-2</v>
+        <v>-1.5547043479613443E-2</v>
       </c>
       <c r="U310">
-        <v>6.2919836205077573E-2</v>
+        <v>-6.2919836205077573E-2</v>
       </c>
       <c r="V310">
         <v>2.1404343661979297E-2</v>
@@ -26859,10 +26859,10 @@
         <v>0.12360686332959159</v>
       </c>
       <c r="T311">
-        <v>2.7646059048058724E-2</v>
+        <v>-2.7646059048058724E-2</v>
       </c>
       <c r="U311">
-        <v>8.8320204632363897E-2</v>
+        <v>-8.8320204632363897E-2</v>
       </c>
       <c r="V311">
         <v>0.16563203149819739</v>
@@ -26954,10 +26954,10 @@
         <v>0.12357500163103821</v>
       </c>
       <c r="T312">
-        <v>3.217154204886441E-2</v>
+        <v>-3.217154204886441E-2</v>
       </c>
       <c r="U312">
-        <v>8.0823312721967078E-2</v>
+        <v>-8.0823312721967078E-2</v>
       </c>
       <c r="V312">
         <v>0.20165568455088323</v>
@@ -27049,10 +27049,10 @@
         <v>0.12357306701649164</v>
       </c>
       <c r="T313">
-        <v>2.7229348356283545E-2</v>
+        <v>-2.7229348356283545E-2</v>
       </c>
       <c r="U313">
-        <v>7.7551653363983064E-2</v>
+        <v>-7.7551653363983064E-2</v>
       </c>
       <c r="V313">
         <v>0.19171505444528503</v>
@@ -27144,10 +27144,10 @@
         <v>0.12085365695090272</v>
       </c>
       <c r="T314">
-        <v>2.2388431535769193E-2</v>
+        <v>-2.2388431535769193E-2</v>
       </c>
       <c r="U314">
-        <v>7.5195908250380583E-2</v>
+        <v>-7.5195908250380583E-2</v>
       </c>
       <c r="V314">
         <v>-0.17124751314883113</v>
@@ -27239,10 +27239,10 @@
         <v>0.12017728378211157</v>
       </c>
       <c r="T315">
-        <v>2.453021864052829E-2</v>
+        <v>-2.453021864052829E-2</v>
       </c>
       <c r="U315">
-        <v>7.14885455773695E-2</v>
+        <v>-7.14885455773695E-2</v>
       </c>
       <c r="V315">
         <v>-0.35138615486272062</v>
@@ -27334,10 +27334,10 @@
         <v>0.12008313629595584</v>
       </c>
       <c r="T316">
-        <v>2.5002542609620093E-2</v>
+        <v>-2.5002542609620093E-2</v>
       </c>
       <c r="U316">
-        <v>6.890030093480437E-2</v>
+        <v>-6.890030093480437E-2</v>
       </c>
       <c r="V316">
         <v>-0.28363607221180143</v>
@@ -27429,10 +27429,10 @@
         <v>0.12006692598108841</v>
       </c>
       <c r="T317">
-        <v>2.6516628328843161E-2</v>
+        <v>-2.6516628328843161E-2</v>
       </c>
       <c r="U317">
-        <v>4.9793255267993608E-2</v>
+        <v>-4.9793255267993608E-2</v>
       </c>
       <c r="V317">
         <v>-0.30890324470798092</v>
@@ -27524,10 +27524,10 @@
         <v>0.1200657426146229</v>
       </c>
       <c r="T318">
-        <v>2.4539711318238844E-2</v>
+        <v>-2.4539711318238844E-2</v>
       </c>
       <c r="U318">
-        <v>5.9337373062051668E-2</v>
+        <v>-5.9337373062051668E-2</v>
       </c>
       <c r="V318">
         <v>-0.30004146372684115</v>
@@ -27619,10 +27619,10 @@
         <v>0.12004812994274575</v>
       </c>
       <c r="T319">
-        <v>2.7372195052977055E-2</v>
+        <v>-2.7372195052977055E-2</v>
       </c>
       <c r="U319">
-        <v>7.0033534565427935E-2</v>
+        <v>-7.0033534565427935E-2</v>
       </c>
       <c r="V319">
         <v>-0.32906328716175715</v>
@@ -27714,10 +27714,10 @@
         <v>0.11933659727102097</v>
       </c>
       <c r="T320">
-        <v>3.0059466326370909E-2</v>
+        <v>-3.0059466326370909E-2</v>
       </c>
       <c r="U320">
-        <v>6.435870556378287E-2</v>
+        <v>-6.435870556378287E-2</v>
       </c>
       <c r="V320">
         <v>-0.1474917663661035</v>
@@ -27809,10 +27809,10 @@
         <v>0.11932516978100133</v>
       </c>
       <c r="T321">
-        <v>3.5490165676121954E-2</v>
+        <v>-3.5490165676121954E-2</v>
       </c>
       <c r="U321">
-        <v>6.8041963189990895E-2</v>
+        <v>-6.8041963189990895E-2</v>
       </c>
       <c r="V321">
         <v>-0.17127711012188129</v>
@@ -27904,10 +27904,10 @@
         <v>0.11870492917352107</v>
       </c>
       <c r="T322">
-        <v>3.5031768876847558E-2</v>
+        <v>-3.5031768876847558E-2</v>
       </c>
       <c r="U322">
-        <v>5.9849002985612465E-2</v>
+        <v>-5.9849002985612465E-2</v>
       </c>
       <c r="V322">
         <v>-0.34637270163153655</v>
@@ -27999,10 +27999,10 @@
         <v>0.11828835880848798</v>
       </c>
       <c r="T323">
-        <v>2.8538980576042761E-2</v>
+        <v>-2.8538980576042761E-2</v>
       </c>
       <c r="U323">
-        <v>-1.4952719805227943E-2</v>
+        <v>1.4952719805227943E-2</v>
       </c>
       <c r="V323">
         <v>-0.20402994632124916</v>
@@ -28094,10 +28094,10 @@
         <v>0.11798708290523938</v>
       </c>
       <c r="T324">
-        <v>2.9065218827084571E-2</v>
+        <v>-2.9065218827084571E-2</v>
       </c>
       <c r="U324">
-        <v>6.4010884284892988E-2</v>
+        <v>-6.4010884284892988E-2</v>
       </c>
       <c r="V324">
         <v>-0.32431884870942618</v>
@@ -28189,10 +28189,10 @@
         <v>0.11756062420778284</v>
       </c>
       <c r="T325">
-        <v>3.4934186629276276E-2</v>
+        <v>-3.4934186629276276E-2</v>
       </c>
       <c r="U325">
-        <v>5.5179559654949806E-2</v>
+        <v>-5.5179559654949806E-2</v>
       </c>
       <c r="V325">
         <v>-0.18005862053849242</v>
@@ -28284,10 +28284,10 @@
         <v>0.11741403437787808</v>
       </c>
       <c r="T326">
-        <v>3.1224039521848823E-2</v>
+        <v>-3.1224039521848823E-2</v>
       </c>
       <c r="U326">
-        <v>5.3318933616086639E-2</v>
+        <v>-5.3318933616086639E-2</v>
       </c>
       <c r="V326">
         <v>-9.5795326178449436E-2</v>
@@ -28379,10 +28379,10 @@
         <v>0.11740031202038663</v>
       </c>
       <c r="T327">
-        <v>2.1179113261737825E-2</v>
+        <v>-2.1179113261737825E-2</v>
       </c>
       <c r="U327">
-        <v>5.2355913255563991E-2</v>
+        <v>-5.2355913255563991E-2</v>
       </c>
       <c r="V327">
         <v>-7.3307183717696844E-2</v>
@@ -28474,10 +28474,10 @@
         <v>0.11716770994223548</v>
       </c>
       <c r="T328">
-        <v>2.1176954717860852E-2</v>
+        <v>-2.1176954717860852E-2</v>
       </c>
       <c r="U328">
-        <v>5.6546091864784209E-2</v>
+        <v>-5.6546091864784209E-2</v>
       </c>
       <c r="V328">
         <v>-0.17336636350713253</v>
@@ -28569,10 +28569,10 @@
         <v>0.11677389009921647</v>
       </c>
       <c r="T329">
-        <v>2.9851674225223057E-2</v>
+        <v>-2.9851674225223057E-2</v>
       </c>
       <c r="U329">
-        <v>6.1039768789550308E-2</v>
+        <v>-6.1039768789550308E-2</v>
       </c>
       <c r="V329">
         <v>-0.30875916141233084</v>
@@ -28664,10 +28664,10 @@
         <v>0.11539276043865676</v>
       </c>
       <c r="T330">
-        <v>3.3343405422758821E-2</v>
+        <v>-3.3343405422758821E-2</v>
       </c>
       <c r="U330">
-        <v>6.6783928863412001E-2</v>
+        <v>-6.6783928863412001E-2</v>
       </c>
       <c r="V330">
         <v>-6.1523805140129006E-2</v>
@@ -28759,10 +28759,10 @@
         <v>0.11466348699232362</v>
       </c>
       <c r="T331">
-        <v>3.1287845455896246E-2</v>
+        <v>-3.1287845455896246E-2</v>
       </c>
       <c r="U331">
-        <v>6.2935665000218854E-2</v>
+        <v>-6.2935665000218854E-2</v>
       </c>
       <c r="V331">
         <v>-0.24254910339869262</v>
@@ -28854,10 +28854,10 @@
         <v>0.11466698773076806</v>
       </c>
       <c r="T332">
-        <v>1.9326573883882148E-2</v>
+        <v>-1.9326573883882148E-2</v>
       </c>
       <c r="U332">
-        <v>5.0229368256959894E-2</v>
+        <v>-5.0229368256959894E-2</v>
       </c>
       <c r="V332">
         <v>-0.23420132507594449</v>
@@ -28949,10 +28949,10 @@
         <v>0.11440051520907794</v>
       </c>
       <c r="T333">
-        <v>2.630796267288904E-2</v>
+        <v>-2.630796267288904E-2</v>
       </c>
       <c r="U333">
-        <v>5.3226182712640124E-2</v>
+        <v>-5.3226182712640124E-2</v>
       </c>
       <c r="V333">
         <v>-0.12511575509914774</v>
@@ -29044,10 +29044,10 @@
         <v>0.11435579224014145</v>
       </c>
       <c r="T334">
-        <v>2.6998093568164627E-2</v>
+        <v>-2.6998093568164627E-2</v>
       </c>
       <c r="U334">
-        <v>4.7245946790575033E-2</v>
+        <v>-4.7245946790575033E-2</v>
       </c>
       <c r="V334">
         <v>-0.16681859053380155</v>
@@ -29139,10 +29139,10 @@
         <v>0.11419132442678957</v>
       </c>
       <c r="T335">
-        <v>3.3676684134098522E-2</v>
+        <v>-3.3676684134098522E-2</v>
       </c>
       <c r="U335">
-        <v>4.7109814704815456E-2</v>
+        <v>-4.7109814704815456E-2</v>
       </c>
       <c r="V335">
         <v>-0.25413361355057784</v>
@@ -29234,10 +29234,10 @@
         <v>0.113413467214541</v>
       </c>
       <c r="T336">
-        <v>3.8863507859421276E-2</v>
+        <v>-3.8863507859421276E-2</v>
       </c>
       <c r="U336">
-        <v>5.3990503334944151E-2</v>
+        <v>-5.3990503334944151E-2</v>
       </c>
       <c r="V336">
         <v>-7.5880809003514571E-2</v>
@@ -29329,10 +29329,10 @@
         <v>0.11320380814378012</v>
       </c>
       <c r="T337">
-        <v>3.8789428578578367E-2</v>
+        <v>-3.8789428578578367E-2</v>
       </c>
       <c r="U337">
-        <v>5.4042160892975311E-2</v>
+        <v>-5.4042160892975311E-2</v>
       </c>
       <c r="V337">
         <v>1.7735005999619524E-2</v>
@@ -29424,10 +29424,10 @@
         <v>0.11311309033608995</v>
       </c>
       <c r="T338">
-        <v>4.6750667401807E-2</v>
+        <v>-4.6750667401807E-2</v>
       </c>
       <c r="U338">
-        <v>6.6778040756654278E-2</v>
+        <v>-6.6778040756654278E-2</v>
       </c>
       <c r="V338">
         <v>-6.0834636413376053E-2</v>
@@ -29519,10 +29519,10 @@
         <v>0.11272434726375247</v>
       </c>
       <c r="T339">
-        <v>4.6299625622392426E-2</v>
+        <v>-4.6299625622392426E-2</v>
       </c>
       <c r="U339">
-        <v>6.3970399508783693E-2</v>
+        <v>-6.3970399508783693E-2</v>
       </c>
       <c r="V339">
         <v>-0.18766137701258234</v>
@@ -29614,10 +29614,10 @@
         <v>0.1125571455509386</v>
       </c>
       <c r="T340">
-        <v>4.5590492667124671E-2</v>
+        <v>-4.5590492667124671E-2</v>
       </c>
       <c r="U340">
-        <v>6.2531360588935492E-2</v>
+        <v>-6.2531360588935492E-2</v>
       </c>
       <c r="V340">
         <v>-0.26855130183525144</v>
@@ -29709,10 +29709,10 @@
         <v>0.11220785566502144</v>
       </c>
       <c r="T341">
-        <v>4.0446971102192641E-2</v>
+        <v>-4.0446971102192641E-2</v>
       </c>
       <c r="U341">
-        <v>6.9476739413976141E-2</v>
+        <v>-6.9476739413976141E-2</v>
       </c>
       <c r="V341">
         <v>-0.39218526530324649</v>
@@ -29804,10 +29804,10 @@
         <v>0.11217203153208227</v>
       </c>
       <c r="T342">
-        <v>4.238870995278976E-2</v>
+        <v>-4.238870995278976E-2</v>
       </c>
       <c r="U342">
-        <v>7.6011553909505203E-2</v>
+        <v>-7.6011553909505203E-2</v>
       </c>
       <c r="V342">
         <v>-0.43365081530410965</v>
@@ -29899,10 +29899,10 @@
         <v>0.11206044640511142</v>
       </c>
       <c r="T343">
-        <v>4.3487976151856955E-2</v>
+        <v>-4.3487976151856955E-2</v>
       </c>
       <c r="U343">
-        <v>7.2096794669662678E-2</v>
+        <v>-7.2096794669662678E-2</v>
       </c>
       <c r="V343">
         <v>-0.36155371062047692</v>
@@ -29994,10 +29994,10 @@
         <v>0.11193670743502521</v>
       </c>
       <c r="T344">
-        <v>4.6918392881023507E-2</v>
+        <v>-4.6918392881023507E-2</v>
       </c>
       <c r="U344">
-        <v>7.0748983335433557E-2</v>
+        <v>-7.0748983335433557E-2</v>
       </c>
       <c r="V344">
         <v>-0.4349508264149593</v>
@@ -30089,10 +30089,10 @@
         <v>0.11187773383927557</v>
       </c>
       <c r="T345">
-        <v>4.8697280099796458E-2</v>
+        <v>-4.8697280099796458E-2</v>
       </c>
       <c r="U345">
-        <v>7.4644372923149405E-2</v>
+        <v>-7.4644372923149405E-2</v>
       </c>
       <c r="V345">
         <v>-0.38589185758370892</v>
@@ -30184,10 +30184,10 @@
         <v>0.11153107920002514</v>
       </c>
       <c r="T346">
-        <v>5.3003365120263268E-2</v>
+        <v>-5.3003365120263268E-2</v>
       </c>
       <c r="U346">
-        <v>7.9540558635460279E-2</v>
+        <v>-7.9540558635460279E-2</v>
       </c>
       <c r="V346">
         <v>-0.50953296806912629</v>
@@ -30279,10 +30279,10 @@
         <v>0.10938602615264099</v>
       </c>
       <c r="T347">
-        <v>5.4570609056536767E-2</v>
+        <v>-5.4570609056536767E-2</v>
       </c>
       <c r="U347">
-        <v>8.2507920423546821E-2</v>
+        <v>-8.2507920423546821E-2</v>
       </c>
       <c r="V347">
         <v>-0.20967370313882405</v>
@@ -30374,10 +30374,10 @@
         <v>0.10924191851182177</v>
       </c>
       <c r="T348">
-        <v>5.517739254989884E-2</v>
+        <v>-5.517739254989884E-2</v>
       </c>
       <c r="U348">
-        <v>8.1123721760545386E-2</v>
+        <v>-8.1123721760545386E-2</v>
       </c>
       <c r="V348">
         <v>-0.28669102858935869</v>
@@ -30469,10 +30469,10 @@
         <v>0.10924127484528108</v>
       </c>
       <c r="T349">
-        <v>5.179828061026015E-2</v>
+        <v>-5.179828061026015E-2</v>
       </c>
       <c r="U349">
-        <v>8.0412486912617709E-2</v>
+        <v>-8.0412486912617709E-2</v>
       </c>
       <c r="V349">
         <v>-0.27781705327394324</v>
@@ -30564,10 +30564,10 @@
         <v>0.10924106738481744</v>
       </c>
       <c r="T350">
-        <v>4.9570945993349103E-2</v>
+        <v>-4.9570945993349103E-2</v>
       </c>
       <c r="U350">
-        <v>8.0756511509094686E-2</v>
+        <v>-8.0756511509094686E-2</v>
       </c>
       <c r="V350">
         <v>-0.27941635451278479</v>
@@ -30659,10 +30659,10 @@
         <v>0.10924113795233571</v>
       </c>
       <c r="T351">
-        <v>5.1740685238033102E-2</v>
+        <v>-5.1740685238033102E-2</v>
       </c>
       <c r="U351">
-        <v>8.8293717441012554E-2</v>
+        <v>-8.8293717441012554E-2</v>
       </c>
       <c r="V351">
         <v>-0.28016832119350799</v>
@@ -30754,10 +30754,10 @@
         <v>0.10924552945376396</v>
       </c>
       <c r="T352">
-        <v>3.3804947362736648E-2</v>
+        <v>-3.3804947362736648E-2</v>
       </c>
       <c r="U352">
-        <v>6.926424292919009E-2</v>
+        <v>-6.926424292919009E-2</v>
       </c>
       <c r="V352">
         <v>-0.27036942964226984</v>
@@ -30849,10 +30849,10 @@
         <v>0.10924441289379412</v>
       </c>
       <c r="T353">
-        <v>3.3549011939282281E-2</v>
+        <v>-3.3549011939282281E-2</v>
       </c>
       <c r="U353">
-        <v>6.2447638717744169E-2</v>
+        <v>-6.2447638717744169E-2</v>
       </c>
       <c r="V353">
         <v>-0.25978345154176186</v>
@@ -30944,10 +30944,10 @@
         <v>0.10924301526984433</v>
       </c>
       <c r="T354">
-        <v>3.0994900690528571E-2</v>
+        <v>-3.0994900690528571E-2</v>
       </c>
       <c r="U354">
-        <v>6.0321054869727497E-2</v>
+        <v>-6.0321054869727497E-2</v>
       </c>
       <c r="V354">
         <v>-0.26631070045377569</v>
@@ -31039,10 +31039,10 @@
         <v>0.10905184190402414</v>
       </c>
       <c r="T355">
-        <v>3.2407711755855217E-2</v>
+        <v>-3.2407711755855217E-2</v>
       </c>
       <c r="U355">
-        <v>6.7668323229463923E-2</v>
+        <v>-6.7668323229463923E-2</v>
       </c>
       <c r="V355">
         <v>-0.17658796954154177</v>
@@ -31134,10 +31134,10 @@
         <v>0.1088869238294284</v>
       </c>
       <c r="T356">
-        <v>3.8674434887475684E-2</v>
+        <v>-3.8674434887475684E-2</v>
       </c>
       <c r="U356">
-        <v>7.0473707799223462E-2</v>
+        <v>-7.0473707799223462E-2</v>
       </c>
       <c r="V356">
         <v>-0.26148534726124772</v>
@@ -31229,10 +31229,10 @@
         <v>0.10888692680627403</v>
       </c>
       <c r="T357">
-        <v>3.4079325793645587E-2</v>
+        <v>-3.4079325793645587E-2</v>
       </c>
       <c r="U357">
-        <v>5.5452096308927779E-2</v>
+        <v>-5.5452096308927779E-2</v>
       </c>
       <c r="V357">
         <v>-0.25498228369309484</v>
@@ -31324,10 +31324,10 @@
         <v>0.10888697401083076</v>
       </c>
       <c r="T358">
-        <v>3.5745579951584894E-2</v>
+        <v>-3.5745579951584894E-2</v>
       </c>
       <c r="U358">
-        <v>5.712244644311415E-2</v>
+        <v>-5.712244644311415E-2</v>
       </c>
       <c r="V358">
         <v>-0.25116001136744615</v>
@@ -31419,10 +31419,10 @@
         <v>0.10888690532553644</v>
       </c>
       <c r="T359">
-        <v>3.087898124526367E-2</v>
+        <v>-3.087898124526367E-2</v>
       </c>
       <c r="U359">
-        <v>6.0696652499836468E-2</v>
+        <v>-6.0696652499836468E-2</v>
       </c>
       <c r="V359">
         <v>-0.25108393619188707</v>
@@ -31514,10 +31514,10 @@
         <v>0.10888695932742611</v>
       </c>
       <c r="T360">
-        <v>2.997226059736624E-2</v>
+        <v>-2.997226059736624E-2</v>
       </c>
       <c r="U360">
-        <v>6.3098983453979685E-2</v>
+        <v>-6.3098983453979685E-2</v>
       </c>
       <c r="V360">
         <v>-0.25385420336201392</v>
@@ -31615,10 +31615,10 @@
         <v>0.17864757049709673</v>
       </c>
       <c r="T361">
-        <v>2.8491151675003046E-2</v>
+        <v>-2.8491151675003046E-2</v>
       </c>
       <c r="U361">
-        <v>5.9437950532514883E-2</v>
+        <v>-5.9437950532514883E-2</v>
       </c>
       <c r="V361">
         <v>-0.24786161406362694</v>
@@ -31722,10 +31722,10 @@
         <v>0.17855903233989817</v>
       </c>
       <c r="T362">
-        <v>4.3416150734532089E-2</v>
+        <v>-4.3416150734532089E-2</v>
       </c>
       <c r="U362">
-        <v>6.2594045869202031E-2</v>
+        <v>-6.2594045869202031E-2</v>
       </c>
       <c r="V362">
         <v>-0.24903963518061456</v>
@@ -31829,10 +31829,10 @@
         <v>0.17855560974703821</v>
       </c>
       <c r="T363">
-        <v>4.2171598801277188E-2</v>
+        <v>-4.2171598801277188E-2</v>
       </c>
       <c r="U363">
-        <v>6.8177775518007966E-2</v>
+        <v>-6.8177775518007966E-2</v>
       </c>
       <c r="V363">
         <v>-0.24405715057596034</v>
@@ -31936,10 +31936,10 @@
         <v>0.17710604764081353</v>
       </c>
       <c r="T364">
-        <v>5.0394769067740874E-2</v>
+        <v>-5.0394769067740874E-2</v>
       </c>
       <c r="U364">
-        <v>7.710227115416135E-2</v>
+        <v>-7.710227115416135E-2</v>
       </c>
       <c r="V364">
         <v>-0.26777374047470826</v>
@@ -32043,10 +32043,10 @@
         <v>0.17576476248108275</v>
       </c>
       <c r="T365">
-        <v>5.0405785332741093E-2</v>
+        <v>-5.0405785332741093E-2</v>
       </c>
       <c r="U365">
-        <v>8.3632683139500674E-2</v>
+        <v>-8.3632683139500674E-2</v>
       </c>
       <c r="V365">
         <v>-0.25657522282063194</v>
@@ -32150,10 +32150,10 @@
         <v>0.17553816522156643</v>
       </c>
       <c r="T366">
-        <v>4.9291594819744766E-2</v>
+        <v>-4.9291594819744766E-2</v>
       </c>
       <c r="U366">
-        <v>8.7653872026094426E-2</v>
+        <v>-8.7653872026094426E-2</v>
       </c>
       <c r="V366">
         <v>-0.26098381653274494</v>
@@ -32257,10 +32257,10 @@
         <v>0.1751655740235987</v>
       </c>
       <c r="T367">
-        <v>5.2597659179975942E-2</v>
+        <v>-5.2597659179975942E-2</v>
       </c>
       <c r="U367">
-        <v>9.0874488519987473E-2</v>
+        <v>-9.0874488519987473E-2</v>
       </c>
       <c r="V367">
         <v>-0.25833124101479754</v>
@@ -32364,10 +32364,10 @@
         <v>0.17438316264475695</v>
       </c>
       <c r="T368">
-        <v>4.2511025216984688E-2</v>
+        <v>-4.2511025216984688E-2</v>
       </c>
       <c r="U368">
-        <v>8.8531077197484542E-2</v>
+        <v>-8.8531077197484542E-2</v>
       </c>
       <c r="V368">
         <v>-0.2726953127741405</v>
@@ -32471,10 +32471,10 @@
         <v>0.17119160842529652</v>
       </c>
       <c r="T369">
-        <v>3.9395635916150695E-2</v>
+        <v>-3.9395635916150695E-2</v>
       </c>
       <c r="U369">
-        <v>8.4873301639376564E-2</v>
+        <v>-8.4873301639376564E-2</v>
       </c>
       <c r="V369">
         <v>-0.25822888642638153</v>
@@ -32578,10 +32578,10 @@
         <v>0.16952356485827061</v>
       </c>
       <c r="T370">
-        <v>4.4367422602631379E-2</v>
+        <v>-4.4367422602631379E-2</v>
       </c>
       <c r="U370">
-        <v>8.9096922907561105E-2</v>
+        <v>-8.9096922907561105E-2</v>
       </c>
       <c r="V370">
         <v>-0.2576961013837753</v>
@@ -32685,10 +32685,10 @@
         <v>0.16928290783740557</v>
       </c>
       <c r="T371">
-        <v>4.131884113396378E-2</v>
+        <v>-4.131884113396378E-2</v>
       </c>
       <c r="U371">
-        <v>8.08919777811834E-2</v>
+        <v>-8.08919777811834E-2</v>
       </c>
       <c r="V371">
         <v>-0.25918743747840312</v>
@@ -32792,10 +32792,10 @@
         <v>0.16922051937470103</v>
       </c>
       <c r="T372">
-        <v>3.4711082075222777E-2</v>
+        <v>-3.4711082075222777E-2</v>
       </c>
       <c r="U372">
-        <v>7.610331178944385E-2</v>
+        <v>-7.610331178944385E-2</v>
       </c>
       <c r="V372">
         <v>-0.25892924036718945</v>
@@ -32899,10 +32899,10 @@
         <v>0.16913415092145351</v>
       </c>
       <c r="T373">
-        <v>4.0091627254190687E-2</v>
+        <v>-4.0091627254190687E-2</v>
       </c>
       <c r="U373">
-        <v>8.2568718441189404E-2</v>
+        <v>-8.2568718441189404E-2</v>
       </c>
       <c r="V373">
         <v>-0.26433850669244086</v>
@@ -33006,10 +33006,10 @@
         <v>0.16850467491273685</v>
       </c>
       <c r="T374">
-        <v>3.8629709181559058E-2</v>
+        <v>-3.8629709181559058E-2</v>
       </c>
       <c r="U374">
-        <v>8.4458577746282515E-2</v>
+        <v>-8.4458577746282515E-2</v>
       </c>
       <c r="V374">
         <v>-0.25794189295373915</v>
@@ -33113,10 +33113,10 @@
         <v>0.16845890169488661</v>
       </c>
       <c r="T375">
-        <v>4.2506632123040511E-2</v>
+        <v>-4.2506632123040511E-2</v>
       </c>
       <c r="U375">
-        <v>9.0091137008097011E-2</v>
+        <v>-9.0091137008097011E-2</v>
       </c>
       <c r="V375">
         <v>-0.26581617522299927</v>
@@ -33220,10 +33220,10 @@
         <v>0.16767866478615523</v>
       </c>
       <c r="T376">
-        <v>4.270038949053534E-2</v>
+        <v>-4.270038949053534E-2</v>
       </c>
       <c r="U376">
-        <v>9.4592414973537764E-2</v>
+        <v>-9.4592414973537764E-2</v>
       </c>
       <c r="V376">
         <v>-0.26944392952563678</v>
@@ -33327,10 +33327,10 @@
         <v>0.16729180986621706</v>
       </c>
       <c r="T377">
-        <v>4.9595538686975082E-2</v>
+        <v>-4.9595538686975082E-2</v>
       </c>
       <c r="U377">
-        <v>0.10315372406669576</v>
+        <v>-0.10315372406669576</v>
       </c>
       <c r="V377">
         <v>-0.27858351597433995</v>
@@ -33434,10 +33434,10 @@
         <v>0.16639678298398802</v>
       </c>
       <c r="T378">
-        <v>5.2040151308285765E-2</v>
+        <v>-5.2040151308285765E-2</v>
       </c>
       <c r="U378">
-        <v>0.10619970003981072</v>
+        <v>-0.10619970003981072</v>
       </c>
       <c r="V378">
         <v>-0.28461245067359364</v>
@@ -33541,10 +33541,10 @@
         <v>0.16597382019209958</v>
       </c>
       <c r="T379">
-        <v>5.5885057324223109E-2</v>
+        <v>-5.5885057324223109E-2</v>
       </c>
       <c r="U379">
-        <v>0.10677911854315436</v>
+        <v>-0.10677911854315436</v>
       </c>
       <c r="V379">
         <v>-0.28446049482016011</v>
@@ -33648,10 +33648,10 @@
         <v>0.16361100676728263</v>
       </c>
       <c r="T380">
-        <v>6.0911613457848013E-2</v>
+        <v>-6.0911613457848013E-2</v>
       </c>
       <c r="U380">
-        <v>0.10961503750143153</v>
+        <v>-0.10961503750143153</v>
       </c>
       <c r="V380">
         <v>-0.28649899951691538</v>
@@ -33755,10 +33755,10 @@
         <v>0.16310828855301121</v>
       </c>
       <c r="T381">
-        <v>5.1282821302545134E-2</v>
+        <v>-5.1282821302545134E-2</v>
       </c>
       <c r="U381">
-        <v>0.10202149722674525</v>
+        <v>-0.10202149722674525</v>
       </c>
       <c r="V381">
         <v>-0.28023070733911304</v>
@@ -33862,10 +33862,10 @@
         <v>0.16157641743668963</v>
       </c>
       <c r="T382">
-        <v>6.8462393607660044E-2</v>
+        <v>-6.8462393607660044E-2</v>
       </c>
       <c r="U382">
-        <v>0.1012362251734622</v>
+        <v>-0.1012362251734622</v>
       </c>
       <c r="V382">
         <v>-0.2791349187395431</v>
@@ -33969,10 +33969,10 @@
         <v>0.16157656546632407</v>
       </c>
       <c r="T383">
-        <v>6.7186919820982904E-2</v>
+        <v>-6.7186919820982904E-2</v>
       </c>
       <c r="U383">
-        <v>9.9694969108687914E-2</v>
+        <v>-9.9694969108687914E-2</v>
       </c>
       <c r="V383">
         <v>-0.27476917758419983</v>
@@ -34076,10 +34076,10 @@
         <v>0.16154397761666051</v>
       </c>
       <c r="T384">
-        <v>6.2870199281761519E-2</v>
+        <v>-6.2870199281761519E-2</v>
       </c>
       <c r="U384">
-        <v>9.2898299037336152E-2</v>
+        <v>-9.2898299037336152E-2</v>
       </c>
       <c r="V384">
         <v>-0.26517268981973707</v>
@@ -34183,10 +34183,10 @@
         <v>0.16142342802116996</v>
       </c>
       <c r="T385">
-        <v>4.5000227191149822E-2</v>
+        <v>-4.5000227191149822E-2</v>
       </c>
       <c r="U385">
-        <v>7.6528703131351072E-2</v>
+        <v>-7.6528703131351072E-2</v>
       </c>
       <c r="V385">
         <v>-0.24433758186694909</v>
@@ -34290,10 +34290,10 @@
         <v>0.1614001024569387</v>
       </c>
       <c r="T386">
-        <v>3.2413297333167002E-2</v>
+        <v>-3.2413297333167002E-2</v>
       </c>
       <c r="U386">
-        <v>7.0302565642876846E-2</v>
+        <v>-7.0302565642876846E-2</v>
       </c>
       <c r="V386">
         <v>-0.23552391129398886</v>
@@ -34397,10 +34397,10 @@
         <v>0.15998661596844521</v>
       </c>
       <c r="T387">
-        <v>3.5347092367266075E-2</v>
+        <v>-3.5347092367266075E-2</v>
       </c>
       <c r="U387">
-        <v>6.8629838043066105E-2</v>
+        <v>-6.8629838043066105E-2</v>
       </c>
       <c r="V387">
         <v>-0.23291469394957076</v>
@@ -34504,10 +34504,10 @@
         <v>0.15720361749149958</v>
       </c>
       <c r="T388">
-        <v>3.5066993932109103E-2</v>
+        <v>-3.5066993932109103E-2</v>
       </c>
       <c r="U388">
-        <v>7.0011469697639495E-2</v>
+        <v>-7.0011469697639495E-2</v>
       </c>
       <c r="V388">
         <v>-0.23466218127622396</v>
@@ -34611,10 +34611,10 @@
         <v>0.15720357717376332</v>
       </c>
       <c r="T389">
-        <v>3.7273082852995465E-2</v>
+        <v>-3.7273082852995465E-2</v>
       </c>
       <c r="U389">
-        <v>6.7388684146074684E-2</v>
+        <v>-6.7388684146074684E-2</v>
       </c>
       <c r="V389">
         <v>-0.38417972595126137</v>
@@ -34665,6 +34665,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="dd854d95-092e-48c7-992a-80d5cc5badc3" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="0902cc7b-e4ce-48dd-a92e-a98e18ec7ffe">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101006CC87EF38A8DD0408B89B7B34D0336DC" ma:contentTypeVersion="20" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="a30c2ca5bc864785a186dec6b0346788">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="0902cc7b-e4ce-48dd-a92e-a98e18ec7ffe" xmlns:ns3="dd854d95-092e-48c7-992a-80d5cc5badc3" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2932ec1554b414302dd4a6579c5666bc" ns2:_="" ns3:_="">
     <xsd:import namespace="0902cc7b-e4ce-48dd-a92e-a98e18ec7ffe"/>
@@ -34919,27 +34939,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9C21325A-2FA6-4D29-AED0-CA44A2859AE9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="dd854d95-092e-48c7-992a-80d5cc5badc3"/>
+    <ds:schemaRef ds:uri="0902cc7b-e4ce-48dd-a92e-a98e18ec7ffe"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="dd854d95-092e-48c7-992a-80d5cc5badc3" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="0902cc7b-e4ce-48dd-a92e-a98e18ec7ffe">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3FDE56E9-7C64-4C15-9C33-5B738E73FACD}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BABE8802-F313-4DEC-9147-95F411D9A097}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -34956,23 +34975,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3FDE56E9-7C64-4C15-9C33-5B738E73FACD}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9C21325A-2FA6-4D29-AED0-CA44A2859AE9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="dd854d95-092e-48c7-992a-80d5cc5badc3"/>
-    <ds:schemaRef ds:uri="0902cc7b-e4ce-48dd-a92e-a98e18ec7ffe"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Actualizar Data-ETFPESOV.xlsx (27/10/2026 00:32)
</commit_message>
<xml_diff>
--- a/ETFPESOV/General/Data-ETFPESOV.xlsx
+++ b/ETFPESOV/General/Data-ETFPESOV.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eldorado275.sharepoint.com/sites/Compartidos/Documentos compartidos/INVERSIONES/Claude - Fernando/Dashboards ETFs/Dashboards/ETFPESOV/General/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="32" documentId="13_ncr:1_{92F23378-0498-4D77-8B70-1F22B2DCC606}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{832548A3-27EB-4C0C-AC3C-4D25B168E83D}"/>
+  <xr:revisionPtr revIDLastSave="34" documentId="13_ncr:1_{92F23378-0498-4D77-8B70-1F22B2DCC606}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{673AAD81-7E84-41F6-AA17-9552641B2E13}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{F6F75CCC-009E-413C-B55D-A670828334F1}"/>
   </bookViews>
@@ -530,7 +530,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E89EACC1-FF2B-4ECD-9B28-49A6BC374F12}">
-  <dimension ref="A1:AI389"/>
+  <dimension ref="A1:AI390"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="27" max="31" width="11.5546875" style="3"/>
@@ -34562,8 +34562,8 @@
       <c r="C389">
         <v>149077720.44977134</v>
       </c>
-      <c r="D389" t="s">
-        <v>23</v>
+      <c r="D389">
+        <v>547</v>
       </c>
       <c r="E389">
         <v>5982.21</v>
@@ -34657,6 +34657,113 @@
       </c>
       <c r="AI389">
         <v>10047.755000000001</v>
+      </c>
+    </row>
+    <row r="390" spans="1:35" x14ac:dyDescent="0.3">
+      <c r="A390" s="1">
+        <v>46321</v>
+      </c>
+      <c r="B390">
+        <v>110.58673230898968</v>
+      </c>
+      <c r="C390">
+        <v>149015621.7863636</v>
+      </c>
+      <c r="D390" t="s">
+        <v>23</v>
+      </c>
+      <c r="E390">
+        <v>2105</v>
+      </c>
+      <c r="F390">
+        <v>2</v>
+      </c>
+      <c r="G390">
+        <v>6.2304747077615721</v>
+      </c>
+      <c r="H390">
+        <v>6.129373223079976</v>
+      </c>
+      <c r="I390">
+        <v>181.72</v>
+      </c>
+      <c r="J390">
+        <v>6.31</v>
+      </c>
+      <c r="K390">
+        <v>6.1899999999999995</v>
+      </c>
+      <c r="L390">
+        <v>10.586732308989678</v>
+      </c>
+      <c r="M390">
+        <v>11.079191052616322</v>
+      </c>
+      <c r="N390">
+        <v>6.5803131862324014</v>
+      </c>
+      <c r="O390">
+        <v>6.59</v>
+      </c>
+      <c r="P390">
+        <v>5.4989128448245158E-3</v>
+      </c>
+      <c r="Q390">
+        <v>5.2218641305133108E-3</v>
+      </c>
+      <c r="R390">
+        <v>0.1078466854227064</v>
+      </c>
+      <c r="S390">
+        <v>0.15681536223562831</v>
+      </c>
+      <c r="T390">
+        <v>-3.1813029847360674E-2</v>
+      </c>
+      <c r="U390">
+        <v>-6.1049079585928645E-2</v>
+      </c>
+      <c r="V390">
+        <v>-0.25030487093484766</v>
+      </c>
+      <c r="W390">
+        <v>-0.46282776112556157</v>
+      </c>
+      <c r="X390">
+        <v>110.79</v>
+      </c>
+      <c r="Y390">
+        <v>-2.5120016823665048</v>
+      </c>
+      <c r="Z390">
+        <v>-3.9109511967821864</v>
+      </c>
+      <c r="AA390" s="3">
+        <v>1.8380838891447482E-3</v>
+      </c>
+      <c r="AB390" s="3">
+        <v>6.0603431449080059E-3</v>
+      </c>
+      <c r="AC390" s="3">
+        <v>5.1737156747969438E-3</v>
+      </c>
+      <c r="AD390" s="3">
+        <v>4.4457987196358665E-3</v>
+      </c>
+      <c r="AE390" s="3">
+        <v>5.0120668383469768E-3</v>
+      </c>
+      <c r="AF390">
+        <v>6823</v>
+      </c>
+      <c r="AG390">
+        <v>8662.9650000000001</v>
+      </c>
+      <c r="AH390">
+        <v>10696.294999999998</v>
+      </c>
+      <c r="AI390">
+        <v>9958.755000000001</v>
       </c>
     </row>
   </sheetData>
@@ -34665,6 +34772,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="dd854d95-092e-48c7-992a-80d5cc5badc3" xsi:nil="true"/>
@@ -34673,15 +34789,6 @@
     </lcf76f155ced4ddcb4097134ff3c332f>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -34940,20 +35047,20 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3FDE56E9-7C64-4C15-9C33-5B738E73FACD}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9C21325A-2FA6-4D29-AED0-CA44A2859AE9}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="dd854d95-092e-48c7-992a-80d5cc5badc3"/>
     <ds:schemaRef ds:uri="0902cc7b-e4ce-48dd-a92e-a98e18ec7ffe"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3FDE56E9-7C64-4C15-9C33-5B738E73FACD}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Actualizar Data-ETFPESOV.xlsx (28/10/2026 00:40)
</commit_message>
<xml_diff>
--- a/ETFPESOV/General/Data-ETFPESOV.xlsx
+++ b/ETFPESOV/General/Data-ETFPESOV.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eldorado275.sharepoint.com/sites/Compartidos/Documentos compartidos/INVERSIONES/Claude - Fernando/Dashboards ETFs/Dashboards/ETFPESOV/General/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="36" documentId="13_ncr:1_{92F23378-0498-4D77-8B70-1F22B2DCC606}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7A688B8F-5C2B-445A-A3BB-047DF36C5700}"/>
+  <xr:revisionPtr revIDLastSave="53" documentId="13_ncr:1_{92F23378-0498-4D77-8B70-1F22B2DCC606}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{57B11A0A-CE08-4EF3-BAAE-5F89E49C8D9F}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{F6F75CCC-009E-413C-B55D-A670828334F1}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="39">
   <si>
     <t>Fecha</t>
   </si>
@@ -539,7 +539,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E89EACC1-FF2B-4ECD-9B28-49A6BC374F12}">
-  <dimension ref="A1:AL390"/>
+  <dimension ref="A1:AT391"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="27" max="31" width="11.5546875" style="3"/>
@@ -1570,7 +1570,7 @@
         <v>9.4562899082472809E-3</v>
       </c>
     </row>
-    <row r="17" spans="1:36" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:46" x14ac:dyDescent="0.3">
       <c r="A17" s="1">
         <v>45771</v>
       </c>
@@ -1632,7 +1632,7 @@
         <v>1.0801057445594512E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:36" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:46" x14ac:dyDescent="0.3">
       <c r="A18" s="1">
         <v>45772</v>
       </c>
@@ -1694,7 +1694,7 @@
         <v>1.1793592036918684E-2</v>
       </c>
     </row>
-    <row r="19" spans="1:36" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:46" x14ac:dyDescent="0.3">
       <c r="A19" s="1">
         <v>45775</v>
       </c>
@@ -1756,7 +1756,7 @@
         <v>1.0740421153611178E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:36" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:46" x14ac:dyDescent="0.3">
       <c r="A20" s="1">
         <v>45776</v>
       </c>
@@ -1818,7 +1818,7 @@
         <v>1.0740421153611178E-2</v>
       </c>
     </row>
-    <row r="21" spans="1:36" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:46" x14ac:dyDescent="0.3">
       <c r="A21" s="1">
         <v>45777</v>
       </c>
@@ -1880,7 +1880,7 @@
         <v>1.2154556386551293E-2</v>
       </c>
     </row>
-    <row r="22" spans="1:36" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:46" x14ac:dyDescent="0.3">
       <c r="A22" s="1">
         <v>45779</v>
       </c>
@@ -1941,8 +1941,9 @@
       <c r="AJ22">
         <v>1.285482056728012E-2</v>
       </c>
-    </row>
-    <row r="23" spans="1:36" x14ac:dyDescent="0.3">
+      <c r="AT22" s="3"/>
+    </row>
+    <row r="23" spans="1:46" x14ac:dyDescent="0.3">
       <c r="A23" s="1">
         <v>45782</v>
       </c>
@@ -2004,7 +2005,7 @@
         <v>1.3645576960565222E-2</v>
       </c>
     </row>
-    <row r="24" spans="1:36" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:46" x14ac:dyDescent="0.3">
       <c r="A24" s="1">
         <v>45783</v>
       </c>
@@ -2066,7 +2067,7 @@
         <v>1.2512501749924378E-2</v>
       </c>
     </row>
-    <row r="25" spans="1:36" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:46" x14ac:dyDescent="0.3">
       <c r="A25" s="1">
         <v>45784</v>
       </c>
@@ -2128,7 +2129,7 @@
         <v>1.3069911383825291E-2</v>
       </c>
     </row>
-    <row r="26" spans="1:36" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:46" x14ac:dyDescent="0.3">
       <c r="A26" s="1">
         <v>45785</v>
       </c>
@@ -2190,7 +2191,7 @@
         <v>1.305590681133237E-2</v>
       </c>
     </row>
-    <row r="27" spans="1:36" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:46" x14ac:dyDescent="0.3">
       <c r="A27" s="1">
         <v>45786</v>
       </c>
@@ -2252,7 +2253,7 @@
         <v>1.1989955513331273E-2</v>
       </c>
     </row>
-    <row r="28" spans="1:36" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:46" x14ac:dyDescent="0.3">
       <c r="A28" s="1">
         <v>45789</v>
       </c>
@@ -2314,7 +2315,7 @@
         <v>1.1907012173202969E-2</v>
       </c>
     </row>
-    <row r="29" spans="1:36" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:46" x14ac:dyDescent="0.3">
       <c r="A29" s="1">
         <v>45790</v>
       </c>
@@ -2376,7 +2377,7 @@
         <v>1.2256028325144153E-2</v>
       </c>
     </row>
-    <row r="30" spans="1:36" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:46" x14ac:dyDescent="0.3">
       <c r="A30" s="1">
         <v>45791</v>
       </c>
@@ -2441,7 +2442,7 @@
         <v>1.2605044477085336E-2</v>
       </c>
     </row>
-    <row r="31" spans="1:36" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:46" x14ac:dyDescent="0.3">
       <c r="A31" s="1">
         <v>45792</v>
       </c>
@@ -2515,7 +2516,7 @@
         <v>1.3245775862324668E-2</v>
       </c>
     </row>
-    <row r="32" spans="1:36" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:46" x14ac:dyDescent="0.3">
       <c r="A32" s="1">
         <v>45793</v>
       </c>
@@ -37893,6 +37894,122 @@
       </c>
       <c r="AL390">
         <v>4.8071829408993889E-3</v>
+      </c>
+    </row>
+    <row r="391" spans="1:38" x14ac:dyDescent="0.3">
+      <c r="A391" s="1">
+        <v>46322</v>
+      </c>
+      <c r="B391">
+        <v>110.57449367869984</v>
+      </c>
+      <c r="C391">
+        <v>148999130.23204803</v>
+      </c>
+      <c r="D391" t="s">
+        <v>22</v>
+      </c>
+      <c r="E391">
+        <v>9791</v>
+      </c>
+      <c r="F391">
+        <v>5</v>
+      </c>
+      <c r="G391">
+        <v>6.226820098201709</v>
+      </c>
+      <c r="H391">
+        <v>6.1319510640682253</v>
+      </c>
+      <c r="I391">
+        <v>181.7</v>
+      </c>
+      <c r="J391">
+        <v>6.31</v>
+      </c>
+      <c r="K391">
+        <v>6.1899999999999995</v>
+      </c>
+      <c r="L391">
+        <v>10.574493678699849</v>
+      </c>
+      <c r="M391">
+        <v>11.066965739931689</v>
+      </c>
+      <c r="N391">
+        <v>6.5804257815830098</v>
+      </c>
+      <c r="O391">
+        <v>6.59</v>
+      </c>
+      <c r="P391">
+        <v>5.4888054029206771E-3</v>
+      </c>
+      <c r="Q391">
+        <v>5.2228319617534423E-3</v>
+      </c>
+      <c r="R391">
+        <v>0.10782533668747564</v>
+      </c>
+      <c r="S391">
+        <v>0.15652405037970035</v>
+      </c>
+      <c r="T391">
+        <v>-3.1805983653443448E-2</v>
+      </c>
+      <c r="U391">
+        <v>-5.9616804372386589E-2</v>
+      </c>
+      <c r="V391">
+        <v>-0.22056025797478895</v>
+      </c>
+      <c r="W391">
+        <v>-0.65649731473331752</v>
+      </c>
+      <c r="X391">
+        <v>110.01</v>
+      </c>
+      <c r="Y391">
+        <v>-2.5227906761652652</v>
+      </c>
+      <c r="Z391">
+        <v>-3.9109511967821864</v>
+      </c>
+      <c r="AA391" s="3">
+        <v>5.1050984718058467E-3</v>
+      </c>
+      <c r="AB391" s="3">
+        <v>5.983632672158434E-3</v>
+      </c>
+      <c r="AC391" s="3">
+        <v>5.2437821197458137E-3</v>
+      </c>
+      <c r="AD391" s="3">
+        <v>4.4697599667025273E-3</v>
+      </c>
+      <c r="AE391" s="3">
+        <v>5.0248974179157215E-3</v>
+      </c>
+      <c r="AF391">
+        <v>6823</v>
+      </c>
+      <c r="AG391">
+        <v>8662.9650000000001</v>
+      </c>
+      <c r="AH391">
+        <v>10634.04</v>
+      </c>
+      <c r="AI391">
+        <v>9877.625</v>
+      </c>
+      <c r="AJ391">
+        <v>4.7777889495442443E-3</v>
+      </c>
+      <c r="AK391">
+        <v>5.5520399158039396E-3</v>
+      </c>
+      <c r="AL391">
+        <v>4.8078159252481047E-3</v>
       </c>
     </row>
   </sheetData>
@@ -37901,26 +38018,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="dd854d95-092e-48c7-992a-80d5cc5badc3" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="0902cc7b-e4ce-48dd-a92e-a98e18ec7ffe">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101006CC87EF38A8DD0408B89B7B34D0336DC" ma:contentTypeVersion="20" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="a30c2ca5bc864785a186dec6b0346788">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="0902cc7b-e4ce-48dd-a92e-a98e18ec7ffe" xmlns:ns3="dd854d95-092e-48c7-992a-80d5cc5badc3" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2932ec1554b414302dd4a6579c5666bc" ns2:_="" ns3:_="">
     <xsd:import namespace="0902cc7b-e4ce-48dd-a92e-a98e18ec7ffe"/>
@@ -38175,26 +38272,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9C21325A-2FA6-4D29-AED0-CA44A2859AE9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="dd854d95-092e-48c7-992a-80d5cc5badc3"/>
-    <ds:schemaRef ds:uri="0902cc7b-e4ce-48dd-a92e-a98e18ec7ffe"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="dd854d95-092e-48c7-992a-80d5cc5badc3" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="0902cc7b-e4ce-48dd-a92e-a98e18ec7ffe">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3FDE56E9-7C64-4C15-9C33-5B738E73FACD}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BABE8802-F313-4DEC-9147-95F411D9A097}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -38211,4 +38309,23 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9C21325A-2FA6-4D29-AED0-CA44A2859AE9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="dd854d95-092e-48c7-992a-80d5cc5badc3"/>
+    <ds:schemaRef ds:uri="0902cc7b-e4ce-48dd-a92e-a98e18ec7ffe"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3FDE56E9-7C64-4C15-9C33-5B738E73FACD}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Actualizar Data-ETFPESOV.xlsx (29/10/2026 01:08)
</commit_message>
<xml_diff>
--- a/ETFPESOV/General/Data-ETFPESOV.xlsx
+++ b/ETFPESOV/General/Data-ETFPESOV.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eldorado275.sharepoint.com/sites/Compartidos/Documentos compartidos/INVERSIONES/Claude - Fernando/Dashboards ETFs/Dashboards/ETFPESOV/General/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="53" documentId="13_ncr:1_{92F23378-0498-4D77-8B70-1F22B2DCC606}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{57B11A0A-CE08-4EF3-BAAE-5F89E49C8D9F}"/>
+  <xr:revisionPtr revIDLastSave="55" documentId="13_ncr:1_{92F23378-0498-4D77-8B70-1F22B2DCC606}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5125336A-44F2-4847-B2F7-ECB47C059442}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{F6F75CCC-009E-413C-B55D-A670828334F1}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="39">
   <si>
     <t>Fecha</t>
   </si>
@@ -539,7 +539,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E89EACC1-FF2B-4ECD-9B28-49A6BC374F12}">
-  <dimension ref="A1:AT391"/>
+  <dimension ref="A1:AT392"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="27" max="31" width="11.5546875" style="3"/>
@@ -37790,8 +37790,8 @@
       <c r="C390">
         <v>149015621.7863636</v>
       </c>
-      <c r="D390" t="s">
-        <v>22</v>
+      <c r="D390">
+        <v>547</v>
       </c>
       <c r="E390">
         <v>2105</v>
@@ -37906,8 +37906,8 @@
       <c r="C391">
         <v>148999130.23204803</v>
       </c>
-      <c r="D391" t="s">
-        <v>22</v>
+      <c r="D391">
+        <v>550</v>
       </c>
       <c r="E391">
         <v>9791</v>
@@ -38010,6 +38010,122 @@
       </c>
       <c r="AL391">
         <v>4.8078159252481047E-3</v>
+      </c>
+    </row>
+    <row r="392" spans="1:38" x14ac:dyDescent="0.3">
+      <c r="A392" s="1">
+        <v>46323</v>
+      </c>
+      <c r="B392">
+        <v>110.44726897189142</v>
+      </c>
+      <c r="C392">
+        <v>148827694.93962368</v>
+      </c>
+      <c r="D392" t="s">
+        <v>22</v>
+      </c>
+      <c r="E392">
+        <v>49390</v>
+      </c>
+      <c r="F392">
+        <v>2</v>
+      </c>
+      <c r="G392">
+        <v>6.2204063063619381</v>
+      </c>
+      <c r="H392">
+        <v>6.1498775469484137</v>
+      </c>
+      <c r="I392">
+        <v>181.49</v>
+      </c>
+      <c r="J392">
+        <v>6.3</v>
+      </c>
+      <c r="K392">
+        <v>6.21</v>
+      </c>
+      <c r="L392">
+        <v>10.447268971891411</v>
+      </c>
+      <c r="M392">
+        <v>10.938599956743001</v>
+      </c>
+      <c r="N392">
+        <v>6.5802944119903</v>
+      </c>
+      <c r="O392">
+        <v>6.59</v>
+      </c>
+      <c r="P392">
+        <v>5.4936314942568574E-3</v>
+      </c>
+      <c r="Q392">
+        <v>4.9611965685411761E-3</v>
+      </c>
+      <c r="R392">
+        <v>0.10782480681294901</v>
+      </c>
+      <c r="S392">
+        <v>0.15621877183546237</v>
+      </c>
+      <c r="T392">
+        <v>-2.763261309838283E-2</v>
+      </c>
+      <c r="U392">
+        <v>-7.0268117369154393E-2</v>
+      </c>
+      <c r="V392">
+        <v>-0.21351905105646551</v>
+      </c>
+      <c r="W392">
+        <v>-0.45345263381872947</v>
+      </c>
+      <c r="X392">
+        <v>110</v>
+      </c>
+      <c r="Y392">
+        <v>-2.6349459206899462</v>
+      </c>
+      <c r="Z392">
+        <v>-3.9109511967821864</v>
+      </c>
+      <c r="AA392" s="3">
+        <v>4.0496154957462283E-3</v>
+      </c>
+      <c r="AB392" s="3">
+        <v>5.7605551990942789E-3</v>
+      </c>
+      <c r="AC392" s="3">
+        <v>5.280372822888243E-3</v>
+      </c>
+      <c r="AD392" s="3">
+        <v>4.4842705717397817E-3</v>
+      </c>
+      <c r="AE392" s="3">
+        <v>5.0253695406609717E-3</v>
+      </c>
+      <c r="AF392">
+        <v>6823</v>
+      </c>
+      <c r="AG392">
+        <v>8662.9650000000001</v>
+      </c>
+      <c r="AH392">
+        <v>10634.04</v>
+      </c>
+      <c r="AI392">
+        <v>9958.755000000001</v>
+      </c>
+      <c r="AJ392">
+        <v>4.7964053804230291E-3</v>
+      </c>
+      <c r="AK392">
+        <v>5.5593251845032932E-3</v>
+      </c>
+      <c r="AL392">
+        <v>4.8385096148013109E-3</v>
       </c>
     </row>
   </sheetData>
@@ -38273,6 +38389,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="dd854d95-092e-48c7-992a-80d5cc5badc3" xsi:nil="true"/>
@@ -38281,15 +38406,6 @@
     </lcf76f155ced4ddcb4097134ff3c332f>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -38312,6 +38428,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3FDE56E9-7C64-4C15-9C33-5B738E73FACD}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9C21325A-2FA6-4D29-AED0-CA44A2859AE9}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -38320,12 +38444,4 @@
     <ds:schemaRef ds:uri="0902cc7b-e4ce-48dd-a92e-a98e18ec7ffe"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3FDE56E9-7C64-4C15-9C33-5B738E73FACD}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>